<commit_message>
Excel actualizado 9 sep 2026
</commit_message>
<xml_diff>
--- a/PM_ESTUDIO_MASTER_COMPLETO.xlsx
+++ b/PM_ESTUDIO_MASTER_COMPLETO.xlsx
@@ -7,11 +7,10 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MASTER GLOBAL" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LEYENDA" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RESTAURANTES" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="VIVIENDA" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HOTELES" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LEYENDA" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RESTAURANTES" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="VIVIENDA" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HOTELES" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -21,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="32">
+  <fonts count="23">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -156,62 +155,8 @@
       <color rgb="009C9088"/>
       <sz val="8"/>
     </font>
-    <font>
-      <name val="Arial"/>
-      <b val="1"/>
-      <color rgb="003D6491"/>
-      <sz val="9"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <b val="1"/>
-      <color rgb="003D6491"/>
-      <sz val="8"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <b val="1"/>
-      <color rgb="00B86328"/>
-      <sz val="8"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <b val="1"/>
-      <color rgb="004A4A4A"/>
-      <sz val="8"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <b val="1"/>
-      <color rgb="00B35D30"/>
-      <sz val="9"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <b val="1"/>
-      <color rgb="00B35D30"/>
-      <sz val="8"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <b val="1"/>
-      <color rgb="00436B3A"/>
-      <sz val="9"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <b val="1"/>
-      <color rgb="00436B3A"/>
-      <sz val="8"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <b val="1"/>
-      <color rgb="001E5C1E"/>
-      <sz val="8"/>
-    </font>
   </fonts>
-  <fills count="30">
+  <fills count="26">
     <fill>
       <patternFill/>
     </fill>
@@ -338,28 +283,8 @@
         <fgColor rgb="00888888"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FAE5D0"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00E3EDE0"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="005C5248"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00EDEDEB"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="8">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -396,38 +321,11 @@
         <color rgb="001A3A5C"/>
       </top>
     </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="medium">
-        <color rgb="008B3A00"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="medium">
-        <color rgb="005C1831"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="medium">
-        <color rgb="001A3A5C"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="131">
+  <cellXfs count="97">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -679,102 +577,6 @@
     <xf numFmtId="0" fontId="8" fillId="16" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="26" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="26" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="26" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="26" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="26" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="26" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="26" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="26" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="27" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="27" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="27" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="27" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="28" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="29" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="29" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="29" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="29" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="29" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="29" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="29" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="29" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1140,3975 +942,6 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L69"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="28" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="22" customWidth="1" min="4" max="4"/>
-    <col width="36" customWidth="1" min="5" max="5"/>
-    <col width="11" customWidth="1" min="6" max="6"/>
-    <col width="28" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="14" customWidth="1" min="9" max="9"/>
-    <col width="14" customWidth="1" min="10" max="10"/>
-    <col width="14" customWidth="1" min="11" max="11"/>
-    <col width="36" customWidth="1" min="12" max="12"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="26" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>PM ESTUDIO — MASTER GLOBAL  ·  1 septiembre 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="8" customHeight="1"/>
-    <row r="3" ht="20" customHeight="1">
-      <c r="A3" s="97" t="inlineStr">
-        <is>
-          <t>PROYECTO</t>
-        </is>
-      </c>
-      <c r="B3" s="97" t="inlineStr">
-        <is>
-          <t>DPTO</t>
-        </is>
-      </c>
-      <c r="C3" s="97" t="inlineStr">
-        <is>
-          <t>RESPONSABLE</t>
-        </is>
-      </c>
-      <c r="D3" s="97" t="inlineStr">
-        <is>
-          <t>ESTADO</t>
-        </is>
-      </c>
-      <c r="E3" s="97" t="inlineStr">
-        <is>
-          <t>HITO PRÓXIMO</t>
-        </is>
-      </c>
-      <c r="F3" s="97" t="inlineStr">
-        <is>
-          <t>FECHA</t>
-        </is>
-      </c>
-      <c r="G3" s="97" t="inlineStr">
-        <is>
-          <t>BLOQUEADOR</t>
-        </is>
-      </c>
-      <c r="H3" s="97" t="inlineStr">
-        <is>
-          <t>CONSTRUCTORA</t>
-        </is>
-      </c>
-      <c r="I3" s="97" t="inlineStr">
-        <is>
-          <t>FASE</t>
-        </is>
-      </c>
-      <c r="J3" s="97" t="inlineStr">
-        <is>
-          <t>ATENCIÓN</t>
-        </is>
-      </c>
-      <c r="K3" s="97" t="inlineStr">
-        <is>
-          <t>NIVEL</t>
-        </is>
-      </c>
-      <c r="L3" s="97" t="inlineStr">
-        <is>
-          <t>OBSERVACIONES</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="16" customHeight="1">
-      <c r="A4" s="98" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  ▸  PROYECTOS ACTIVOS  —  1 septiembre 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="18" customHeight="1">
-      <c r="A5" s="99" t="inlineStr">
-        <is>
-          <t>PEDRAZA</t>
-        </is>
-      </c>
-      <c r="B5" s="100" t="inlineStr">
-        <is>
-          <t>VIVIENDA</t>
-        </is>
-      </c>
-      <c r="C5" s="101" t="inlineStr">
-        <is>
-          <t>Olatz/Paula</t>
-        </is>
-      </c>
-      <c r="D5" s="101" t="inlineStr">
-        <is>
-          <t>Remates finales</t>
-        </is>
-      </c>
-      <c r="E5" s="101" t="inlineStr">
-        <is>
-          <t>Reunión 1 sep con clientes y constructora</t>
-        </is>
-      </c>
-      <c r="F5" s="101" t="inlineStr">
-        <is>
-          <t>1 sep</t>
-        </is>
-      </c>
-      <c r="G5" s="101" t="inlineStr">
-        <is>
-          <t>2ª fase caballerías pendiente de definir</t>
-        </is>
-      </c>
-      <c r="H5" s="101" t="inlineStr">
-        <is>
-          <t>Amarco</t>
-        </is>
-      </c>
-      <c r="I5" s="101" t="inlineStr">
-        <is>
-          <t>REMATES</t>
-        </is>
-      </c>
-      <c r="J5" s="102" t="inlineStr">
-        <is>
-          <t>ATENCIÓN ALTA</t>
-        </is>
-      </c>
-      <c r="K5" s="102" t="inlineStr">
-        <is>
-          <t>ATENCIÓN ALTA</t>
-        </is>
-      </c>
-      <c r="L5" s="101" t="inlineStr">
-        <is>
-          <t>Lista repasos pendiente. 2ª fase caballerías por definir.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="18" customHeight="1">
-      <c r="A6" s="103" t="inlineStr">
-        <is>
-          <t>ZAHARA</t>
-        </is>
-      </c>
-      <c r="B6" s="104" t="inlineStr">
-        <is>
-          <t>VIVIENDA</t>
-        </is>
-      </c>
-      <c r="C6" s="51" t="inlineStr">
-        <is>
-          <t>Paula</t>
-        </is>
-      </c>
-      <c r="D6" s="51" t="inlineStr">
-        <is>
-          <t>Remates</t>
-        </is>
-      </c>
-      <c r="E6" s="51" t="inlineStr">
-        <is>
-          <t>Dormitorio de abajo pendiente</t>
-        </is>
-      </c>
-      <c r="F6" s="51" t="inlineStr">
-        <is>
-          <t>Sep 2026</t>
-        </is>
-      </c>
-      <c r="G6" s="51" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H6" s="51" t="inlineStr">
-        <is>
-          <t>Raúl</t>
-        </is>
-      </c>
-      <c r="I6" s="51" t="inlineStr">
-        <is>
-          <t>REMATES</t>
-        </is>
-      </c>
-      <c r="J6" s="105" t="inlineStr">
-        <is>
-          <t>SEGUIMIENTO</t>
-        </is>
-      </c>
-      <c r="K6" s="105" t="inlineStr">
-        <is>
-          <t>SEGUIMIENTO</t>
-        </is>
-      </c>
-      <c r="L6" s="51" t="inlineStr">
-        <is>
-          <t>Pedidos hechos. Ale con listas de deco faltante.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="18" customHeight="1">
-      <c r="A7" s="103" t="inlineStr">
-        <is>
-          <t>VALENCIA</t>
-        </is>
-      </c>
-      <c r="B7" s="104" t="inlineStr">
-        <is>
-          <t>VIVIENDA</t>
-        </is>
-      </c>
-      <c r="C7" s="51" t="inlineStr">
-        <is>
-          <t>Sara/Andrea</t>
-        </is>
-      </c>
-      <c r="D7" s="51" t="inlineStr">
-        <is>
-          <t>Entregado 29 ago</t>
-        </is>
-      </c>
-      <c r="E7" s="51" t="inlineStr">
-        <is>
-          <t>Mobiliario exterior mediados sep</t>
-        </is>
-      </c>
-      <c r="F7" s="51" t="inlineStr">
-        <is>
-          <t>Sep 2026</t>
-        </is>
-      </c>
-      <c r="G7" s="51" t="inlineStr">
-        <is>
-          <t>Problemas de obra asumidos</t>
-        </is>
-      </c>
-      <c r="H7" s="51" t="inlineStr">
-        <is>
-          <t>Raúl</t>
-        </is>
-      </c>
-      <c r="I7" s="51" t="inlineStr">
-        <is>
-          <t>REMATES</t>
-        </is>
-      </c>
-      <c r="J7" s="105" t="inlineStr">
-        <is>
-          <t>SEGUIMIENTO</t>
-        </is>
-      </c>
-      <c r="K7" s="105" t="inlineStr">
-        <is>
-          <t>SEGUIMIENTO</t>
-        </is>
-      </c>
-      <c r="L7" s="51" t="inlineStr">
-        <is>
-          <t>Entregado. Mob. exterior mediados sep.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="18" customHeight="1">
-      <c r="A8" s="99" t="inlineStr">
-        <is>
-          <t>ALCALÁ 58</t>
-        </is>
-      </c>
-      <c r="B8" s="100" t="inlineStr">
-        <is>
-          <t>VIVIENDA</t>
-        </is>
-      </c>
-      <c r="C8" s="101" t="inlineStr">
-        <is>
-          <t>Alicia/Javi</t>
-        </is>
-      </c>
-      <c r="D8" s="101" t="inlineStr">
-        <is>
-          <t>Fin de obra</t>
-        </is>
-      </c>
-      <c r="E8" s="101" t="inlineStr">
-        <is>
-          <t>Comunicar fecha nueva al cliente</t>
-        </is>
-      </c>
-      <c r="F8" s="101" t="inlineStr">
-        <is>
-          <t>Sep 2026</t>
-        </is>
-      </c>
-      <c r="G8" s="101" t="inlineStr">
-        <is>
-          <t>Va retrasado — cliente sin informar</t>
-        </is>
-      </c>
-      <c r="H8" s="101" t="inlineStr">
-        <is>
-          <t>Consultores Proy.</t>
-        </is>
-      </c>
-      <c r="I8" s="101" t="inlineStr">
-        <is>
-          <t>FIN OBRA</t>
-        </is>
-      </c>
-      <c r="J8" s="102" t="inlineStr">
-        <is>
-          <t>ATENCIÓN ALTA</t>
-        </is>
-      </c>
-      <c r="K8" s="102" t="inlineStr">
-        <is>
-          <t>ATENCIÓN ALTA</t>
-        </is>
-      </c>
-      <c r="L8" s="101" t="inlineStr">
-        <is>
-          <t>⚠ Va retrasado. Comunicar nueva fecha al cliente hoy.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="18" customHeight="1">
-      <c r="A9" s="99" t="inlineStr">
-        <is>
-          <t>LA FLORIDA</t>
-        </is>
-      </c>
-      <c r="B9" s="100" t="inlineStr">
-        <is>
-          <t>VIVIENDA</t>
-        </is>
-      </c>
-      <c r="C9" s="101" t="inlineStr">
-        <is>
-          <t>Paula</t>
-        </is>
-      </c>
-      <c r="D9" s="101" t="inlineStr">
-        <is>
-          <t>Obra en ejecución</t>
-        </is>
-      </c>
-      <c r="E9" s="101" t="inlineStr">
-        <is>
-          <t>Montaje última semana sep</t>
-        </is>
-      </c>
-      <c r="F9" s="101" t="inlineStr">
-        <is>
-          <t>Sep 2026</t>
-        </is>
-      </c>
-      <c r="G9" s="101" t="inlineStr">
-        <is>
-          <t>Paula debe visitar obra para confirmar fecha</t>
-        </is>
-      </c>
-      <c r="H9" s="101" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I9" s="101" t="inlineStr">
-        <is>
-          <t>OBRA</t>
-        </is>
-      </c>
-      <c r="J9" s="102" t="inlineStr">
-        <is>
-          <t>ATENCIÓN ALTA</t>
-        </is>
-      </c>
-      <c r="K9" s="102" t="inlineStr">
-        <is>
-          <t>ATENCIÓN ALTA</t>
-        </is>
-      </c>
-      <c r="L9" s="101" t="inlineStr">
-        <is>
-          <t>Deco organizada 2ª sem sep. Montaje última sem sep.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="18" customHeight="1">
-      <c r="A10" s="99" t="inlineStr">
-        <is>
-          <t>LA RINCONADA</t>
-        </is>
-      </c>
-      <c r="B10" s="100" t="inlineStr">
-        <is>
-          <t>VIVIENDA</t>
-        </is>
-      </c>
-      <c r="C10" s="101" t="inlineStr">
-        <is>
-          <t>Cristina/Nela</t>
-        </is>
-      </c>
-      <c r="D10" s="101" t="inlineStr">
-        <is>
-          <t>Obra en ejecución</t>
-        </is>
-      </c>
-      <c r="E10" s="101" t="inlineStr">
-        <is>
-          <t>FIN OBRA fin oct · Entrega deco nov</t>
-        </is>
-      </c>
-      <c r="F10" s="101" t="inlineStr">
-        <is>
-          <t>Nov 2026</t>
-        </is>
-      </c>
-      <c r="G10" s="101" t="inlineStr">
-        <is>
-          <t>⚠ Presu deco sin enviar — Ale revisar URGENTE</t>
-        </is>
-      </c>
-      <c r="H10" s="101" t="inlineStr">
-        <is>
-          <t>Raúl</t>
-        </is>
-      </c>
-      <c r="I10" s="101" t="inlineStr">
-        <is>
-          <t>OBRA</t>
-        </is>
-      </c>
-      <c r="J10" s="102" t="inlineStr">
-        <is>
-          <t>ATENCIÓN ALTA</t>
-        </is>
-      </c>
-      <c r="K10" s="102" t="inlineStr">
-        <is>
-          <t>ATENCIÓN ALTA</t>
-        </is>
-      </c>
-      <c r="L10" s="101" t="inlineStr">
-        <is>
-          <t>Presu deco pendiente revisión Ale. FIN OBRA fin oct (pdte aceptación). Entrega nov.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="18" customHeight="1">
-      <c r="A11" s="99" t="inlineStr">
-        <is>
-          <t>VIUDA DE ALDAMA 3</t>
-        </is>
-      </c>
-      <c r="B11" s="100" t="inlineStr">
-        <is>
-          <t>VIVIENDA</t>
-        </is>
-      </c>
-      <c r="C11" s="101" t="inlineStr">
-        <is>
-          <t>Nela/Andrea</t>
-        </is>
-      </c>
-      <c r="D11" s="101" t="inlineStr">
-        <is>
-          <t>Proyecto ejecución</t>
-        </is>
-      </c>
-      <c r="E11" s="101" t="inlineStr">
-        <is>
-          <t>Reunión jue 3 sep (Natalia+Raúl+Ale+Nela)</t>
-        </is>
-      </c>
-      <c r="F11" s="101" t="inlineStr">
-        <is>
-          <t>Nov 2026</t>
-        </is>
-      </c>
-      <c r="G11" s="101" t="inlineStr">
-        <is>
-          <t>Presupuestos obra+deco pendientes actualizar</t>
-        </is>
-      </c>
-      <c r="H11" s="101" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I11" s="101" t="inlineStr">
-        <is>
-          <t>PROY E</t>
-        </is>
-      </c>
-      <c r="J11" s="102" t="inlineStr">
-        <is>
-          <t>ATENCIÓN ALTA</t>
-        </is>
-      </c>
-      <c r="K11" s="102" t="inlineStr">
-        <is>
-          <t>ATENCIÓN ALTA</t>
-        </is>
-      </c>
-      <c r="L11" s="101" t="inlineStr">
-        <is>
-          <t>Reunión 3 sep. Objetivo: arrancar obra septiembre.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="18" customHeight="1">
-      <c r="A12" s="103" t="inlineStr">
-        <is>
-          <t>VIUDA DE ALDAMA 2</t>
-        </is>
-      </c>
-      <c r="B12" s="104" t="inlineStr">
-        <is>
-          <t>VIVIENDA</t>
-        </is>
-      </c>
-      <c r="C12" s="51" t="inlineStr">
-        <is>
-          <t>Sin asignar</t>
-        </is>
-      </c>
-      <c r="D12" s="51" t="inlineStr">
-        <is>
-          <t>Proyecto nuevo</t>
-        </is>
-      </c>
-      <c r="E12" s="51" t="inlineStr">
-        <is>
-          <t>Organizar con cliente en septiembre</t>
-        </is>
-      </c>
-      <c r="F12" s="51" t="inlineStr">
-        <is>
-          <t>2027</t>
-        </is>
-      </c>
-      <c r="G12" s="51" t="inlineStr">
-        <is>
-          <t>Sin responsable asignado</t>
-        </is>
-      </c>
-      <c r="H12" s="51" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I12" s="51" t="inlineStr">
-        <is>
-          <t>PENDIENTE</t>
-        </is>
-      </c>
-      <c r="J12" s="105" t="inlineStr">
-        <is>
-          <t>SEGUIMIENTO</t>
-        </is>
-      </c>
-      <c r="K12" s="105" t="inlineStr">
-        <is>
-          <t>SEGUIMIENTO</t>
-        </is>
-      </c>
-      <c r="L12" s="51" t="inlineStr">
-        <is>
-          <t>Nuevo proyecto. Arranque septiembre.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="18" customHeight="1">
-      <c r="A13" s="99" t="inlineStr">
-        <is>
-          <t>SANTANDER VIV</t>
-        </is>
-      </c>
-      <c r="B13" s="100" t="inlineStr">
-        <is>
-          <t>VIVIENDA</t>
-        </is>
-      </c>
-      <c r="C13" s="101" t="inlineStr">
-        <is>
-          <t>Sara</t>
-        </is>
-      </c>
-      <c r="D13" s="101" t="inlineStr">
-        <is>
-          <t>Obra en ejecución</t>
-        </is>
-      </c>
-      <c r="E13" s="101" t="inlineStr">
-        <is>
-          <t>Visita obra 14 sep · Deco sem 21 sep</t>
-        </is>
-      </c>
-      <c r="F13" s="101" t="inlineStr">
-        <is>
-          <t>Dic 2026</t>
-        </is>
-      </c>
-      <c r="G13" s="101" t="inlineStr">
-        <is>
-          <t>Muchas decisiones pendientes de cliente</t>
-        </is>
-      </c>
-      <c r="H13" s="101" t="inlineStr">
-        <is>
-          <t>Constructora cliente</t>
-        </is>
-      </c>
-      <c r="I13" s="101" t="inlineStr">
-        <is>
-          <t>PROY E</t>
-        </is>
-      </c>
-      <c r="J13" s="102" t="inlineStr">
-        <is>
-          <t>ATENCIÓN ALTA</t>
-        </is>
-      </c>
-      <c r="K13" s="102" t="inlineStr">
-        <is>
-          <t>ATENCIÓN ALTA</t>
-        </is>
-      </c>
-      <c r="L13" s="101" t="inlineStr">
-        <is>
-          <t>Visita 14 sep. Reuniones deco sem 21 sep. Montaje dic.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="18" customHeight="1">
-      <c r="A14" s="103" t="inlineStr">
-        <is>
-          <t>IBIZA</t>
-        </is>
-      </c>
-      <c r="B14" s="104" t="inlineStr">
-        <is>
-          <t>VIVIENDA</t>
-        </is>
-      </c>
-      <c r="C14" s="51" t="inlineStr">
-        <is>
-          <t>Sara</t>
-        </is>
-      </c>
-      <c r="D14" s="51" t="inlineStr">
-        <is>
-          <t>Obra parada (municipio)</t>
-        </is>
-      </c>
-      <c r="E14" s="51" t="inlineStr">
-        <is>
-          <t>Reanudar sep · Preparar deco</t>
-        </is>
-      </c>
-      <c r="F14" s="51" t="inlineStr">
-        <is>
-          <t>Dic 2026</t>
-        </is>
-      </c>
-      <c r="G14" s="51" t="inlineStr">
-        <is>
-          <t>Obra parada por municipio. Pagos pendientes clientes.</t>
-        </is>
-      </c>
-      <c r="H14" s="51" t="inlineStr">
-        <is>
-          <t>Albañil local</t>
-        </is>
-      </c>
-      <c r="I14" s="51" t="inlineStr">
-        <is>
-          <t>PDTE LIC</t>
-        </is>
-      </c>
-      <c r="J14" s="105" t="inlineStr">
-        <is>
-          <t>SEGUIMIENTO</t>
-        </is>
-      </c>
-      <c r="K14" s="105" t="inlineStr">
-        <is>
-          <t>SEGUIMIENTO</t>
-        </is>
-      </c>
-      <c r="L14" s="51" t="inlineStr">
-        <is>
-          <t>Parada hasta sep. Arrancar proy deco al reanudar. Montaje dic.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="18" customHeight="1">
-      <c r="A15" s="103" t="inlineStr">
-        <is>
-          <t>HERMOSILLA</t>
-        </is>
-      </c>
-      <c r="B15" s="104" t="inlineStr">
-        <is>
-          <t>VIVIENDA</t>
-        </is>
-      </c>
-      <c r="C15" s="51" t="inlineStr">
-        <is>
-          <t>Nela/Olatz</t>
-        </is>
-      </c>
-      <c r="D15" s="51" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="E15" s="51" t="inlineStr">
-        <is>
-          <t>Olatz contactar cliente al volver</t>
-        </is>
-      </c>
-      <c r="F15" s="51" t="inlineStr">
-        <is>
-          <t>Mar 2027</t>
-        </is>
-      </c>
-      <c r="G15" s="51" t="inlineStr">
-        <is>
-          <t>Sin info de cliente ni constructora</t>
-        </is>
-      </c>
-      <c r="H15" s="51" t="inlineStr">
-        <is>
-          <t>Raumplan</t>
-        </is>
-      </c>
-      <c r="I15" s="51" t="inlineStr">
-        <is>
-          <t>PENDIENTE</t>
-        </is>
-      </c>
-      <c r="J15" s="105" t="inlineStr">
-        <is>
-          <t>SEGUIMIENTO</t>
-        </is>
-      </c>
-      <c r="K15" s="105" t="inlineStr">
-        <is>
-          <t>SEGUIMIENTO</t>
-        </is>
-      </c>
-      <c r="L15" s="51" t="inlineStr">
-        <is>
-          <t>Sin noticias. Olatz contactar al volver.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="18" customHeight="1">
-      <c r="A16" s="99" t="inlineStr">
-        <is>
-          <t>MONTESQUINZA</t>
-        </is>
-      </c>
-      <c r="B16" s="100" t="inlineStr">
-        <is>
-          <t>VIVIENDA</t>
-        </is>
-      </c>
-      <c r="C16" s="101" t="inlineStr">
-        <is>
-          <t>Sara</t>
-        </is>
-      </c>
-      <c r="D16" s="101" t="inlineStr">
-        <is>
-          <t>Obra en ejecución</t>
-        </is>
-      </c>
-      <c r="E16" s="101" t="inlineStr">
-        <is>
-          <t>Revisar notificación licencia/DR</t>
-        </is>
-      </c>
-      <c r="F16" s="101" t="inlineStr">
-        <is>
-          <t>Mar 2027</t>
-        </is>
-      </c>
-      <c r="G16" s="101" t="inlineStr">
-        <is>
-          <t>⚠ Notificación licencia/DR recibida pendiente revisar</t>
-        </is>
-      </c>
-      <c r="H16" s="101" t="inlineStr">
-        <is>
-          <t>Consultores Proy.</t>
-        </is>
-      </c>
-      <c r="I16" s="101" t="inlineStr">
-        <is>
-          <t>OBRA</t>
-        </is>
-      </c>
-      <c r="J16" s="102" t="inlineStr">
-        <is>
-          <t>ATENCIÓN ALTA</t>
-        </is>
-      </c>
-      <c r="K16" s="102" t="inlineStr">
-        <is>
-          <t>ATENCIÓN ALTA</t>
-        </is>
-      </c>
-      <c r="L16" s="101" t="inlineStr">
-        <is>
-          <t>Obra avanzando. Notificación DR — revisar urgente.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="18" customHeight="1">
-      <c r="A17" s="103" t="inlineStr">
-        <is>
-          <t>GAMAL STO. DOMINGO</t>
-        </is>
-      </c>
-      <c r="B17" s="104" t="inlineStr">
-        <is>
-          <t>VIVIENDA</t>
-        </is>
-      </c>
-      <c r="C17" s="51" t="inlineStr">
-        <is>
-          <t>Sofía/Olatz</t>
-        </is>
-      </c>
-      <c r="D17" s="51" t="inlineStr">
-        <is>
-          <t>Montaje realizado</t>
-        </is>
-      </c>
-      <c r="E17" s="51" t="inlineStr">
-        <is>
-          <t>Confirmar remates o cierre</t>
-        </is>
-      </c>
-      <c r="F17" s="51" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G17" s="51" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H17" s="51" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I17" s="51" t="inlineStr">
-        <is>
-          <t>REMATES</t>
-        </is>
-      </c>
-      <c r="J17" s="105" t="inlineStr">
-        <is>
-          <t>SEGUIMIENTO</t>
-        </is>
-      </c>
-      <c r="K17" s="105" t="inlineStr">
-        <is>
-          <t>SEGUIMIENTO</t>
-        </is>
-      </c>
-      <c r="L17" s="51" t="inlineStr">
-        <is>
-          <t>Montaje realizado. Confirmar si hay remates o se cierra.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="18" customHeight="1">
-      <c r="A18" s="99" t="inlineStr">
-        <is>
-          <t>CAMINO SUR 70</t>
-        </is>
-      </c>
-      <c r="B18" s="100" t="inlineStr">
-        <is>
-          <t>VIVIENDA</t>
-        </is>
-      </c>
-      <c r="C18" s="101" t="inlineStr">
-        <is>
-          <t>Cristina/Nela</t>
-        </is>
-      </c>
-      <c r="D18" s="101" t="inlineStr">
-        <is>
-          <t>Remates</t>
-        </is>
-      </c>
-      <c r="E18" s="101" t="inlineStr">
-        <is>
-          <t>Fallos Contraluz iluminación</t>
-        </is>
-      </c>
-      <c r="F18" s="101" t="inlineStr">
-        <is>
-          <t>Sep 2026</t>
-        </is>
-      </c>
-      <c r="G18" s="101" t="inlineStr">
-        <is>
-          <t>Fallos grandes Contraluz. Remates papel pendientes.</t>
-        </is>
-      </c>
-      <c r="H18" s="101" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I18" s="101" t="inlineStr">
-        <is>
-          <t>REMATES</t>
-        </is>
-      </c>
-      <c r="J18" s="102" t="inlineStr">
-        <is>
-          <t>ATENCIÓN ALTA</t>
-        </is>
-      </c>
-      <c r="K18" s="102" t="inlineStr">
-        <is>
-          <t>ATENCIÓN ALTA</t>
-        </is>
-      </c>
-      <c r="L18" s="101" t="inlineStr">
-        <is>
-          <t>Visita clientes 1 sep. Fallos Contraluz iluminación. Remates papel.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="18" customHeight="1">
-      <c r="A19" s="103" t="inlineStr">
-        <is>
-          <t>CAMINO SUR 35</t>
-        </is>
-      </c>
-      <c r="B19" s="104" t="inlineStr">
-        <is>
-          <t>VIVIENDA</t>
-        </is>
-      </c>
-      <c r="C19" s="51" t="inlineStr">
-        <is>
-          <t>Nela</t>
-        </is>
-      </c>
-      <c r="D19" s="51" t="inlineStr">
-        <is>
-          <t>Renders en curso</t>
-        </is>
-      </c>
-      <c r="E19" s="51" t="inlineStr">
-        <is>
-          <t>6 fases de renders — sin deco todavía</t>
-        </is>
-      </c>
-      <c r="F19" s="51" t="inlineStr">
-        <is>
-          <t>2027</t>
-        </is>
-      </c>
-      <c r="G19" s="51" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H19" s="51" t="inlineStr">
-        <is>
-          <t>Project Work</t>
-        </is>
-      </c>
-      <c r="I19" s="51" t="inlineStr">
-        <is>
-          <t>RENDERS</t>
-        </is>
-      </c>
-      <c r="J19" s="105" t="inlineStr">
-        <is>
-          <t>SEGUIMIENTO</t>
-        </is>
-      </c>
-      <c r="K19" s="105" t="inlineStr">
-        <is>
-          <t>SEGUIMIENTO</t>
-        </is>
-      </c>
-      <c r="L19" s="51" t="inlineStr">
-        <is>
-          <t>Pancho con correcciones renders (6 fases). Sin deco.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="18" customHeight="1">
-      <c r="A20" s="103" t="inlineStr">
-        <is>
-          <t>TORRE VALENCIA</t>
-        </is>
-      </c>
-      <c r="B20" s="104" t="inlineStr">
-        <is>
-          <t>VIVIENDA</t>
-        </is>
-      </c>
-      <c r="C20" s="51" t="inlineStr">
-        <is>
-          <t>Paula</t>
-        </is>
-      </c>
-      <c r="D20" s="51" t="inlineStr">
-        <is>
-          <t>Proyecto ejecución</t>
-        </is>
-      </c>
-      <c r="E20" s="51" t="inlineStr">
-        <is>
-          <t>Paula visita próxima sem</t>
-        </is>
-      </c>
-      <c r="F20" s="51" t="inlineStr">
-        <is>
-          <t>2027</t>
-        </is>
-      </c>
-      <c r="G20" s="51" t="inlineStr">
-        <is>
-          <t>Cliente sin decisiones domótica</t>
-        </is>
-      </c>
-      <c r="H20" s="51" t="inlineStr">
-        <is>
-          <t>Ecobuild</t>
-        </is>
-      </c>
-      <c r="I20" s="51" t="inlineStr">
-        <is>
-          <t>PROY E</t>
-        </is>
-      </c>
-      <c r="J20" s="105" t="inlineStr">
-        <is>
-          <t>SEGUIMIENTO</t>
-        </is>
-      </c>
-      <c r="K20" s="105" t="inlineStr">
-        <is>
-          <t>SEGUIMIENTO</t>
-        </is>
-      </c>
-      <c r="L20" s="51" t="inlineStr">
-        <is>
-          <t>Replanteo iluminación realizado. Cliente sin decisiones domótica.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="18" customHeight="1">
-      <c r="A21" s="103" t="inlineStr">
-        <is>
-          <t>PASEO LAGOS 105</t>
-        </is>
-      </c>
-      <c r="B21" s="104" t="inlineStr">
-        <is>
-          <t>VIVIENDA</t>
-        </is>
-      </c>
-      <c r="C21" s="51" t="inlineStr">
-        <is>
-          <t>Sara/Andrea</t>
-        </is>
-      </c>
-      <c r="D21" s="51" t="inlineStr">
-        <is>
-          <t>Proyecto básico</t>
-        </is>
-      </c>
-      <c r="E21" s="51" t="inlineStr">
-        <is>
-          <t>Reunión 15 sep · renders + presentación</t>
-        </is>
-      </c>
-      <c r="F21" s="51" t="inlineStr">
-        <is>
-          <t>2027</t>
-        </is>
-      </c>
-      <c r="G21" s="51" t="inlineStr">
-        <is>
-          <t>Obra retrasa a ppios 2027 (humedades)</t>
-        </is>
-      </c>
-      <c r="H21" s="51" t="inlineStr">
-        <is>
-          <t>Raúl/Jamena</t>
-        </is>
-      </c>
-      <c r="I21" s="51" t="inlineStr">
-        <is>
-          <t>PROY B</t>
-        </is>
-      </c>
-      <c r="J21" s="105" t="inlineStr">
-        <is>
-          <t>SEGUIMIENTO</t>
-        </is>
-      </c>
-      <c r="K21" s="105" t="inlineStr">
-        <is>
-          <t>SEGUIMIENTO</t>
-        </is>
-      </c>
-      <c r="L21" s="51" t="inlineStr">
-        <is>
-          <t>Reunión 15 sep. Obra ppios 2027.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="18" customHeight="1">
-      <c r="A22" s="103" t="inlineStr">
-        <is>
-          <t>VALCARCE</t>
-        </is>
-      </c>
-      <c r="B22" s="104" t="inlineStr">
-        <is>
-          <t>VIVIENDA</t>
-        </is>
-      </c>
-      <c r="C22" s="51" t="inlineStr">
-        <is>
-          <t>Paula</t>
-        </is>
-      </c>
-      <c r="D22" s="51" t="inlineStr">
-        <is>
-          <t>Remates</t>
-        </is>
-      </c>
-      <c r="E22" s="51" t="inlineStr">
-        <is>
-          <t>Remates papel y Raúl pendientes</t>
-        </is>
-      </c>
-      <c r="F22" s="51" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G22" s="51" t="inlineStr">
-        <is>
-          <t>David (empapelador) da largas</t>
-        </is>
-      </c>
-      <c r="H22" s="51" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I22" s="51" t="inlineStr">
-        <is>
-          <t>REMATES</t>
-        </is>
-      </c>
-      <c r="J22" s="105" t="inlineStr">
-        <is>
-          <t>SEGUIMIENTO</t>
-        </is>
-      </c>
-      <c r="K22" s="105" t="inlineStr">
-        <is>
-          <t>SEGUIMIENTO</t>
-        </is>
-      </c>
-      <c r="L22" s="51" t="inlineStr">
-        <is>
-          <t>Remates papel (David). Remates Raúl: cliente espere 2 semanas.</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="18" customHeight="1">
-      <c r="A23" s="103" t="inlineStr">
-        <is>
-          <t>PESQUERA</t>
-        </is>
-      </c>
-      <c r="B23" s="104" t="inlineStr">
-        <is>
-          <t>VIVIENDA</t>
-        </is>
-      </c>
-      <c r="C23" s="51" t="inlineStr">
-        <is>
-          <t>Paula</t>
-        </is>
-      </c>
-      <c r="D23" s="51" t="inlineStr">
-        <is>
-          <t>Pedidos</t>
-        </is>
-      </c>
-      <c r="E23" s="51" t="inlineStr">
-        <is>
-          <t>Deco en oficina pendiente enviar</t>
-        </is>
-      </c>
-      <c r="F23" s="51" t="inlineStr">
-        <is>
-          <t>Dic 2026</t>
-        </is>
-      </c>
-      <c r="G23" s="51" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H23" s="51" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I23" s="51" t="inlineStr">
-        <is>
-          <t>PEDIDOS</t>
-        </is>
-      </c>
-      <c r="J23" s="105" t="inlineStr">
-        <is>
-          <t>SEGUIMIENTO</t>
-        </is>
-      </c>
-      <c r="K23" s="105" t="inlineStr">
-        <is>
-          <t>SEGUIMIENTO</t>
-        </is>
-      </c>
-      <c r="L23" s="51" t="inlineStr">
-        <is>
-          <t>Deco en oficina pdte enviar. Constructora en marcha. Cliente: navidades.</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="18" customHeight="1">
-      <c r="A24" s="99" t="inlineStr">
-        <is>
-          <t>PASEO LAGOS 121</t>
-        </is>
-      </c>
-      <c r="B24" s="100" t="inlineStr">
-        <is>
-          <t>VIVIENDA</t>
-        </is>
-      </c>
-      <c r="C24" s="101" t="inlineStr">
-        <is>
-          <t>Olatz</t>
-        </is>
-      </c>
-      <c r="D24" s="101" t="inlineStr">
-        <is>
-          <t>Proyecto deco</t>
-        </is>
-      </c>
-      <c r="E24" s="101" t="inlineStr">
-        <is>
-          <t>Reunión 2 sep · Presentación Nela</t>
-        </is>
-      </c>
-      <c r="F24" s="101" t="inlineStr">
-        <is>
-          <t>Feb 2027</t>
-        </is>
-      </c>
-      <c r="G24" s="101" t="inlineStr">
-        <is>
-          <t>Presentación pendiente revisión Ale — URGENTE</t>
-        </is>
-      </c>
-      <c r="H24" s="101" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I24" s="101" t="inlineStr">
-        <is>
-          <t>PROY DECO</t>
-        </is>
-      </c>
-      <c r="J24" s="102" t="inlineStr">
-        <is>
-          <t>ATENCIÓN ALTA</t>
-        </is>
-      </c>
-      <c r="K24" s="102" t="inlineStr">
-        <is>
-          <t>ATENCIÓN ALTA</t>
-        </is>
-      </c>
-      <c r="L24" s="101" t="inlineStr">
-        <is>
-          <t>⚠ Reunión 2 sep. Presentación Nela — Ale revisar URGENTE.</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="18" customHeight="1">
-      <c r="A25" s="103" t="inlineStr">
-        <is>
-          <t>VIV PALOMA RD</t>
-        </is>
-      </c>
-      <c r="B25" s="104" t="inlineStr">
-        <is>
-          <t>VIVIENDA</t>
-        </is>
-      </c>
-      <c r="C25" s="51" t="inlineStr">
-        <is>
-          <t>Olatz/Andrea</t>
-        </is>
-      </c>
-      <c r="D25" s="51" t="inlineStr">
-        <is>
-          <t>Proyecto deco</t>
-        </is>
-      </c>
-      <c r="E25" s="51" t="inlineStr">
-        <is>
-          <t>Reunión septiembre</t>
-        </is>
-      </c>
-      <c r="F25" s="51" t="inlineStr">
-        <is>
-          <t>Jul 2027</t>
-        </is>
-      </c>
-      <c r="G25" s="51" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H25" s="51" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I25" s="51" t="inlineStr">
-        <is>
-          <t>PROY DECO</t>
-        </is>
-      </c>
-      <c r="J25" s="105" t="inlineStr">
-        <is>
-          <t>SEGUIMIENTO</t>
-        </is>
-      </c>
-      <c r="K25" s="105" t="inlineStr">
-        <is>
-          <t>SEGUIMIENTO</t>
-        </is>
-      </c>
-      <c r="L25" s="51" t="inlineStr">
-        <is>
-          <t>Reunión agosto con Ale. Siguiente sep.</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="18" customHeight="1">
-      <c r="A26" s="103" t="inlineStr">
-        <is>
-          <t>TEPEYAC</t>
-        </is>
-      </c>
-      <c r="B26" s="104" t="inlineStr">
-        <is>
-          <t>VIVIENDA</t>
-        </is>
-      </c>
-      <c r="C26" s="51" t="inlineStr">
-        <is>
-          <t>Paula</t>
-        </is>
-      </c>
-      <c r="D26" s="51" t="inlineStr">
-        <is>
-          <t>Parado</t>
-        </is>
-      </c>
-      <c r="E26" s="51" t="inlineStr">
-        <is>
-          <t>Reunión pendiente Raúl+Paula+cliente</t>
-        </is>
-      </c>
-      <c r="F26" s="51" t="inlineStr">
-        <is>
-          <t>2027</t>
-        </is>
-      </c>
-      <c r="G26" s="51" t="inlineStr">
-        <is>
-          <t>Sin reunión programada</t>
-        </is>
-      </c>
-      <c r="H26" s="51" t="inlineStr">
-        <is>
-          <t>Raúl</t>
-        </is>
-      </c>
-      <c r="I26" s="51" t="inlineStr">
-        <is>
-          <t>PENDIENTE</t>
-        </is>
-      </c>
-      <c r="J26" s="105" t="inlineStr">
-        <is>
-          <t>SEGUIMIENTO</t>
-        </is>
-      </c>
-      <c r="K26" s="105" t="inlineStr">
-        <is>
-          <t>SEGUIMIENTO</t>
-        </is>
-      </c>
-      <c r="L26" s="51" t="inlineStr">
-        <is>
-          <t>Parado. Reunión pdte para presupuesto obra.</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="18" customHeight="1">
-      <c r="A27" s="103" t="inlineStr">
-        <is>
-          <t>ABUBILLA</t>
-        </is>
-      </c>
-      <c r="B27" s="104" t="inlineStr">
-        <is>
-          <t>VIVIENDA</t>
-        </is>
-      </c>
-      <c r="C27" s="51" t="inlineStr">
-        <is>
-          <t>Paula</t>
-        </is>
-      </c>
-      <c r="D27" s="51" t="inlineStr">
-        <is>
-          <t>Remates</t>
-        </is>
-      </c>
-      <c r="E27" s="51" t="inlineStr">
-        <is>
-          <t>Semana del 7 sep</t>
-        </is>
-      </c>
-      <c r="F27" s="51" t="inlineStr">
-        <is>
-          <t>Sep 2026</t>
-        </is>
-      </c>
-      <c r="G27" s="51" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H27" s="51" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I27" s="51" t="inlineStr">
-        <is>
-          <t>REMATES</t>
-        </is>
-      </c>
-      <c r="J27" s="105" t="inlineStr">
-        <is>
-          <t>SEGUIMIENTO</t>
-        </is>
-      </c>
-      <c r="K27" s="105" t="inlineStr">
-        <is>
-          <t>SEGUIMIENTO</t>
-        </is>
-      </c>
-      <c r="L27" s="51" t="inlineStr">
-        <is>
-          <t>Remates sofá y cortinas. Semana del 7 sep.</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="18" customHeight="1">
-      <c r="A28" s="106" t="inlineStr">
-        <is>
-          <t>FOX + LA DESPENSA</t>
-        </is>
-      </c>
-      <c r="B28" s="107" t="inlineStr">
-        <is>
-          <t>RESTAURANTES</t>
-        </is>
-      </c>
-      <c r="C28" s="51" t="inlineStr">
-        <is>
-          <t>Sofía/Naiara</t>
-        </is>
-      </c>
-      <c r="D28" s="51" t="inlineStr">
-        <is>
-          <t>Remates</t>
-        </is>
-      </c>
-      <c r="E28" s="51" t="inlineStr">
-        <is>
-          <t>Apertura 23 sep</t>
-        </is>
-      </c>
-      <c r="F28" s="51" t="inlineStr">
-        <is>
-          <t>23 sep</t>
-        </is>
-      </c>
-      <c r="G28" s="51" t="inlineStr">
-        <is>
-          <t>Amboage pendiente antes del 17 sep</t>
-        </is>
-      </c>
-      <c r="H28" s="51" t="inlineStr">
-        <is>
-          <t>Amboage</t>
-        </is>
-      </c>
-      <c r="I28" s="51" t="inlineStr">
-        <is>
-          <t>REMATES</t>
-        </is>
-      </c>
-      <c r="J28" s="105" t="inlineStr">
-        <is>
-          <t>SEGUIMIENTO</t>
-        </is>
-      </c>
-      <c r="K28" s="105" t="inlineStr">
-        <is>
-          <t>SEGUIMIENTO</t>
-        </is>
-      </c>
-      <c r="L28" s="51" t="inlineStr">
-        <is>
-          <t>Amboage pdte antes 17 sep. Apertura 23 sep.</t>
-        </is>
-      </c>
-    </row>
-    <row r="29" ht="18" customHeight="1">
-      <c r="A29" s="108" t="inlineStr">
-        <is>
-          <t>PUERTO RICO</t>
-        </is>
-      </c>
-      <c r="B29" s="109" t="inlineStr">
-        <is>
-          <t>RESTAURANTES</t>
-        </is>
-      </c>
-      <c r="C29" s="101" t="inlineStr">
-        <is>
-          <t>Sofía</t>
-        </is>
-      </c>
-      <c r="D29" s="101" t="inlineStr">
-        <is>
-          <t>Proyecto ejecución</t>
-        </is>
-      </c>
-      <c r="E29" s="101" t="inlineStr">
-        <is>
-          <t>Mediciones 2ª sem oct</t>
-        </is>
-      </c>
-      <c r="F29" s="101" t="inlineStr">
-        <is>
-          <t>Mar/Abr 2027</t>
-        </is>
-      </c>
-      <c r="G29" s="101" t="inlineStr">
-        <is>
-          <t>Decidir carpintero (Amboage descartado)</t>
-        </is>
-      </c>
-      <c r="H29" s="101" t="inlineStr">
-        <is>
-          <t>Amboage(pdte cambio)</t>
-        </is>
-      </c>
-      <c r="I29" s="101" t="inlineStr">
-        <is>
-          <t>PROY E</t>
-        </is>
-      </c>
-      <c r="J29" s="102" t="inlineStr">
-        <is>
-          <t>ATENCIÓN ALTA</t>
-        </is>
-      </c>
-      <c r="K29" s="102" t="inlineStr">
-        <is>
-          <t>ATENCIÓN ALTA</t>
-        </is>
-      </c>
-      <c r="L29" s="101" t="inlineStr">
-        <is>
-          <t>Mediciones oct. Fab nov-ene. Instalación feb. Apertura mar/abr.</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" ht="18" customHeight="1">
-      <c r="A30" s="106" t="inlineStr">
-        <is>
-          <t>RUBAIYAT MADRID</t>
-        </is>
-      </c>
-      <c r="B30" s="107" t="inlineStr">
-        <is>
-          <t>RESTAURANTES</t>
-        </is>
-      </c>
-      <c r="C30" s="51" t="inlineStr">
-        <is>
-          <t>Naiara</t>
-        </is>
-      </c>
-      <c r="D30" s="51" t="inlineStr">
-        <is>
-          <t>Proyecto deco</t>
-        </is>
-      </c>
-      <c r="E30" s="51" t="inlineStr">
-        <is>
-          <t>Cerrar deco terraza sem sep</t>
-        </is>
-      </c>
-      <c r="F30" s="51" t="inlineStr">
-        <is>
-          <t>Sep 2026</t>
-        </is>
-      </c>
-      <c r="G30" s="51" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H30" s="51" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I30" s="51" t="inlineStr">
-        <is>
-          <t>PROY DECO</t>
-        </is>
-      </c>
-      <c r="J30" s="105" t="inlineStr">
-        <is>
-          <t>SEGUIMIENTO</t>
-        </is>
-      </c>
-      <c r="K30" s="105" t="inlineStr">
-        <is>
-          <t>SEGUIMIENTO</t>
-        </is>
-      </c>
-      <c r="L30" s="51" t="inlineStr">
-        <is>
-          <t>Cerrando deco terraza. Cortina, mueble, ampliación. Terminar sem sep.</t>
-        </is>
-      </c>
-    </row>
-    <row r="31" ht="18" customHeight="1">
-      <c r="A31" s="108" t="inlineStr">
-        <is>
-          <t>RUBAIYAT SÃO PAULO</t>
-        </is>
-      </c>
-      <c r="B31" s="109" t="inlineStr">
-        <is>
-          <t>RESTAURANTES</t>
-        </is>
-      </c>
-      <c r="C31" s="101" t="inlineStr">
-        <is>
-          <t>Naiara</t>
-        </is>
-      </c>
-      <c r="D31" s="101" t="inlineStr">
-        <is>
-          <t>Anteproyecto</t>
-        </is>
-      </c>
-      <c r="E31" s="101" t="inlineStr">
-        <is>
-          <t>Viaje 29 sep (2 noches)</t>
-        </is>
-      </c>
-      <c r="F31" s="101" t="inlineStr">
-        <is>
-          <t>2027</t>
-        </is>
-      </c>
-      <c r="G31" s="101" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H31" s="101" t="inlineStr">
-        <is>
-          <t>Constructora local</t>
-        </is>
-      </c>
-      <c r="I31" s="101" t="inlineStr">
-        <is>
-          <t>ANT.PROY</t>
-        </is>
-      </c>
-      <c r="J31" s="102" t="inlineStr">
-        <is>
-          <t>ATENCIÓN ALTA</t>
-        </is>
-      </c>
-      <c r="K31" s="102" t="inlineStr">
-        <is>
-          <t>ATENCIÓN ALTA</t>
-        </is>
-      </c>
-      <c r="L31" s="101" t="inlineStr">
-        <is>
-          <t>Preparar anteproyecto. Revisión ~22 sep. Viaje 29 sep. Obra enero por fases.</t>
-        </is>
-      </c>
-    </row>
-    <row r="32" ht="18" customHeight="1">
-      <c r="A32" s="106" t="inlineStr">
-        <is>
-          <t>BERNABÉU</t>
-        </is>
-      </c>
-      <c r="B32" s="107" t="inlineStr">
-        <is>
-          <t>RESTAURANTES</t>
-        </is>
-      </c>
-      <c r="C32" s="51" t="inlineStr">
-        <is>
-          <t>Naiara</t>
-        </is>
-      </c>
-      <c r="D32" s="51" t="inlineStr">
-        <is>
-          <t>Terminado — pendiente cierre</t>
-        </is>
-      </c>
-      <c r="E32" s="51" t="inlineStr">
-        <is>
-          <t>Cierre oficial: números + mesa + perchas</t>
-        </is>
-      </c>
-      <c r="F32" s="51" t="inlineStr">
-        <is>
-          <t>Sep 2026</t>
-        </is>
-      </c>
-      <c r="G32" s="51" t="inlineStr">
-        <is>
-          <t>Mesas estropeadas: decisión cliente pendiente</t>
-        </is>
-      </c>
-      <c r="H32" s="51" t="inlineStr">
-        <is>
-          <t>Consultores Proy.</t>
-        </is>
-      </c>
-      <c r="I32" s="51" t="inlineStr">
-        <is>
-          <t>CIERRE</t>
-        </is>
-      </c>
-      <c r="J32" s="105" t="inlineStr">
-        <is>
-          <t>SEGUIMIENTO</t>
-        </is>
-      </c>
-      <c r="K32" s="105" t="inlineStr">
-        <is>
-          <t>SEGUIMIENTO</t>
-        </is>
-      </c>
-      <c r="L32" s="51" t="inlineStr">
-        <is>
-          <t>Terminado. Pendiente cierre oficial.</t>
-        </is>
-      </c>
-    </row>
-    <row r="33" ht="18" customHeight="1">
-      <c r="A33" s="108" t="inlineStr">
-        <is>
-          <t>MALLORCA SEVILLA</t>
-        </is>
-      </c>
-      <c r="B33" s="109" t="inlineStr">
-        <is>
-          <t>RESTAURANTES</t>
-        </is>
-      </c>
-      <c r="C33" s="101" t="inlineStr">
-        <is>
-          <t>Sofía/Naiara</t>
-        </is>
-      </c>
-      <c r="D33" s="101" t="inlineStr">
-        <is>
-          <t>Obra</t>
-        </is>
-      </c>
-      <c r="E33" s="101" t="inlineStr">
-        <is>
-          <t>Reunión 1 sep · A construir</t>
-        </is>
-      </c>
-      <c r="F33" s="101" t="inlineStr">
-        <is>
-          <t>2027</t>
-        </is>
-      </c>
-      <c r="G33" s="101" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H33" s="101" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I33" s="101" t="inlineStr">
-        <is>
-          <t>OBRA</t>
-        </is>
-      </c>
-      <c r="J33" s="102" t="inlineStr">
-        <is>
-          <t>ATENCIÓN ALTA</t>
-        </is>
-      </c>
-      <c r="K33" s="102" t="inlineStr">
-        <is>
-          <t>ATENCIÓN ALTA</t>
-        </is>
-      </c>
-      <c r="L33" s="101" t="inlineStr">
-        <is>
-          <t>Licencia concedida. Demolición hecha. A construir.</t>
-        </is>
-      </c>
-    </row>
-    <row r="34" ht="18" customHeight="1">
-      <c r="A34" s="106" t="inlineStr">
-        <is>
-          <t>HIPÓDROMO</t>
-        </is>
-      </c>
-      <c r="B34" s="107" t="inlineStr">
-        <is>
-          <t>RESTAURANTES</t>
-        </is>
-      </c>
-      <c r="C34" s="51" t="inlineStr">
-        <is>
-          <t>Sofía/Naiara</t>
-        </is>
-      </c>
-      <c r="D34" s="51" t="inlineStr">
-        <is>
-          <t>Pendiente licencia</t>
-        </is>
-      </c>
-      <c r="E34" s="51" t="inlineStr">
-        <is>
-          <t>Hablar con María PM</t>
-        </is>
-      </c>
-      <c r="F34" s="51" t="inlineStr">
-        <is>
-          <t>Pdte</t>
-        </is>
-      </c>
-      <c r="G34" s="51" t="inlineStr">
-        <is>
-          <t>Sin noticias</t>
-        </is>
-      </c>
-      <c r="H34" s="51" t="inlineStr">
-        <is>
-          <t>4 constructoras</t>
-        </is>
-      </c>
-      <c r="I34" s="51" t="inlineStr">
-        <is>
-          <t>PDTE LIC</t>
-        </is>
-      </c>
-      <c r="J34" s="105" t="inlineStr">
-        <is>
-          <t>SEGUIMIENTO</t>
-        </is>
-      </c>
-      <c r="K34" s="105" t="inlineStr">
-        <is>
-          <t>SEGUIMIENTO</t>
-        </is>
-      </c>
-      <c r="L34" s="51" t="inlineStr">
-        <is>
-          <t>Sin noticias. Pendiente hablar con María PM.</t>
-        </is>
-      </c>
-    </row>
-    <row r="35" ht="18" customHeight="1">
-      <c r="A35" s="106" t="inlineStr">
-        <is>
-          <t>VIV JOANN (Anteproy.)</t>
-        </is>
-      </c>
-      <c r="B35" s="107" t="inlineStr">
-        <is>
-          <t>RESTAURANTES</t>
-        </is>
-      </c>
-      <c r="C35" s="51" t="inlineStr">
-        <is>
-          <t>Sofía</t>
-        </is>
-      </c>
-      <c r="D35" s="51" t="inlineStr">
-        <is>
-          <t>Proyecto básico</t>
-        </is>
-      </c>
-      <c r="E35" s="51" t="inlineStr">
-        <is>
-          <t>Arrancando PB</t>
-        </is>
-      </c>
-      <c r="F35" s="51" t="inlineStr">
-        <is>
-          <t>2027</t>
-        </is>
-      </c>
-      <c r="G35" s="51" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H35" s="51" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I35" s="51" t="inlineStr">
-        <is>
-          <t>PROY B</t>
-        </is>
-      </c>
-      <c r="J35" s="105" t="inlineStr">
-        <is>
-          <t>SEGUIMIENTO</t>
-        </is>
-      </c>
-      <c r="K35" s="105" t="inlineStr">
-        <is>
-          <t>SEGUIMIENTO</t>
-        </is>
-      </c>
-      <c r="L35" s="51" t="inlineStr">
-        <is>
-          <t>Arrancando PB. Planning enviado. Obra desde 2027.</t>
-        </is>
-      </c>
-    </row>
-    <row r="36" ht="18" customHeight="1">
-      <c r="A36" s="108" t="inlineStr">
-        <is>
-          <t>COBUE</t>
-        </is>
-      </c>
-      <c r="B36" s="109" t="inlineStr">
-        <is>
-          <t>RESTAURANTES</t>
-        </is>
-      </c>
-      <c r="C36" s="101" t="inlineStr">
-        <is>
-          <t>Sofía/Naiara</t>
-        </is>
-      </c>
-      <c r="D36" s="101" t="inlineStr">
-        <is>
-          <t>Proyecto entregado · licitando</t>
-        </is>
-      </c>
-      <c r="E36" s="101" t="inlineStr">
-        <is>
-          <t>Apertura 21 enero</t>
-        </is>
-      </c>
-      <c r="F36" s="101" t="inlineStr">
-        <is>
-          <t>21 ene</t>
-        </is>
-      </c>
-      <c r="G36" s="101" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H36" s="101" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I36" s="101" t="inlineStr">
-        <is>
-          <t>OBRA</t>
-        </is>
-      </c>
-      <c r="J36" s="102" t="inlineStr">
-        <is>
-          <t>ATENCIÓN ALTA</t>
-        </is>
-      </c>
-      <c r="K36" s="102" t="inlineStr">
-        <is>
-          <t>ATENCIÓN ALTA</t>
-        </is>
-      </c>
-      <c r="L36" s="101" t="inlineStr">
-        <is>
-          <t>Entrega valoración+renders esta sem. Licitando. Apertura 21 ene.</t>
-        </is>
-      </c>
-    </row>
-    <row r="37" ht="18" customHeight="1">
-      <c r="A37" s="106" t="inlineStr">
-        <is>
-          <t>PASEO LAGOS 132</t>
-        </is>
-      </c>
-      <c r="B37" s="107" t="inlineStr">
-        <is>
-          <t>RESTAURANTES</t>
-        </is>
-      </c>
-      <c r="C37" s="51" t="inlineStr">
-        <is>
-          <t>Sofía/Naiara</t>
-        </is>
-      </c>
-      <c r="D37" s="51" t="inlineStr">
-        <is>
-          <t>Proyecto ejecución</t>
-        </is>
-      </c>
-      <c r="E37" s="51" t="inlineStr">
-        <is>
-          <t>Cerrar acabados y definiciones</t>
-        </is>
-      </c>
-      <c r="F37" s="51" t="inlineStr">
-        <is>
-          <t>May 2027</t>
-        </is>
-      </c>
-      <c r="G37" s="51" t="inlineStr">
-        <is>
-          <t>Pendiente cerrar acabados, techos, carpintería, iluminación</t>
-        </is>
-      </c>
-      <c r="H37" s="51" t="inlineStr">
-        <is>
-          <t>Ferbocar</t>
-        </is>
-      </c>
-      <c r="I37" s="51" t="inlineStr">
-        <is>
-          <t>PROY E</t>
-        </is>
-      </c>
-      <c r="J37" s="105" t="inlineStr">
-        <is>
-          <t>SEGUIMIENTO</t>
-        </is>
-      </c>
-      <c r="K37" s="105" t="inlineStr">
-        <is>
-          <t>SEGUIMIENTO</t>
-        </is>
-      </c>
-      <c r="L37" s="51" t="inlineStr">
-        <is>
-          <t>Pendiente cerrar: acabados, techos, carpintería, iluminación, domótica.</t>
-        </is>
-      </c>
-    </row>
-    <row r="38" ht="18" customHeight="1">
-      <c r="A38" s="106" t="inlineStr">
-        <is>
-          <t>CARBON</t>
-        </is>
-      </c>
-      <c r="B38" s="107" t="inlineStr">
-        <is>
-          <t>RESTAURANTES</t>
-        </is>
-      </c>
-      <c r="C38" s="51" t="inlineStr">
-        <is>
-          <t>Sofía</t>
-        </is>
-      </c>
-      <c r="D38" s="51" t="inlineStr">
-        <is>
-          <t>Remates</t>
-        </is>
-      </c>
-      <c r="E38" s="51" t="inlineStr">
-        <is>
-          <t>Ejecutar aislamiento acústico</t>
-        </is>
-      </c>
-      <c r="F38" s="51" t="inlineStr">
-        <is>
-          <t>Sep 2026</t>
-        </is>
-      </c>
-      <c r="G38" s="51" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H38" s="51" t="inlineStr">
-        <is>
-          <t>Empresa acústica</t>
-        </is>
-      </c>
-      <c r="I38" s="51" t="inlineStr">
-        <is>
-          <t>REMATES</t>
-        </is>
-      </c>
-      <c r="J38" s="105" t="inlineStr">
-        <is>
-          <t>SEGUIMIENTO</t>
-        </is>
-      </c>
-      <c r="K38" s="105" t="inlineStr">
-        <is>
-          <t>SEGUIMIENTO</t>
-        </is>
-      </c>
-      <c r="L38" s="51" t="inlineStr">
-        <is>
-          <t>Remate aislamiento acústico pendiente de ejecutar.</t>
-        </is>
-      </c>
-    </row>
-    <row r="39" ht="18" customHeight="1">
-      <c r="A39" s="106" t="inlineStr">
-        <is>
-          <t>CLÍNICA LONGEVIDAD</t>
-        </is>
-      </c>
-      <c r="B39" s="107" t="inlineStr">
-        <is>
-          <t>RESTAURANTES</t>
-        </is>
-      </c>
-      <c r="C39" s="51" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D39" s="51" t="inlineStr">
-        <is>
-          <t>Sin novedades</t>
-        </is>
-      </c>
-      <c r="E39" s="51" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F39" s="51" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G39" s="51" t="inlineStr">
-        <is>
-          <t>Sin feedback clientes</t>
-        </is>
-      </c>
-      <c r="H39" s="51" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I39" s="51" t="inlineStr">
-        <is>
-          <t>PENDIENTE</t>
-        </is>
-      </c>
-      <c r="J39" s="105" t="inlineStr">
-        <is>
-          <t>SEGUIMIENTO</t>
-        </is>
-      </c>
-      <c r="K39" s="105" t="inlineStr">
-        <is>
-          <t>SEGUIMIENTO</t>
-        </is>
-      </c>
-      <c r="L39" s="51" t="inlineStr">
-        <is>
-          <t>Sin novedades.</t>
-        </is>
-      </c>
-    </row>
-    <row r="40" ht="18" customHeight="1">
-      <c r="A40" s="110" t="inlineStr">
-        <is>
-          <t>DON RAMÓN</t>
-        </is>
-      </c>
-      <c r="B40" s="111" t="inlineStr">
-        <is>
-          <t>HOTELES</t>
-        </is>
-      </c>
-      <c r="C40" s="51" t="inlineStr">
-        <is>
-          <t>Marta</t>
-        </is>
-      </c>
-      <c r="D40" s="51" t="inlineStr">
-        <is>
-          <t>Remates</t>
-        </is>
-      </c>
-      <c r="E40" s="51" t="inlineStr">
-        <is>
-          <t>Revisión remates montaje 1 sep</t>
-        </is>
-      </c>
-      <c r="F40" s="51" t="inlineStr">
-        <is>
-          <t>Sep 2026</t>
-        </is>
-      </c>
-      <c r="G40" s="51" t="inlineStr">
-        <is>
-          <t>Problema mueble cocinas/carpintero (no resp. estudio)</t>
-        </is>
-      </c>
-      <c r="H40" s="51" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I40" s="51" t="inlineStr">
-        <is>
-          <t>REMATES</t>
-        </is>
-      </c>
-      <c r="J40" s="105" t="inlineStr">
-        <is>
-          <t>SEGUIMIENTO</t>
-        </is>
-      </c>
-      <c r="K40" s="105" t="inlineStr">
-        <is>
-          <t>SEGUIMIENTO</t>
-        </is>
-      </c>
-      <c r="L40" s="51" t="inlineStr">
-        <is>
-          <t>Montaje 1 sep realizado. Marta y Ale. Revisión remates.</t>
-        </is>
-      </c>
-    </row>
-    <row r="41" ht="18" customHeight="1">
-      <c r="A41" s="112" t="inlineStr">
-        <is>
-          <t>ONE SHOT BILBAO</t>
-        </is>
-      </c>
-      <c r="B41" s="113" t="inlineStr">
-        <is>
-          <t>HOTELES</t>
-        </is>
-      </c>
-      <c r="C41" s="101" t="inlineStr">
-        <is>
-          <t>Marta</t>
-        </is>
-      </c>
-      <c r="D41" s="101" t="inlineStr">
-        <is>
-          <t>Proyecto ejecución</t>
-        </is>
-      </c>
-      <c r="E41" s="101" t="inlineStr">
-        <is>
-          <t>Montaje fin oct</t>
-        </is>
-      </c>
-      <c r="F41" s="101" t="inlineStr">
-        <is>
-          <t>Oct 2026</t>
-        </is>
-      </c>
-      <c r="G41" s="101" t="inlineStr">
-        <is>
-          <t>⚠ Cliente+MO cambiaron elementos unilateralmente</t>
-        </is>
-      </c>
-      <c r="H41" s="101" t="inlineStr">
-        <is>
-          <t>Martínez Otero</t>
-        </is>
-      </c>
-      <c r="I41" s="101" t="inlineStr">
-        <is>
-          <t>PROY E</t>
-        </is>
-      </c>
-      <c r="J41" s="102" t="inlineStr">
-        <is>
-          <t>ATENCIÓN ALTA</t>
-        </is>
-      </c>
-      <c r="K41" s="102" t="inlineStr">
-        <is>
-          <t>ATENCIÓN ALTA</t>
-        </is>
-      </c>
-      <c r="L41" s="101" t="inlineStr">
-        <is>
-          <t>⚠ Hablar con MO. Fin oct. Visita 1-2 días montaje.</t>
-        </is>
-      </c>
-    </row>
-    <row r="42" ht="18" customHeight="1">
-      <c r="A42" s="110" t="inlineStr">
-        <is>
-          <t>ROCA MAYA</t>
-        </is>
-      </c>
-      <c r="B42" s="111" t="inlineStr">
-        <is>
-          <t>HOTELES</t>
-        </is>
-      </c>
-      <c r="C42" s="51" t="inlineStr">
-        <is>
-          <t>Marta/Jesús</t>
-        </is>
-      </c>
-      <c r="D42" s="51" t="inlineStr">
-        <is>
-          <t>Proyecto ejecución</t>
-        </is>
-      </c>
-      <c r="E42" s="51" t="inlineStr">
-        <is>
-          <t>Detalles listos sep → fabricar</t>
-        </is>
-      </c>
-      <c r="F42" s="51" t="inlineStr">
-        <is>
-          <t>Sem Santa</t>
-        </is>
-      </c>
-      <c r="G42" s="51" t="inlineStr">
-        <is>
-          <t>Sin detalle de climatización</t>
-        </is>
-      </c>
-      <c r="H42" s="51" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I42" s="51" t="inlineStr">
-        <is>
-          <t>PROY E</t>
-        </is>
-      </c>
-      <c r="J42" s="105" t="inlineStr">
-        <is>
-          <t>SEGUIMIENTO</t>
-        </is>
-      </c>
-      <c r="K42" s="105" t="inlineStr">
-        <is>
-          <t>SEGUIMIENTO</t>
-        </is>
-      </c>
-      <c r="L42" s="51" t="inlineStr">
-        <is>
-          <t>Muestras OK. Detalles listos sep→fabricar. Entrega Sem Santa: hab→ZZCC→azotea.</t>
-        </is>
-      </c>
-    </row>
-    <row r="43" ht="18" customHeight="1">
-      <c r="A43" s="110" t="inlineStr">
-        <is>
-          <t>HOTEL ÚNICO BCN</t>
-        </is>
-      </c>
-      <c r="B43" s="111" t="inlineStr">
-        <is>
-          <t>HOTELES</t>
-        </is>
-      </c>
-      <c r="C43" s="51" t="inlineStr">
-        <is>
-          <t>Marta</t>
-        </is>
-      </c>
-      <c r="D43" s="51" t="inlineStr">
-        <is>
-          <t>Proyecto ejecución</t>
-        </is>
-      </c>
-      <c r="E43" s="51" t="inlineStr">
-        <is>
-          <t>Entregar todo sep y licitar</t>
-        </is>
-      </c>
-      <c r="F43" s="51" t="inlineStr">
-        <is>
-          <t>Sep 2026</t>
-        </is>
-      </c>
-      <c r="G43" s="51" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H43" s="51" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I43" s="51" t="inlineStr">
-        <is>
-          <t>PROY E</t>
-        </is>
-      </c>
-      <c r="J43" s="105" t="inlineStr">
-        <is>
-          <t>SEGUIMIENTO</t>
-        </is>
-      </c>
-      <c r="K43" s="105" t="inlineStr">
-        <is>
-          <t>SEGUIMIENTO</t>
-        </is>
-      </c>
-      <c r="L43" s="51" t="inlineStr">
-        <is>
-          <t>Fichas técnicas definidas. Auna propuesto proveedor. Entregar sep y licitar.</t>
-        </is>
-      </c>
-    </row>
-    <row r="44" ht="18" customHeight="1">
-      <c r="A44" s="112" t="inlineStr">
-        <is>
-          <t>VÍA 66</t>
-        </is>
-      </c>
-      <c r="B44" s="113" t="inlineStr">
-        <is>
-          <t>HOTELES</t>
-        </is>
-      </c>
-      <c r="C44" s="101" t="inlineStr">
-        <is>
-          <t>Jesús</t>
-        </is>
-      </c>
-      <c r="D44" s="101" t="inlineStr">
-        <is>
-          <t>Proyecto ejecución</t>
-        </is>
-      </c>
-      <c r="E44" s="101" t="inlineStr">
-        <is>
-          <t>Entregadas 2ª+3ª plantas. ZZCC fase 2 enero</t>
-        </is>
-      </c>
-      <c r="F44" s="101" t="inlineStr">
-        <is>
-          <t>Ene 2027</t>
-        </is>
-      </c>
-      <c r="G44" s="101" t="inlineStr">
-        <is>
-          <t>⚠ Error interno muebles tipo. MO con retrasos.</t>
-        </is>
-      </c>
-      <c r="H44" s="101" t="inlineStr">
-        <is>
-          <t>Martínez Otero</t>
-        </is>
-      </c>
-      <c r="I44" s="101" t="inlineStr">
-        <is>
-          <t>PROY E</t>
-        </is>
-      </c>
-      <c r="J44" s="102" t="inlineStr">
-        <is>
-          <t>ATENCIÓN ALTA</t>
-        </is>
-      </c>
-      <c r="K44" s="102" t="inlineStr">
-        <is>
-          <t>ATENCIÓN ALTA</t>
-        </is>
-      </c>
-      <c r="L44" s="101" t="inlineStr">
-        <is>
-          <t>⚠ Muebles necesitan adaptación por habitación. ZZCC fase 2 enero.</t>
-        </is>
-      </c>
-    </row>
-    <row r="45" ht="18" customHeight="1">
-      <c r="A45" s="112" t="inlineStr">
-        <is>
-          <t>PSN PORTAL</t>
-        </is>
-      </c>
-      <c r="B45" s="113" t="inlineStr">
-        <is>
-          <t>HOTELES</t>
-        </is>
-      </c>
-      <c r="C45" s="101" t="inlineStr">
-        <is>
-          <t>Jesús</t>
-        </is>
-      </c>
-      <c r="D45" s="101" t="inlineStr">
-        <is>
-          <t>Proyecto ejecución</t>
-        </is>
-      </c>
-      <c r="E45" s="101" t="inlineStr">
-        <is>
-          <t>Entrega sep · Obra 1 nov</t>
-        </is>
-      </c>
-      <c r="F45" s="101" t="inlineStr">
-        <is>
-          <t>Nov 2026</t>
-        </is>
-      </c>
-      <c r="G45" s="101" t="inlineStr">
-        <is>
-          <t>Pendiente revisión Ale antes de entregar</t>
-        </is>
-      </c>
-      <c r="H45" s="101" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I45" s="101" t="inlineStr">
-        <is>
-          <t>PROY E</t>
-        </is>
-      </c>
-      <c r="J45" s="102" t="inlineStr">
-        <is>
-          <t>ATENCIÓN ALTA</t>
-        </is>
-      </c>
-      <c r="K45" s="102" t="inlineStr">
-        <is>
-          <t>ATENCIÓN ALTA</t>
-        </is>
-      </c>
-      <c r="L45" s="101" t="inlineStr">
-        <is>
-          <t>Entrega sep. Valoración Raúl fin sep. Obra 1 nov.</t>
-        </is>
-      </c>
-    </row>
-    <row r="46" ht="18" customHeight="1">
-      <c r="A46" s="112" t="inlineStr">
-        <is>
-          <t>CASA ALMAGRO</t>
-        </is>
-      </c>
-      <c r="B46" s="113" t="inlineStr">
-        <is>
-          <t>HOTELES</t>
-        </is>
-      </c>
-      <c r="C46" s="101" t="inlineStr">
-        <is>
-          <t>Jesús/Marta</t>
-        </is>
-      </c>
-      <c r="D46" s="101" t="inlineStr">
-        <is>
-          <t>Proyecto ejecución</t>
-        </is>
-      </c>
-      <c r="E46" s="101" t="inlineStr">
-        <is>
-          <t>Obra mediados nov/ppios dic</t>
-        </is>
-      </c>
-      <c r="F46" s="101" t="inlineStr">
-        <is>
-          <t>Feb 2027</t>
-        </is>
-      </c>
-      <c r="G46" s="101" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H46" s="101" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I46" s="101" t="inlineStr">
-        <is>
-          <t>PROY E</t>
-        </is>
-      </c>
-      <c r="J46" s="102" t="inlineStr">
-        <is>
-          <t>ATENCIÓN ALTA</t>
-        </is>
-      </c>
-      <c r="K46" s="102" t="inlineStr">
-        <is>
-          <t>ATENCIÓN ALTA</t>
-        </is>
-      </c>
-      <c r="L46" s="101" t="inlineStr">
-        <is>
-          <t>Kickoff realizado. Restaurante hotel Madrid. Obra nov/dic. ~2 meses. 200k€.</t>
-        </is>
-      </c>
-    </row>
-    <row r="47" ht="18" customHeight="1">
-      <c r="A47" s="110" t="inlineStr">
-        <is>
-          <t>HOTEL SEVILLA</t>
-        </is>
-      </c>
-      <c r="B47" s="111" t="inlineStr">
-        <is>
-          <t>HOTELES</t>
-        </is>
-      </c>
-      <c r="C47" s="51" t="inlineStr">
-        <is>
-          <t>Marta</t>
-        </is>
-      </c>
-      <c r="D47" s="51" t="inlineStr">
-        <is>
-          <t>Proyecto actualizado</t>
-        </is>
-      </c>
-      <c r="E47" s="51" t="inlineStr">
-        <is>
-          <t>Sin planning realista</t>
-        </is>
-      </c>
-      <c r="F47" s="51" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G47" s="51" t="inlineStr">
-        <is>
-          <t>Ampliación no aceptada. Obra casi parada.</t>
-        </is>
-      </c>
-      <c r="H47" s="51" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I47" s="51" t="inlineStr">
-        <is>
-          <t>PROY E</t>
-        </is>
-      </c>
-      <c r="J47" s="105" t="inlineStr">
-        <is>
-          <t>SEGUIMIENTO</t>
-        </is>
-      </c>
-      <c r="K47" s="105" t="inlineStr">
-        <is>
-          <t>SEGUIMIENTO</t>
-        </is>
-      </c>
-      <c r="L47" s="51" t="inlineStr">
-        <is>
-          <t>Proyecto actualizado. Ampliación no aceptada. Obra casi parada.</t>
-        </is>
-      </c>
-    </row>
-    <row r="48" ht="18" customHeight="1">
-      <c r="A48" s="110" t="inlineStr">
-        <is>
-          <t>HOTEL GIJÓN</t>
-        </is>
-      </c>
-      <c r="B48" s="111" t="inlineStr">
-        <is>
-          <t>HOTELES</t>
-        </is>
-      </c>
-      <c r="C48" s="51" t="inlineStr">
-        <is>
-          <t>Marta/Jesús</t>
-        </is>
-      </c>
-      <c r="D48" s="51" t="inlineStr">
-        <is>
-          <t>En espera</t>
-        </is>
-      </c>
-      <c r="E48" s="51" t="inlineStr">
-        <is>
-          <t>Pendiente últimos planos instalaciones</t>
-        </is>
-      </c>
-      <c r="F48" s="51" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G48" s="51" t="inlineStr">
-        <is>
-          <t>Problemas instalaciones condicionan techos</t>
-        </is>
-      </c>
-      <c r="H48" s="51" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I48" s="51" t="inlineStr">
-        <is>
-          <t>PENDIENTE</t>
-        </is>
-      </c>
-      <c r="J48" s="105" t="inlineStr">
-        <is>
-          <t>SEGUIMIENTO</t>
-        </is>
-      </c>
-      <c r="K48" s="105" t="inlineStr">
-        <is>
-          <t>SEGUIMIENTO</t>
-        </is>
-      </c>
-      <c r="L48" s="51" t="inlineStr">
-        <is>
-          <t>Problemas instalaciones. Pendiente últimos planos.</t>
-        </is>
-      </c>
-    </row>
-    <row r="49" ht="18" customHeight="1">
-      <c r="A49" s="110" t="inlineStr">
-        <is>
-          <t>VINCCI VALENCIA</t>
-        </is>
-      </c>
-      <c r="B49" s="111" t="inlineStr">
-        <is>
-          <t>HOTELES</t>
-        </is>
-      </c>
-      <c r="C49" s="51" t="inlineStr">
-        <is>
-          <t>Marta/Jesús</t>
-        </is>
-      </c>
-      <c r="D49" s="51" t="inlineStr">
-        <is>
-          <t>Proyecto entregado</t>
-        </is>
-      </c>
-      <c r="E49" s="51" t="inlineStr">
-        <is>
-          <t>Piloto enero 2027</t>
-        </is>
-      </c>
-      <c r="F49" s="51" t="inlineStr">
-        <is>
-          <t>Jul 2027</t>
-        </is>
-      </c>
-      <c r="G49" s="51" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H49" s="51" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I49" s="51" t="inlineStr">
-        <is>
-          <t>PROY E</t>
-        </is>
-      </c>
-      <c r="J49" s="105" t="inlineStr">
-        <is>
-          <t>SEGUIMIENTO</t>
-        </is>
-      </c>
-      <c r="K49" s="105" t="inlineStr">
-        <is>
-          <t>SEGUIMIENTO</t>
-        </is>
-      </c>
-      <c r="L49" s="51" t="inlineStr">
-        <is>
-          <t>Piloto enero 2027. Montaje final jul/ago 2027.</t>
-        </is>
-      </c>
-    </row>
-    <row r="50" ht="18" customHeight="1">
-      <c r="A50" s="110" t="inlineStr">
-        <is>
-          <t>MARTÍNEZ CAMPOS</t>
-        </is>
-      </c>
-      <c r="B50" s="111" t="inlineStr">
-        <is>
-          <t>HOTELES</t>
-        </is>
-      </c>
-      <c r="C50" s="51" t="inlineStr">
-        <is>
-          <t>Jesús</t>
-        </is>
-      </c>
-      <c r="D50" s="51" t="inlineStr">
-        <is>
-          <t>En espera</t>
-        </is>
-      </c>
-      <c r="E50" s="51" t="inlineStr">
-        <is>
-          <t>Reunión cuando vuelva Jesús</t>
-        </is>
-      </c>
-      <c r="F50" s="51" t="inlineStr">
-        <is>
-          <t>2027</t>
-        </is>
-      </c>
-      <c r="G50" s="51" t="inlineStr">
-        <is>
-          <t>Sin noticias</t>
-        </is>
-      </c>
-      <c r="H50" s="51" t="inlineStr">
-        <is>
-          <t>Raúl (previsto)</t>
-        </is>
-      </c>
-      <c r="I50" s="51" t="inlineStr">
-        <is>
-          <t>PENDIENTE</t>
-        </is>
-      </c>
-      <c r="J50" s="105" t="inlineStr">
-        <is>
-          <t>SEGUIMIENTO</t>
-        </is>
-      </c>
-      <c r="K50" s="105" t="inlineStr">
-        <is>
-          <t>SEGUIMIENTO</t>
-        </is>
-      </c>
-      <c r="L50" s="51" t="inlineStr">
-        <is>
-          <t>Sin noticias.</t>
-        </is>
-      </c>
-    </row>
-    <row r="51" ht="18" customHeight="1">
-      <c r="A51" s="110" t="inlineStr">
-        <is>
-          <t>CASA KORREOS</t>
-        </is>
-      </c>
-      <c r="B51" s="111" t="inlineStr">
-        <is>
-          <t>HOTELES</t>
-        </is>
-      </c>
-      <c r="C51" s="51" t="inlineStr">
-        <is>
-          <t>Jesús</t>
-        </is>
-      </c>
-      <c r="D51" s="51" t="inlineStr">
-        <is>
-          <t>En espera</t>
-        </is>
-      </c>
-      <c r="E51" s="51" t="inlineStr">
-        <is>
-          <t>Reunión cuando vuelva Jesús</t>
-        </is>
-      </c>
-      <c r="F51" s="51" t="inlineStr">
-        <is>
-          <t>2027</t>
-        </is>
-      </c>
-      <c r="G51" s="51" t="inlineStr">
-        <is>
-          <t>Sin noticias</t>
-        </is>
-      </c>
-      <c r="H51" s="51" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I51" s="51" t="inlineStr">
-        <is>
-          <t>PENDIENTE</t>
-        </is>
-      </c>
-      <c r="J51" s="105" t="inlineStr">
-        <is>
-          <t>SEGUIMIENTO</t>
-        </is>
-      </c>
-      <c r="K51" s="105" t="inlineStr">
-        <is>
-          <t>SEGUIMIENTO</t>
-        </is>
-      </c>
-      <c r="L51" s="51" t="inlineStr">
-        <is>
-          <t>Sin noticias.</t>
-        </is>
-      </c>
-    </row>
-    <row r="52" ht="18" customHeight="1">
-      <c r="A52" s="114" t="inlineStr">
-        <is>
-          <t>GONZALO CÓRDOBA</t>
-        </is>
-      </c>
-      <c r="B52" s="115" t="inlineStr">
-        <is>
-          <t>HOTELES</t>
-        </is>
-      </c>
-      <c r="C52" s="116" t="inlineStr">
-        <is>
-          <t>Jesús</t>
-        </is>
-      </c>
-      <c r="D52" s="116" t="inlineStr">
-        <is>
-          <t>Supervisión</t>
-        </is>
-      </c>
-      <c r="E52" s="116" t="inlineStr">
-        <is>
-          <t>Consultas puntuales</t>
-        </is>
-      </c>
-      <c r="F52" s="116" t="inlineStr">
-        <is>
-          <t>Continuo</t>
-        </is>
-      </c>
-      <c r="G52" s="116" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H52" s="116" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I52" s="116" t="inlineStr">
-        <is>
-          <t>PENDIENTE</t>
-        </is>
-      </c>
-      <c r="J52" s="117" t="inlineStr">
-        <is>
-          <t>ESTABLE</t>
-        </is>
-      </c>
-      <c r="K52" s="117" t="inlineStr">
-        <is>
-          <t>ESTABLE</t>
-        </is>
-      </c>
-      <c r="L52" s="116" t="inlineStr">
-        <is>
-          <t>Solo consultas puntuales.</t>
-        </is>
-      </c>
-    </row>
-    <row r="53" ht="18" customHeight="1">
-      <c r="A53" s="114" t="inlineStr">
-        <is>
-          <t>AYALA OFICINAS</t>
-        </is>
-      </c>
-      <c r="B53" s="115" t="inlineStr">
-        <is>
-          <t>HOTELES</t>
-        </is>
-      </c>
-      <c r="C53" s="116" t="inlineStr">
-        <is>
-          <t>Ale/Jesús</t>
-        </is>
-      </c>
-      <c r="D53" s="116" t="inlineStr">
-        <is>
-          <t>Supervisión</t>
-        </is>
-      </c>
-      <c r="E53" s="116" t="inlineStr">
-        <is>
-          <t>Montaje diciembre</t>
-        </is>
-      </c>
-      <c r="F53" s="116" t="inlineStr">
-        <is>
-          <t>Dic 2026</t>
-        </is>
-      </c>
-      <c r="G53" s="116" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H53" s="116" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I53" s="116" t="inlineStr">
-        <is>
-          <t>PROY DECO</t>
-        </is>
-      </c>
-      <c r="J53" s="117" t="inlineStr">
-        <is>
-          <t>ESTABLE</t>
-        </is>
-      </c>
-      <c r="K53" s="117" t="inlineStr">
-        <is>
-          <t>ESTABLE</t>
-        </is>
-      </c>
-      <c r="L53" s="116" t="inlineStr">
-        <is>
-          <t>Presu deco entregado. Montaje diciembre.</t>
-        </is>
-      </c>
-    </row>
-    <row r="54" ht="18" customHeight="1">
-      <c r="A54" s="114" t="inlineStr">
-        <is>
-          <t>KANDA SÁNCHEZ PACHECO</t>
-        </is>
-      </c>
-      <c r="B54" s="115" t="inlineStr">
-        <is>
-          <t>HOTELES</t>
-        </is>
-      </c>
-      <c r="C54" s="116" t="inlineStr">
-        <is>
-          <t>Jesús/Marta</t>
-        </is>
-      </c>
-      <c r="D54" s="116" t="inlineStr">
-        <is>
-          <t>Supervisión</t>
-        </is>
-      </c>
-      <c r="E54" s="116" t="inlineStr">
-        <is>
-          <t>Sin feedback</t>
-        </is>
-      </c>
-      <c r="F54" s="116" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G54" s="116" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H54" s="116" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I54" s="116" t="inlineStr">
-        <is>
-          <t>PENDIENTE</t>
-        </is>
-      </c>
-      <c r="J54" s="117" t="inlineStr">
-        <is>
-          <t>ESTABLE</t>
-        </is>
-      </c>
-      <c r="K54" s="117" t="inlineStr">
-        <is>
-          <t>ESTABLE</t>
-        </is>
-      </c>
-      <c r="L54" s="116" t="inlineStr">
-        <is>
-          <t>Sin noticias.</t>
-        </is>
-      </c>
-    </row>
-    <row r="55" ht="18" customHeight="1">
-      <c r="A55" s="114" t="inlineStr">
-        <is>
-          <t>KANDA CATALINA SUÁREZ</t>
-        </is>
-      </c>
-      <c r="B55" s="115" t="inlineStr">
-        <is>
-          <t>HOTELES</t>
-        </is>
-      </c>
-      <c r="C55" s="116" t="inlineStr">
-        <is>
-          <t>Jesús/Marta</t>
-        </is>
-      </c>
-      <c r="D55" s="116" t="inlineStr">
-        <is>
-          <t>Supervisión</t>
-        </is>
-      </c>
-      <c r="E55" s="116" t="inlineStr">
-        <is>
-          <t>Sin feedback</t>
-        </is>
-      </c>
-      <c r="F55" s="116" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G55" s="116" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H55" s="116" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I55" s="116" t="inlineStr">
-        <is>
-          <t>PENDIENTE</t>
-        </is>
-      </c>
-      <c r="J55" s="117" t="inlineStr">
-        <is>
-          <t>ESTABLE</t>
-        </is>
-      </c>
-      <c r="K55" s="117" t="inlineStr">
-        <is>
-          <t>ESTABLE</t>
-        </is>
-      </c>
-      <c r="L55" s="116" t="inlineStr">
-        <is>
-          <t>Sin noticias.</t>
-        </is>
-      </c>
-    </row>
-    <row r="56" ht="16" customHeight="1">
-      <c r="A56" s="118" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  ▸  LATENTES / EN ESPERA</t>
-        </is>
-      </c>
-    </row>
-    <row r="57" ht="18" customHeight="1">
-      <c r="A57" s="119" t="inlineStr">
-        <is>
-          <t>ANA HONTANAR</t>
-        </is>
-      </c>
-      <c r="B57" s="120" t="inlineStr">
-        <is>
-          <t>VIVIENDA</t>
-        </is>
-      </c>
-      <c r="C57" s="121" t="inlineStr">
-        <is>
-          <t>Paula</t>
-        </is>
-      </c>
-      <c r="D57" s="121" t="inlineStr">
-        <is>
-          <t>En espera</t>
-        </is>
-      </c>
-      <c r="E57" s="121" t="inlineStr">
-        <is>
-          <t>Después de verano</t>
-        </is>
-      </c>
-      <c r="F57" s="121" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G57" s="121" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H57" s="121" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I57" s="121" t="inlineStr">
-        <is>
-          <t>PENDIENTE</t>
-        </is>
-      </c>
-      <c r="J57" s="122" t="inlineStr">
-        <is>
-          <t>PARADO</t>
-        </is>
-      </c>
-      <c r="K57" s="122" t="inlineStr">
-        <is>
-          <t>PARADO</t>
-        </is>
-      </c>
-      <c r="L57" s="121" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="58" ht="18" customHeight="1">
-      <c r="A58" s="119" t="inlineStr">
-        <is>
-          <t>JAIME PESQUERA</t>
-        </is>
-      </c>
-      <c r="B58" s="120" t="inlineStr">
-        <is>
-          <t>VIVIENDA</t>
-        </is>
-      </c>
-      <c r="C58" s="121" t="inlineStr">
-        <is>
-          <t>Paula</t>
-        </is>
-      </c>
-      <c r="D58" s="121" t="inlineStr">
-        <is>
-          <t>En espera</t>
-        </is>
-      </c>
-      <c r="E58" s="121" t="inlineStr">
-        <is>
-          <t>Después de verano</t>
-        </is>
-      </c>
-      <c r="F58" s="121" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G58" s="121" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H58" s="121" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I58" s="121" t="inlineStr">
-        <is>
-          <t>PENDIENTE</t>
-        </is>
-      </c>
-      <c r="J58" s="122" t="inlineStr">
-        <is>
-          <t>PARADO</t>
-        </is>
-      </c>
-      <c r="K58" s="122" t="inlineStr">
-        <is>
-          <t>PARADO</t>
-        </is>
-      </c>
-      <c r="L58" s="121" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="59" ht="18" customHeight="1">
-      <c r="A59" s="119" t="inlineStr">
-        <is>
-          <t>HABITACIÓN ABI</t>
-        </is>
-      </c>
-      <c r="B59" s="120" t="inlineStr">
-        <is>
-          <t>VIVIENDA</t>
-        </is>
-      </c>
-      <c r="C59" s="121" t="inlineStr">
-        <is>
-          <t>Andrea</t>
-        </is>
-      </c>
-      <c r="D59" s="121" t="inlineStr">
-        <is>
-          <t>En espera</t>
-        </is>
-      </c>
-      <c r="E59" s="121" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F59" s="121" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G59" s="121" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H59" s="121" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I59" s="121" t="inlineStr">
-        <is>
-          <t>PENDIENTE</t>
-        </is>
-      </c>
-      <c r="J59" s="122" t="inlineStr">
-        <is>
-          <t>PARADO</t>
-        </is>
-      </c>
-      <c r="K59" s="122" t="inlineStr">
-        <is>
-          <t>PARADO</t>
-        </is>
-      </c>
-      <c r="L59" s="121" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="60" ht="18" customHeight="1">
-      <c r="A60" s="119" t="inlineStr">
-        <is>
-          <t>ANTIC COLONIAL</t>
-        </is>
-      </c>
-      <c r="B60" s="120" t="inlineStr">
-        <is>
-          <t>VIVIENDA</t>
-        </is>
-      </c>
-      <c r="C60" s="121" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D60" s="121" t="inlineStr">
-        <is>
-          <t>En espera</t>
-        </is>
-      </c>
-      <c r="E60" s="121" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F60" s="121" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G60" s="121" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H60" s="121" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I60" s="121" t="inlineStr">
-        <is>
-          <t>PENDIENTE</t>
-        </is>
-      </c>
-      <c r="J60" s="122" t="inlineStr">
-        <is>
-          <t>PARADO</t>
-        </is>
-      </c>
-      <c r="K60" s="122" t="inlineStr">
-        <is>
-          <t>PARADO</t>
-        </is>
-      </c>
-      <c r="L60" s="121" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="61" ht="18" customHeight="1">
-      <c r="A61" s="119" t="inlineStr">
-        <is>
-          <t>MONTALBÁN</t>
-        </is>
-      </c>
-      <c r="B61" s="120" t="inlineStr">
-        <is>
-          <t>VIVIENDA</t>
-        </is>
-      </c>
-      <c r="C61" s="121" t="inlineStr">
-        <is>
-          <t>Olatz</t>
-        </is>
-      </c>
-      <c r="D61" s="121" t="inlineStr">
-        <is>
-          <t>En espera</t>
-        </is>
-      </c>
-      <c r="E61" s="121" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F61" s="121" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G61" s="121" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H61" s="121" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I61" s="121" t="inlineStr">
-        <is>
-          <t>PENDIENTE</t>
-        </is>
-      </c>
-      <c r="J61" s="122" t="inlineStr">
-        <is>
-          <t>PARADO</t>
-        </is>
-      </c>
-      <c r="K61" s="122" t="inlineStr">
-        <is>
-          <t>PARADO</t>
-        </is>
-      </c>
-      <c r="L61" s="121" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="62" ht="18" customHeight="1">
-      <c r="A62" s="123" t="inlineStr">
-        <is>
-          <t>SANTANDER REST</t>
-        </is>
-      </c>
-      <c r="B62" s="124" t="inlineStr">
-        <is>
-          <t>RESTAURANTES</t>
-        </is>
-      </c>
-      <c r="C62" s="121" t="inlineStr">
-        <is>
-          <t>Admón.</t>
-        </is>
-      </c>
-      <c r="D62" s="121" t="inlineStr">
-        <is>
-          <t>Gestión cobro</t>
-        </is>
-      </c>
-      <c r="E62" s="121" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F62" s="121" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G62" s="121" t="inlineStr">
-        <is>
-          <t>Disputa judicial</t>
-        </is>
-      </c>
-      <c r="H62" s="121" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I62" s="121" t="inlineStr">
-        <is>
-          <t>PENDIENTE</t>
-        </is>
-      </c>
-      <c r="J62" s="122" t="inlineStr">
-        <is>
-          <t>PARADO</t>
-        </is>
-      </c>
-      <c r="K62" s="122" t="inlineStr">
-        <is>
-          <t>PARADO</t>
-        </is>
-      </c>
-      <c r="L62" s="121" t="inlineStr">
-        <is>
-          <t>Gestión interna cobro.</t>
-        </is>
-      </c>
-    </row>
-    <row r="63" ht="18" customHeight="1">
-      <c r="A63" s="123" t="inlineStr">
-        <is>
-          <t>JOANN DOMINICANA</t>
-        </is>
-      </c>
-      <c r="B63" s="124" t="inlineStr">
-        <is>
-          <t>RESTAURANTES</t>
-        </is>
-      </c>
-      <c r="C63" s="121" t="inlineStr">
-        <is>
-          <t>Sofía</t>
-        </is>
-      </c>
-      <c r="D63" s="121" t="inlineStr">
-        <is>
-          <t>En espera</t>
-        </is>
-      </c>
-      <c r="E63" s="121" t="inlineStr">
-        <is>
-          <t>Pendiente entrar</t>
-        </is>
-      </c>
-      <c r="F63" s="121" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G63" s="121" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H63" s="121" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I63" s="121" t="inlineStr">
-        <is>
-          <t>PENDIENTE</t>
-        </is>
-      </c>
-      <c r="J63" s="122" t="inlineStr">
-        <is>
-          <t>PARADO</t>
-        </is>
-      </c>
-      <c r="K63" s="122" t="inlineStr">
-        <is>
-          <t>PARADO</t>
-        </is>
-      </c>
-      <c r="L63" s="121" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="64" ht="18" customHeight="1">
-      <c r="A64" s="123" t="inlineStr">
-        <is>
-          <t>SOPHIE</t>
-        </is>
-      </c>
-      <c r="B64" s="124" t="inlineStr">
-        <is>
-          <t>RESTAURANTES</t>
-        </is>
-      </c>
-      <c r="C64" s="121" t="inlineStr">
-        <is>
-          <t>Sofía</t>
-        </is>
-      </c>
-      <c r="D64" s="121" t="inlineStr">
-        <is>
-          <t>En espera</t>
-        </is>
-      </c>
-      <c r="E64" s="121" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F64" s="121" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G64" s="121" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H64" s="121" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I64" s="121" t="inlineStr">
-        <is>
-          <t>PENDIENTE</t>
-        </is>
-      </c>
-      <c r="J64" s="122" t="inlineStr">
-        <is>
-          <t>PARADO</t>
-        </is>
-      </c>
-      <c r="K64" s="122" t="inlineStr">
-        <is>
-          <t>PARADO</t>
-        </is>
-      </c>
-      <c r="L64" s="121" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="65" ht="18" customHeight="1">
-      <c r="A65" s="125" t="inlineStr">
-        <is>
-          <t>PANTANO RURAL</t>
-        </is>
-      </c>
-      <c r="B65" s="126" t="inlineStr">
-        <is>
-          <t>HOTELES</t>
-        </is>
-      </c>
-      <c r="C65" s="121" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D65" s="121" t="inlineStr">
-        <is>
-          <t>En espera</t>
-        </is>
-      </c>
-      <c r="E65" s="121" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F65" s="121" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G65" s="121" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H65" s="121" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I65" s="121" t="inlineStr">
-        <is>
-          <t>PENDIENTE</t>
-        </is>
-      </c>
-      <c r="J65" s="122" t="inlineStr">
-        <is>
-          <t>PARADO</t>
-        </is>
-      </c>
-      <c r="K65" s="122" t="inlineStr">
-        <is>
-          <t>PARADO</t>
-        </is>
-      </c>
-      <c r="L65" s="121" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="66" ht="18" customHeight="1">
-      <c r="A66" s="125" t="inlineStr">
-        <is>
-          <t>4 MASOS</t>
-        </is>
-      </c>
-      <c r="B66" s="126" t="inlineStr">
-        <is>
-          <t>HOTELES</t>
-        </is>
-      </c>
-      <c r="C66" s="121" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D66" s="121" t="inlineStr">
-        <is>
-          <t>En espera</t>
-        </is>
-      </c>
-      <c r="E66" s="121" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F66" s="121" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G66" s="121" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H66" s="121" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I66" s="121" t="inlineStr">
-        <is>
-          <t>PENDIENTE</t>
-        </is>
-      </c>
-      <c r="J66" s="122" t="inlineStr">
-        <is>
-          <t>PARADO</t>
-        </is>
-      </c>
-      <c r="K66" s="122" t="inlineStr">
-        <is>
-          <t>PARADO</t>
-        </is>
-      </c>
-      <c r="L66" s="121" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="67" ht="18" customHeight="1">
-      <c r="A67" s="125" t="inlineStr">
-        <is>
-          <t>BLESS</t>
-        </is>
-      </c>
-      <c r="B67" s="126" t="inlineStr">
-        <is>
-          <t>HOTELES</t>
-        </is>
-      </c>
-      <c r="C67" s="121" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D67" s="121" t="inlineStr">
-        <is>
-          <t>En espera</t>
-        </is>
-      </c>
-      <c r="E67" s="121" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F67" s="121" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G67" s="121" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H67" s="121" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I67" s="121" t="inlineStr">
-        <is>
-          <t>PENDIENTE</t>
-        </is>
-      </c>
-      <c r="J67" s="122" t="inlineStr">
-        <is>
-          <t>PARADO</t>
-        </is>
-      </c>
-      <c r="K67" s="122" t="inlineStr">
-        <is>
-          <t>PARADO</t>
-        </is>
-      </c>
-      <c r="L67" s="121" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="69">
-      <c r="A69" s="127" t="inlineStr">
-        <is>
-          <t>Actualizado: 1 septiembre 2026  ·  51 proyectos activos  ·  11 latentes</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="4">
-    <mergeCell ref="A56:L56"/>
-    <mergeCell ref="A69:L69"/>
-    <mergeCell ref="A1:L1"/>
-    <mergeCell ref="A4:L4"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
   <dimension ref="A1:C26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -5404,7 +1237,7 @@
     <row r="26">
       <c r="A26" s="35" t="inlineStr">
         <is>
-          <t>Actualizado: 01/09/2026</t>
+          <t>Actualizado: 07/09/2026  ·  Sara de vacaciones 3-14 sep</t>
         </is>
       </c>
     </row>
@@ -5416,7 +1249,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -5454,20 +1287,15 @@
     <row r="2" ht="14" customHeight="1">
       <c r="G2" s="37" t="inlineStr">
         <is>
-          <t>SEP</t>
-        </is>
-      </c>
-      <c r="H2" s="37" t="inlineStr">
-        <is>
           <t>OCT</t>
         </is>
       </c>
-      <c r="L2" s="37" t="inlineStr">
+      <c r="K2" s="37" t="inlineStr">
         <is>
           <t>NOV</t>
         </is>
       </c>
-      <c r="P2" s="37" t="inlineStr">
+      <c r="O2" s="37" t="inlineStr">
         <is>
           <t>NOV</t>
         </is>
@@ -5506,57 +1334,57 @@
       </c>
       <c r="G3" s="39" t="inlineStr">
         <is>
-          <t>1 SEP</t>
+          <t>7 SEP</t>
         </is>
       </c>
       <c r="H3" s="39" t="inlineStr">
         <is>
-          <t>8 SEP</t>
+          <t>14 SEP</t>
         </is>
       </c>
       <c r="I3" s="39" t="inlineStr">
         <is>
-          <t>15 SEP</t>
+          <t>21 SEP</t>
         </is>
       </c>
       <c r="J3" s="39" t="inlineStr">
         <is>
-          <t>22 SEP</t>
+          <t>28 SEP</t>
         </is>
       </c>
       <c r="K3" s="39" t="inlineStr">
         <is>
-          <t>29 SEP</t>
+          <t>5 OCT</t>
         </is>
       </c>
       <c r="L3" s="39" t="inlineStr">
         <is>
-          <t>6 OCT</t>
+          <t>12 OCT</t>
         </is>
       </c>
       <c r="M3" s="39" t="inlineStr">
         <is>
-          <t>13 OCT</t>
+          <t>19 OCT</t>
         </is>
       </c>
       <c r="N3" s="39" t="inlineStr">
         <is>
-          <t>20 OCT</t>
+          <t>26 OCT</t>
         </is>
       </c>
       <c r="O3" s="39" t="inlineStr">
         <is>
-          <t>27 OCT</t>
+          <t>2 NOV</t>
         </is>
       </c>
       <c r="P3" s="39" t="inlineStr">
         <is>
-          <t>3 NOV</t>
+          <t>9 NOV</t>
         </is>
       </c>
       <c r="Q3" s="39" t="inlineStr">
         <is>
-          <t>10 NOV</t>
+          <t>16 NOV</t>
         </is>
       </c>
     </row>
@@ -6429,22 +2257,6 @@
           <t xml:space="preserve">  LATENTES / PAUSADOS</t>
         </is>
       </c>
-      <c r="B17" s="128" t="n"/>
-      <c r="C17" s="128" t="n"/>
-      <c r="D17" s="128" t="n"/>
-      <c r="E17" s="128" t="n"/>
-      <c r="F17" s="128" t="n"/>
-      <c r="G17" s="128" t="n"/>
-      <c r="H17" s="128" t="n"/>
-      <c r="I17" s="128" t="n"/>
-      <c r="J17" s="128" t="n"/>
-      <c r="K17" s="128" t="n"/>
-      <c r="L17" s="128" t="n"/>
-      <c r="M17" s="128" t="n"/>
-      <c r="N17" s="128" t="n"/>
-      <c r="O17" s="128" t="n"/>
-      <c r="P17" s="128" t="n"/>
-      <c r="Q17" s="128" t="n"/>
     </row>
     <row r="18" ht="20" customHeight="1">
       <c r="A18" s="69" t="inlineStr"/>
@@ -6558,16 +2370,16 @@
   </sheetData>
   <mergeCells count="5">
     <mergeCell ref="A17:Q17"/>
-    <mergeCell ref="H2:K2"/>
-    <mergeCell ref="P2:Q2"/>
-    <mergeCell ref="L2:O2"/>
+    <mergeCell ref="G2:J2"/>
+    <mergeCell ref="K2:N2"/>
+    <mergeCell ref="O2:Q2"/>
     <mergeCell ref="A1:Q1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -6605,20 +2417,15 @@
     <row r="2" ht="14" customHeight="1">
       <c r="G2" s="37" t="inlineStr">
         <is>
-          <t>SEP</t>
-        </is>
-      </c>
-      <c r="H2" s="37" t="inlineStr">
-        <is>
           <t>OCT</t>
         </is>
       </c>
-      <c r="L2" s="37" t="inlineStr">
+      <c r="K2" s="37" t="inlineStr">
         <is>
           <t>NOV</t>
         </is>
       </c>
-      <c r="P2" s="37" t="inlineStr">
+      <c r="O2" s="37" t="inlineStr">
         <is>
           <t>NOV</t>
         </is>
@@ -6657,57 +2464,57 @@
       </c>
       <c r="G3" s="77" t="inlineStr">
         <is>
-          <t>1 SEP</t>
+          <t>7 SEP</t>
         </is>
       </c>
       <c r="H3" s="77" t="inlineStr">
         <is>
-          <t>8 SEP</t>
+          <t>14 SEP</t>
         </is>
       </c>
       <c r="I3" s="77" t="inlineStr">
         <is>
-          <t>15 SEP</t>
+          <t>21 SEP</t>
         </is>
       </c>
       <c r="J3" s="77" t="inlineStr">
         <is>
-          <t>22 SEP</t>
+          <t>28 SEP</t>
         </is>
       </c>
       <c r="K3" s="77" t="inlineStr">
         <is>
-          <t>29 SEP</t>
+          <t>5 OCT</t>
         </is>
       </c>
       <c r="L3" s="77" t="inlineStr">
         <is>
-          <t>6 OCT</t>
+          <t>12 OCT</t>
         </is>
       </c>
       <c r="M3" s="77" t="inlineStr">
         <is>
-          <t>13 OCT</t>
+          <t>19 OCT</t>
         </is>
       </c>
       <c r="N3" s="77" t="inlineStr">
         <is>
-          <t>20 OCT</t>
+          <t>26 OCT</t>
         </is>
       </c>
       <c r="O3" s="77" t="inlineStr">
         <is>
-          <t>27 OCT</t>
+          <t>2 NOV</t>
         </is>
       </c>
       <c r="P3" s="77" t="inlineStr">
         <is>
-          <t>3 NOV</t>
+          <t>9 NOV</t>
         </is>
       </c>
       <c r="Q3" s="77" t="inlineStr">
         <is>
-          <t>10 NOV</t>
+          <t>16 NOV</t>
         </is>
       </c>
     </row>
@@ -8413,22 +4220,6 @@
           <t xml:space="preserve">  LATENTES / PAUSADOS</t>
         </is>
       </c>
-      <c r="B28" s="129" t="n"/>
-      <c r="C28" s="129" t="n"/>
-      <c r="D28" s="129" t="n"/>
-      <c r="E28" s="129" t="n"/>
-      <c r="F28" s="129" t="n"/>
-      <c r="G28" s="129" t="n"/>
-      <c r="H28" s="129" t="n"/>
-      <c r="I28" s="129" t="n"/>
-      <c r="J28" s="129" t="n"/>
-      <c r="K28" s="129" t="n"/>
-      <c r="L28" s="129" t="n"/>
-      <c r="M28" s="129" t="n"/>
-      <c r="N28" s="129" t="n"/>
-      <c r="O28" s="129" t="n"/>
-      <c r="P28" s="129" t="n"/>
-      <c r="Q28" s="129" t="n"/>
     </row>
     <row r="29" ht="20" customHeight="1">
       <c r="A29" s="69" t="inlineStr">
@@ -8615,17 +4406,17 @@
     </row>
   </sheetData>
   <mergeCells count="5">
-    <mergeCell ref="H2:K2"/>
-    <mergeCell ref="P2:Q2"/>
-    <mergeCell ref="L2:O2"/>
+    <mergeCell ref="G2:J2"/>
     <mergeCell ref="A28:Q28"/>
+    <mergeCell ref="K2:N2"/>
+    <mergeCell ref="O2:Q2"/>
     <mergeCell ref="A1:Q1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -8663,20 +4454,15 @@
     <row r="2" ht="14" customHeight="1">
       <c r="G2" s="37" t="inlineStr">
         <is>
-          <t>SEP</t>
-        </is>
-      </c>
-      <c r="H2" s="37" t="inlineStr">
-        <is>
           <t>OCT</t>
         </is>
       </c>
-      <c r="L2" s="37" t="inlineStr">
+      <c r="K2" s="37" t="inlineStr">
         <is>
           <t>NOV</t>
         </is>
       </c>
-      <c r="P2" s="37" t="inlineStr">
+      <c r="O2" s="37" t="inlineStr">
         <is>
           <t>NOV</t>
         </is>
@@ -8715,57 +4501,57 @@
       </c>
       <c r="G3" s="90" t="inlineStr">
         <is>
-          <t>1 SEP</t>
+          <t>7 SEP</t>
         </is>
       </c>
       <c r="H3" s="90" t="inlineStr">
         <is>
-          <t>8 SEP</t>
+          <t>14 SEP</t>
         </is>
       </c>
       <c r="I3" s="90" t="inlineStr">
         <is>
-          <t>15 SEP</t>
+          <t>21 SEP</t>
         </is>
       </c>
       <c r="J3" s="90" t="inlineStr">
         <is>
-          <t>22 SEP</t>
+          <t>28 SEP</t>
         </is>
       </c>
       <c r="K3" s="90" t="inlineStr">
         <is>
-          <t>29 SEP</t>
+          <t>5 OCT</t>
         </is>
       </c>
       <c r="L3" s="90" t="inlineStr">
         <is>
-          <t>6 OCT</t>
+          <t>12 OCT</t>
         </is>
       </c>
       <c r="M3" s="90" t="inlineStr">
         <is>
-          <t>13 OCT</t>
+          <t>19 OCT</t>
         </is>
       </c>
       <c r="N3" s="90" t="inlineStr">
         <is>
-          <t>20 OCT</t>
+          <t>26 OCT</t>
         </is>
       </c>
       <c r="O3" s="90" t="inlineStr">
         <is>
-          <t>27 OCT</t>
+          <t>2 NOV</t>
         </is>
       </c>
       <c r="P3" s="90" t="inlineStr">
         <is>
-          <t>3 NOV</t>
+          <t>9 NOV</t>
         </is>
       </c>
       <c r="Q3" s="90" t="inlineStr">
         <is>
-          <t>10 NOV</t>
+          <t>16 NOV</t>
         </is>
       </c>
     </row>
@@ -9555,22 +5341,6 @@
           <t xml:space="preserve">  SUPERVISIÓN / SEGUIMIENTO PUNTUAL</t>
         </is>
       </c>
-      <c r="B16" s="130" t="n"/>
-      <c r="C16" s="130" t="n"/>
-      <c r="D16" s="130" t="n"/>
-      <c r="E16" s="130" t="n"/>
-      <c r="F16" s="130" t="n"/>
-      <c r="G16" s="130" t="n"/>
-      <c r="H16" s="130" t="n"/>
-      <c r="I16" s="130" t="n"/>
-      <c r="J16" s="130" t="n"/>
-      <c r="K16" s="130" t="n"/>
-      <c r="L16" s="130" t="n"/>
-      <c r="M16" s="130" t="n"/>
-      <c r="N16" s="130" t="n"/>
-      <c r="O16" s="130" t="n"/>
-      <c r="P16" s="130" t="n"/>
-      <c r="Q16" s="130" t="n"/>
     </row>
     <row r="17" ht="20" customHeight="1">
       <c r="A17" s="69" t="inlineStr">
@@ -9781,22 +5551,6 @@
           <t xml:space="preserve">  LATENTES / PAUSADOS</t>
         </is>
       </c>
-      <c r="B22" s="130" t="n"/>
-      <c r="C22" s="130" t="n"/>
-      <c r="D22" s="130" t="n"/>
-      <c r="E22" s="130" t="n"/>
-      <c r="F22" s="130" t="n"/>
-      <c r="G22" s="130" t="n"/>
-      <c r="H22" s="130" t="n"/>
-      <c r="I22" s="130" t="n"/>
-      <c r="J22" s="130" t="n"/>
-      <c r="K22" s="130" t="n"/>
-      <c r="L22" s="130" t="n"/>
-      <c r="M22" s="130" t="n"/>
-      <c r="N22" s="130" t="n"/>
-      <c r="O22" s="130" t="n"/>
-      <c r="P22" s="130" t="n"/>
-      <c r="Q22" s="130" t="n"/>
     </row>
     <row r="23" ht="20" customHeight="1">
       <c r="A23" s="69" t="inlineStr"/>
@@ -9910,10 +5664,10 @@
   </sheetData>
   <mergeCells count="6">
     <mergeCell ref="A22:Q22"/>
-    <mergeCell ref="H2:K2"/>
     <mergeCell ref="A16:Q16"/>
-    <mergeCell ref="L2:O2"/>
-    <mergeCell ref="P2:Q2"/>
+    <mergeCell ref="G2:J2"/>
+    <mergeCell ref="K2:N2"/>
+    <mergeCell ref="O2:Q2"/>
     <mergeCell ref="A1:Q1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
sync: ausencias Bizneo 2026-10-29 12:29 UTC
</commit_message>
<xml_diff>
--- a/PM_ESTUDIO_MASTER_COMPLETO.xlsx
+++ b/PM_ESTUDIO_MASTER_COMPLETO.xlsx
@@ -25,10 +25,10 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="4">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
-    <numFmt numFmtId="165" formatCode="DD/MM/YYYY"/>
-    <numFmt numFmtId="166" formatCode="yyyy-mm-dd h:mm:ss"/>
-    <numFmt numFmtId="167" formatCode="DD/MM/YYYY HH:MM"/>
+    <numFmt numFmtId="164" formatCode="DD/MM/YYYY"/>
+    <numFmt numFmtId="165" formatCode="DD/MM/YYYY HH:MM"/>
+    <numFmt numFmtId="166" formatCode="yyyy-mm-dd"/>
+    <numFmt numFmtId="167" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
   <fonts count="19">
     <font>
@@ -259,7 +259,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="52">
+  <cellXfs count="56">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -399,19 +399,31 @@
     <xf numFmtId="0" fontId="17" fillId="16" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="17" fillId="16" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="17" fillId="16" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="167" fontId="17" fillId="16" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="17" fillId="16" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="164" fontId="18" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="165" fontId="18" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="167" fontId="18" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="17" fillId="16" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="17" fillId="16" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="18" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="18" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -9138,7 +9150,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q114"/>
+  <dimension ref="A1:Q115"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -9268,10 +9280,10 @@
           <t>Vacaciones🏖️</t>
         </is>
       </c>
-      <c r="E2" s="47" t="n">
+      <c r="E2" s="52" t="n">
         <v>46027</v>
       </c>
-      <c r="F2" s="47" t="n">
+      <c r="F2" s="52" t="n">
         <v>46029</v>
       </c>
       <c r="G2" s="46" t="inlineStr"/>
@@ -9295,11 +9307,11 @@
           <t>SI</t>
         </is>
       </c>
-      <c r="N2" s="48" t="n">
-        <v>46323.51385416667</v>
+      <c r="N2" s="53" t="n">
+        <v>46324.52037037037</v>
       </c>
       <c r="O2" s="46" t="n"/>
-      <c r="P2" s="48" t="n">
+      <c r="P2" s="53" t="n">
         <v>46323.51385416667</v>
       </c>
       <c r="Q2" s="46" t="inlineStr"/>
@@ -9325,10 +9337,10 @@
           <t>Vacaciones🏖️</t>
         </is>
       </c>
-      <c r="E3" s="47" t="n">
+      <c r="E3" s="52" t="n">
         <v>46021</v>
       </c>
-      <c r="F3" s="47" t="n">
+      <c r="F3" s="52" t="n">
         <v>46027</v>
       </c>
       <c r="G3" s="46" t="inlineStr"/>
@@ -9352,11 +9364,11 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="N3" s="48" t="n">
-        <v>46323.51385416667</v>
+      <c r="N3" s="53" t="n">
+        <v>46324.52037037037</v>
       </c>
       <c r="O3" s="46" t="n"/>
-      <c r="P3" s="48" t="n">
+      <c r="P3" s="53" t="n">
         <v>46323.51385416667</v>
       </c>
       <c r="Q3" s="46" t="inlineStr"/>
@@ -9382,10 +9394,10 @@
           <t>Vacaciones🏖️</t>
         </is>
       </c>
-      <c r="E4" s="47" t="n">
+      <c r="E4" s="52" t="n">
         <v>46024</v>
       </c>
-      <c r="F4" s="47" t="n">
+      <c r="F4" s="52" t="n">
         <v>46024</v>
       </c>
       <c r="G4" s="46" t="inlineStr"/>
@@ -9409,11 +9421,11 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="N4" s="48" t="n">
-        <v>46323.51385416667</v>
+      <c r="N4" s="53" t="n">
+        <v>46324.52037037037</v>
       </c>
       <c r="O4" s="46" t="n"/>
-      <c r="P4" s="48" t="n">
+      <c r="P4" s="53" t="n">
         <v>46323.51385416667</v>
       </c>
       <c r="Q4" s="46" t="inlineStr"/>
@@ -9439,10 +9451,10 @@
           <t>Vacaciones🏖️</t>
         </is>
       </c>
-      <c r="E5" s="47" t="n">
+      <c r="E5" s="52" t="n">
         <v>46027</v>
       </c>
-      <c r="F5" s="47" t="n">
+      <c r="F5" s="52" t="n">
         <v>46027</v>
       </c>
       <c r="G5" s="46" t="inlineStr"/>
@@ -9466,11 +9478,11 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="N5" s="48" t="n">
-        <v>46323.51385416667</v>
+      <c r="N5" s="53" t="n">
+        <v>46324.52037037037</v>
       </c>
       <c r="O5" s="46" t="n"/>
-      <c r="P5" s="48" t="n">
+      <c r="P5" s="53" t="n">
         <v>46323.51385416667</v>
       </c>
       <c r="Q5" s="46" t="inlineStr"/>
@@ -9496,10 +9508,10 @@
           <t>Vacaciones🏖️</t>
         </is>
       </c>
-      <c r="E6" s="47" t="n">
+      <c r="E6" s="52" t="n">
         <v>46048</v>
       </c>
-      <c r="F6" s="47" t="n">
+      <c r="F6" s="52" t="n">
         <v>46048</v>
       </c>
       <c r="G6" s="46" t="inlineStr"/>
@@ -9523,11 +9535,11 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="N6" s="48" t="n">
-        <v>46323.51385416667</v>
+      <c r="N6" s="53" t="n">
+        <v>46324.52037037037</v>
       </c>
       <c r="O6" s="46" t="n"/>
-      <c r="P6" s="48" t="n">
+      <c r="P6" s="53" t="n">
         <v>46323.51385416667</v>
       </c>
       <c r="Q6" s="46" t="inlineStr"/>
@@ -9553,10 +9565,10 @@
           <t>Vacaciones🏖️</t>
         </is>
       </c>
-      <c r="E7" s="47" t="n">
+      <c r="E7" s="52" t="n">
         <v>46251</v>
       </c>
-      <c r="F7" s="47" t="n">
+      <c r="F7" s="52" t="n">
         <v>46254</v>
       </c>
       <c r="G7" s="46" t="inlineStr"/>
@@ -9580,11 +9592,11 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="N7" s="48" t="n">
-        <v>46323.51385416667</v>
+      <c r="N7" s="53" t="n">
+        <v>46324.52037037037</v>
       </c>
       <c r="O7" s="46" t="n"/>
-      <c r="P7" s="48" t="n">
+      <c r="P7" s="53" t="n">
         <v>46323.51385416667</v>
       </c>
       <c r="Q7" s="46" t="inlineStr"/>
@@ -9610,10 +9622,10 @@
           <t>Vacaciones🏖️</t>
         </is>
       </c>
-      <c r="E8" s="47" t="n">
+      <c r="E8" s="52" t="n">
         <v>46050</v>
       </c>
-      <c r="F8" s="47" t="n">
+      <c r="F8" s="52" t="n">
         <v>46050</v>
       </c>
       <c r="G8" s="46" t="inlineStr"/>
@@ -9637,11 +9649,11 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="N8" s="48" t="n">
-        <v>46323.51385416667</v>
+      <c r="N8" s="53" t="n">
+        <v>46324.52037037037</v>
       </c>
       <c r="O8" s="46" t="n"/>
-      <c r="P8" s="48" t="n">
+      <c r="P8" s="53" t="n">
         <v>46323.51385416667</v>
       </c>
       <c r="Q8" s="46" t="inlineStr"/>
@@ -9667,10 +9679,10 @@
           <t>Vacaciones🏖️</t>
         </is>
       </c>
-      <c r="E9" s="47" t="n">
+      <c r="E9" s="52" t="n">
         <v>46051</v>
       </c>
-      <c r="F9" s="47" t="n">
+      <c r="F9" s="52" t="n">
         <v>46051</v>
       </c>
       <c r="G9" s="46" t="inlineStr"/>
@@ -9694,11 +9706,11 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="N9" s="48" t="n">
-        <v>46323.51385416667</v>
+      <c r="N9" s="53" t="n">
+        <v>46324.52037037037</v>
       </c>
       <c r="O9" s="46" t="n"/>
-      <c r="P9" s="48" t="n">
+      <c r="P9" s="53" t="n">
         <v>46323.51385416667</v>
       </c>
       <c r="Q9" s="46" t="inlineStr"/>
@@ -9724,10 +9736,10 @@
           <t>Vacaciones🏖️</t>
         </is>
       </c>
-      <c r="E10" s="47" t="n">
+      <c r="E10" s="52" t="n">
         <v>46052</v>
       </c>
-      <c r="F10" s="47" t="n">
+      <c r="F10" s="52" t="n">
         <v>46052</v>
       </c>
       <c r="G10" s="46" t="inlineStr"/>
@@ -9751,11 +9763,11 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="N10" s="48" t="n">
-        <v>46323.51385416667</v>
+      <c r="N10" s="53" t="n">
+        <v>46324.52037037037</v>
       </c>
       <c r="O10" s="46" t="n"/>
-      <c r="P10" s="48" t="n">
+      <c r="P10" s="53" t="n">
         <v>46323.51385416667</v>
       </c>
       <c r="Q10" s="46" t="inlineStr"/>
@@ -9781,10 +9793,10 @@
           <t>Vacaciones🏖️</t>
         </is>
       </c>
-      <c r="E11" s="47" t="n">
+      <c r="E11" s="52" t="n">
         <v>46024</v>
       </c>
-      <c r="F11" s="47" t="n">
+      <c r="F11" s="52" t="n">
         <v>46024</v>
       </c>
       <c r="G11" s="46" t="inlineStr"/>
@@ -9808,11 +9820,11 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="N11" s="48" t="n">
-        <v>46323.51385416667</v>
+      <c r="N11" s="53" t="n">
+        <v>46324.52037037037</v>
       </c>
       <c r="O11" s="46" t="n"/>
-      <c r="P11" s="48" t="n">
+      <c r="P11" s="53" t="n">
         <v>46323.51385416667</v>
       </c>
       <c r="Q11" s="46" t="inlineStr"/>
@@ -9838,10 +9850,10 @@
           <t>Vacaciones🏖️</t>
         </is>
       </c>
-      <c r="E12" s="47" t="n">
+      <c r="E12" s="52" t="n">
         <v>46027</v>
       </c>
-      <c r="F12" s="47" t="n">
+      <c r="F12" s="52" t="n">
         <v>46027</v>
       </c>
       <c r="G12" s="46" t="inlineStr"/>
@@ -9865,11 +9877,11 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="N12" s="48" t="n">
-        <v>46323.51385416667</v>
+      <c r="N12" s="53" t="n">
+        <v>46324.52037037037</v>
       </c>
       <c r="O12" s="46" t="n"/>
-      <c r="P12" s="48" t="n">
+      <c r="P12" s="53" t="n">
         <v>46323.51385416667</v>
       </c>
       <c r="Q12" s="46" t="inlineStr"/>
@@ -9895,10 +9907,10 @@
           <t>Vacaciones🏖️</t>
         </is>
       </c>
-      <c r="E13" s="47" t="n">
+      <c r="E13" s="52" t="n">
         <v>46024</v>
       </c>
-      <c r="F13" s="47" t="n">
+      <c r="F13" s="52" t="n">
         <v>46024</v>
       </c>
       <c r="G13" s="46" t="inlineStr"/>
@@ -9922,11 +9934,11 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="N13" s="48" t="n">
-        <v>46323.51385416667</v>
+      <c r="N13" s="53" t="n">
+        <v>46324.52037037037</v>
       </c>
       <c r="O13" s="46" t="n"/>
-      <c r="P13" s="48" t="n">
+      <c r="P13" s="53" t="n">
         <v>46323.51385416667</v>
       </c>
       <c r="Q13" s="46" t="inlineStr"/>
@@ -9948,10 +9960,10 @@
         </is>
       </c>
       <c r="D14" s="49" t="inlineStr"/>
-      <c r="E14" s="50" t="n">
+      <c r="E14" s="54" t="n">
         <v>46014</v>
       </c>
-      <c r="F14" s="50" t="n">
+      <c r="F14" s="54" t="n">
         <v>46028</v>
       </c>
       <c r="G14" s="49" t="inlineStr"/>
@@ -9975,11 +9987,11 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="N14" s="51" t="n">
-        <v>46323.51385416667</v>
+      <c r="N14" s="55" t="n">
+        <v>46324.52037037037</v>
       </c>
       <c r="O14" s="49" t="n"/>
-      <c r="P14" s="51" t="n">
+      <c r="P14" s="55" t="n">
         <v>46323.51385416667</v>
       </c>
       <c r="Q14" s="49" t="inlineStr">
@@ -10009,10 +10021,10 @@
           <t>Vacaciones🏖️</t>
         </is>
       </c>
-      <c r="E15" s="47" t="n">
+      <c r="E15" s="52" t="n">
         <v>46029</v>
       </c>
-      <c r="F15" s="47" t="n">
+      <c r="F15" s="52" t="n">
         <v>46029</v>
       </c>
       <c r="G15" s="46" t="inlineStr"/>
@@ -10036,11 +10048,11 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="N15" s="48" t="n">
-        <v>46323.51385416667</v>
+      <c r="N15" s="53" t="n">
+        <v>46324.52037037037</v>
       </c>
       <c r="O15" s="46" t="n"/>
-      <c r="P15" s="48" t="n">
+      <c r="P15" s="53" t="n">
         <v>46323.51385416667</v>
       </c>
       <c r="Q15" s="46" t="inlineStr"/>
@@ -10066,10 +10078,10 @@
           <t>Vacaciones🏖️</t>
         </is>
       </c>
-      <c r="E16" s="47" t="n">
+      <c r="E16" s="52" t="n">
         <v>46027</v>
       </c>
-      <c r="F16" s="47" t="n">
+      <c r="F16" s="52" t="n">
         <v>46027</v>
       </c>
       <c r="G16" s="46" t="inlineStr"/>
@@ -10093,11 +10105,11 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="N16" s="48" t="n">
-        <v>46323.51385416667</v>
+      <c r="N16" s="53" t="n">
+        <v>46324.52037037037</v>
       </c>
       <c r="O16" s="46" t="n"/>
-      <c r="P16" s="48" t="n">
+      <c r="P16" s="53" t="n">
         <v>46323.51385416667</v>
       </c>
       <c r="Q16" s="46" t="inlineStr"/>
@@ -10123,10 +10135,10 @@
           <t>Vacaciones🏖️</t>
         </is>
       </c>
-      <c r="E17" s="47" t="n">
+      <c r="E17" s="52" t="n">
         <v>46024</v>
       </c>
-      <c r="F17" s="47" t="n">
+      <c r="F17" s="52" t="n">
         <v>46024</v>
       </c>
       <c r="G17" s="46" t="inlineStr"/>
@@ -10150,11 +10162,11 @@
           <t>SI</t>
         </is>
       </c>
-      <c r="N17" s="48" t="n">
-        <v>46323.51385416667</v>
+      <c r="N17" s="53" t="n">
+        <v>46324.52037037037</v>
       </c>
       <c r="O17" s="46" t="n"/>
-      <c r="P17" s="48" t="n">
+      <c r="P17" s="53" t="n">
         <v>46323.51385416667</v>
       </c>
       <c r="Q17" s="46" t="inlineStr"/>
@@ -10180,10 +10192,10 @@
           <t>Vacaciones🏖️</t>
         </is>
       </c>
-      <c r="E18" s="47" t="n">
+      <c r="E18" s="52" t="n">
         <v>46027</v>
       </c>
-      <c r="F18" s="47" t="n">
+      <c r="F18" s="52" t="n">
         <v>46027</v>
       </c>
       <c r="G18" s="46" t="inlineStr"/>
@@ -10207,11 +10219,11 @@
           <t>SI</t>
         </is>
       </c>
-      <c r="N18" s="48" t="n">
-        <v>46323.51385416667</v>
+      <c r="N18" s="53" t="n">
+        <v>46324.52037037037</v>
       </c>
       <c r="O18" s="46" t="n"/>
-      <c r="P18" s="48" t="n">
+      <c r="P18" s="53" t="n">
         <v>46323.51385416667</v>
       </c>
       <c r="Q18" s="46" t="inlineStr"/>
@@ -10237,10 +10249,10 @@
           <t>Vacaciones🏖️</t>
         </is>
       </c>
-      <c r="E19" s="47" t="n">
+      <c r="E19" s="52" t="n">
         <v>46027</v>
       </c>
-      <c r="F19" s="47" t="n">
+      <c r="F19" s="52" t="n">
         <v>46027</v>
       </c>
       <c r="G19" s="46" t="inlineStr"/>
@@ -10264,11 +10276,11 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="N19" s="48" t="n">
-        <v>46323.51385416667</v>
+      <c r="N19" s="53" t="n">
+        <v>46324.52037037037</v>
       </c>
       <c r="O19" s="46" t="n"/>
-      <c r="P19" s="48" t="n">
+      <c r="P19" s="53" t="n">
         <v>46323.51385416667</v>
       </c>
       <c r="Q19" s="46" t="inlineStr"/>
@@ -10294,10 +10306,10 @@
           <t>Vacaciones🏖️</t>
         </is>
       </c>
-      <c r="E20" s="47" t="n">
+      <c r="E20" s="52" t="n">
         <v>46024</v>
       </c>
-      <c r="F20" s="47" t="n">
+      <c r="F20" s="52" t="n">
         <v>46024</v>
       </c>
       <c r="G20" s="46" t="inlineStr"/>
@@ -10321,11 +10333,11 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="N20" s="48" t="n">
-        <v>46323.51385416667</v>
+      <c r="N20" s="53" t="n">
+        <v>46324.52037037037</v>
       </c>
       <c r="O20" s="46" t="n"/>
-      <c r="P20" s="48" t="n">
+      <c r="P20" s="53" t="n">
         <v>46323.51385416667</v>
       </c>
       <c r="Q20" s="46" t="inlineStr"/>
@@ -10351,10 +10363,10 @@
           <t>Vacaciones🏖️</t>
         </is>
       </c>
-      <c r="E21" s="47" t="n">
+      <c r="E21" s="52" t="n">
         <v>46037</v>
       </c>
-      <c r="F21" s="47" t="n">
+      <c r="F21" s="52" t="n">
         <v>46041</v>
       </c>
       <c r="G21" s="46" t="inlineStr"/>
@@ -10378,11 +10390,11 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="N21" s="48" t="n">
-        <v>46323.51385416667</v>
+      <c r="N21" s="53" t="n">
+        <v>46324.52037037037</v>
       </c>
       <c r="O21" s="46" t="n"/>
-      <c r="P21" s="48" t="n">
+      <c r="P21" s="53" t="n">
         <v>46323.51385416667</v>
       </c>
       <c r="Q21" s="46" t="inlineStr"/>
@@ -10408,10 +10420,10 @@
           <t>Vacaciones🏖️</t>
         </is>
       </c>
-      <c r="E22" s="47" t="n">
+      <c r="E22" s="52" t="n">
         <v>46069</v>
       </c>
-      <c r="F22" s="47" t="n">
+      <c r="F22" s="52" t="n">
         <v>46071</v>
       </c>
       <c r="G22" s="46" t="inlineStr"/>
@@ -10435,11 +10447,11 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="N22" s="48" t="n">
-        <v>46323.51385416667</v>
+      <c r="N22" s="53" t="n">
+        <v>46324.52037037037</v>
       </c>
       <c r="O22" s="46" t="n"/>
-      <c r="P22" s="48" t="n">
+      <c r="P22" s="53" t="n">
         <v>46323.51385416667</v>
       </c>
       <c r="Q22" s="46" t="inlineStr"/>
@@ -10465,10 +10477,10 @@
           <t>Vacaciones🏖️</t>
         </is>
       </c>
-      <c r="E23" s="47" t="n">
+      <c r="E23" s="52" t="n">
         <v>46027</v>
       </c>
-      <c r="F23" s="47" t="n">
+      <c r="F23" s="52" t="n">
         <v>46027</v>
       </c>
       <c r="G23" s="46" t="inlineStr"/>
@@ -10492,11 +10504,11 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="N23" s="48" t="n">
-        <v>46323.51385416667</v>
+      <c r="N23" s="53" t="n">
+        <v>46324.52037037037</v>
       </c>
       <c r="O23" s="46" t="n"/>
-      <c r="P23" s="48" t="n">
+      <c r="P23" s="53" t="n">
         <v>46323.51385416667</v>
       </c>
       <c r="Q23" s="46" t="inlineStr"/>
@@ -10522,10 +10534,10 @@
           <t>Vacaciones🏖️</t>
         </is>
       </c>
-      <c r="E24" s="47" t="n">
+      <c r="E24" s="52" t="n">
         <v>46024</v>
       </c>
-      <c r="F24" s="47" t="n">
+      <c r="F24" s="52" t="n">
         <v>46024</v>
       </c>
       <c r="G24" s="46" t="inlineStr"/>
@@ -10549,11 +10561,11 @@
           <t>SI</t>
         </is>
       </c>
-      <c r="N24" s="48" t="n">
-        <v>46323.51385416667</v>
+      <c r="N24" s="53" t="n">
+        <v>46324.52037037037</v>
       </c>
       <c r="O24" s="46" t="n"/>
-      <c r="P24" s="48" t="n">
+      <c r="P24" s="53" t="n">
         <v>46323.51385416667</v>
       </c>
       <c r="Q24" s="46" t="inlineStr"/>
@@ -10579,10 +10591,10 @@
           <t>Vacaciones🏖️</t>
         </is>
       </c>
-      <c r="E25" s="47" t="n">
+      <c r="E25" s="52" t="n">
         <v>46027</v>
       </c>
-      <c r="F25" s="47" t="n">
+      <c r="F25" s="52" t="n">
         <v>46027</v>
       </c>
       <c r="G25" s="46" t="inlineStr"/>
@@ -10606,11 +10618,11 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="N25" s="48" t="n">
-        <v>46323.51385416667</v>
+      <c r="N25" s="53" t="n">
+        <v>46324.52037037037</v>
       </c>
       <c r="O25" s="46" t="n"/>
-      <c r="P25" s="48" t="n">
+      <c r="P25" s="53" t="n">
         <v>46323.51385416667</v>
       </c>
       <c r="Q25" s="46" t="inlineStr"/>
@@ -10636,10 +10648,10 @@
           <t>Vacaciones🏖️</t>
         </is>
       </c>
-      <c r="E26" s="47" t="n">
+      <c r="E26" s="52" t="n">
         <v>46034</v>
       </c>
-      <c r="F26" s="47" t="n">
+      <c r="F26" s="52" t="n">
         <v>46035</v>
       </c>
       <c r="G26" s="46" t="inlineStr"/>
@@ -10663,11 +10675,11 @@
           <t>SI</t>
         </is>
       </c>
-      <c r="N26" s="48" t="n">
-        <v>46323.51385416667</v>
+      <c r="N26" s="53" t="n">
+        <v>46324.52037037037</v>
       </c>
       <c r="O26" s="46" t="n"/>
-      <c r="P26" s="48" t="n">
+      <c r="P26" s="53" t="n">
         <v>46323.51385416667</v>
       </c>
       <c r="Q26" s="46" t="inlineStr"/>
@@ -10693,10 +10705,10 @@
           <t>Vacaciones🏖️</t>
         </is>
       </c>
-      <c r="E27" s="47" t="n">
+      <c r="E27" s="52" t="n">
         <v>46066</v>
       </c>
-      <c r="F27" s="47" t="n">
+      <c r="F27" s="52" t="n">
         <v>46069</v>
       </c>
       <c r="G27" s="46" t="inlineStr"/>
@@ -10720,11 +10732,11 @@
           <t>SI</t>
         </is>
       </c>
-      <c r="N27" s="48" t="n">
-        <v>46323.51385416667</v>
+      <c r="N27" s="53" t="n">
+        <v>46324.52037037037</v>
       </c>
       <c r="O27" s="46" t="n"/>
-      <c r="P27" s="48" t="n">
+      <c r="P27" s="53" t="n">
         <v>46323.51385416667</v>
       </c>
       <c r="Q27" s="46" t="inlineStr"/>
@@ -10750,10 +10762,10 @@
           <t>Vacaciones🏖️</t>
         </is>
       </c>
-      <c r="E28" s="47" t="n">
+      <c r="E28" s="52" t="n">
         <v>46090</v>
       </c>
-      <c r="F28" s="47" t="n">
+      <c r="F28" s="52" t="n">
         <v>46090</v>
       </c>
       <c r="G28" s="46" t="inlineStr"/>
@@ -10777,11 +10789,11 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="N28" s="48" t="n">
-        <v>46323.51385416667</v>
+      <c r="N28" s="53" t="n">
+        <v>46324.52037037037</v>
       </c>
       <c r="O28" s="46" t="n"/>
-      <c r="P28" s="48" t="n">
+      <c r="P28" s="53" t="n">
         <v>46323.51385416667</v>
       </c>
       <c r="Q28" s="46" t="inlineStr"/>
@@ -10807,10 +10819,10 @@
           <t>Vacaciones🏖️</t>
         </is>
       </c>
-      <c r="E29" s="47" t="n">
+      <c r="E29" s="52" t="n">
         <v>46048</v>
       </c>
-      <c r="F29" s="47" t="n">
+      <c r="F29" s="52" t="n">
         <v>46049</v>
       </c>
       <c r="G29" s="46" t="inlineStr"/>
@@ -10834,11 +10846,11 @@
           <t>SI</t>
         </is>
       </c>
-      <c r="N29" s="48" t="n">
-        <v>46323.51385416667</v>
+      <c r="N29" s="53" t="n">
+        <v>46324.52037037037</v>
       </c>
       <c r="O29" s="46" t="n"/>
-      <c r="P29" s="48" t="n">
+      <c r="P29" s="53" t="n">
         <v>46323.51385416667</v>
       </c>
       <c r="Q29" s="46" t="inlineStr"/>
@@ -10864,10 +10876,10 @@
           <t>Vacaciones🏖️</t>
         </is>
       </c>
-      <c r="E30" s="47" t="n">
+      <c r="E30" s="52" t="n">
         <v>46041</v>
       </c>
-      <c r="F30" s="47" t="n">
+      <c r="F30" s="52" t="n">
         <v>46041</v>
       </c>
       <c r="G30" s="46" t="inlineStr"/>
@@ -10891,11 +10903,11 @@
           <t>SI</t>
         </is>
       </c>
-      <c r="N30" s="48" t="n">
-        <v>46323.51385416667</v>
+      <c r="N30" s="53" t="n">
+        <v>46324.52037037037</v>
       </c>
       <c r="O30" s="46" t="n"/>
-      <c r="P30" s="48" t="n">
+      <c r="P30" s="53" t="n">
         <v>46323.51385416667</v>
       </c>
       <c r="Q30" s="46" t="inlineStr"/>
@@ -10921,10 +10933,10 @@
           <t>Vacaciones🏖️</t>
         </is>
       </c>
-      <c r="E31" s="47" t="n">
+      <c r="E31" s="52" t="n">
         <v>46043</v>
       </c>
-      <c r="F31" s="47" t="n">
+      <c r="F31" s="52" t="n">
         <v>46044</v>
       </c>
       <c r="G31" s="46" t="inlineStr"/>
@@ -10948,11 +10960,11 @@
           <t>SI</t>
         </is>
       </c>
-      <c r="N31" s="48" t="n">
-        <v>46323.51385416667</v>
+      <c r="N31" s="53" t="n">
+        <v>46324.52037037037</v>
       </c>
       <c r="O31" s="46" t="n"/>
-      <c r="P31" s="48" t="n">
+      <c r="P31" s="53" t="n">
         <v>46323.51385416667</v>
       </c>
       <c r="Q31" s="46" t="inlineStr"/>
@@ -10978,10 +10990,10 @@
           <t>Ausencia</t>
         </is>
       </c>
-      <c r="E32" s="47" t="n">
+      <c r="E32" s="52" t="n">
         <v>46111</v>
       </c>
-      <c r="F32" s="47" t="n">
+      <c r="F32" s="52" t="n">
         <v>46111</v>
       </c>
       <c r="G32" s="46" t="inlineStr"/>
@@ -11005,11 +11017,11 @@
           <t>SI</t>
         </is>
       </c>
-      <c r="N32" s="48" t="n">
-        <v>46323.51385416667</v>
+      <c r="N32" s="53" t="n">
+        <v>46324.52037037037</v>
       </c>
       <c r="O32" s="46" t="n"/>
-      <c r="P32" s="48" t="n">
+      <c r="P32" s="53" t="n">
         <v>46323.51385416667</v>
       </c>
       <c r="Q32" s="46" t="inlineStr"/>
@@ -11035,10 +11047,10 @@
           <t>Vacaciones🏖️</t>
         </is>
       </c>
-      <c r="E33" s="47" t="n">
+      <c r="E33" s="52" t="n">
         <v>46112</v>
       </c>
-      <c r="F33" s="47" t="n">
+      <c r="F33" s="52" t="n">
         <v>46118</v>
       </c>
       <c r="G33" s="46" t="inlineStr"/>
@@ -11062,11 +11074,11 @@
           <t>SI</t>
         </is>
       </c>
-      <c r="N33" s="48" t="n">
-        <v>46323.51385416667</v>
+      <c r="N33" s="53" t="n">
+        <v>46324.52037037037</v>
       </c>
       <c r="O33" s="46" t="n"/>
-      <c r="P33" s="48" t="n">
+      <c r="P33" s="53" t="n">
         <v>46323.51385416667</v>
       </c>
       <c r="Q33" s="46" t="inlineStr"/>
@@ -11092,10 +11104,10 @@
           <t>Vacaciones🏖️</t>
         </is>
       </c>
-      <c r="E34" s="47" t="n">
+      <c r="E34" s="52" t="n">
         <v>46052</v>
       </c>
-      <c r="F34" s="47" t="n">
+      <c r="F34" s="52" t="n">
         <v>46052</v>
       </c>
       <c r="G34" s="46" t="inlineStr"/>
@@ -11119,11 +11131,11 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="N34" s="48" t="n">
-        <v>46323.51385416667</v>
+      <c r="N34" s="53" t="n">
+        <v>46324.52037037037</v>
       </c>
       <c r="O34" s="46" t="n"/>
-      <c r="P34" s="48" t="n">
+      <c r="P34" s="53" t="n">
         <v>46323.51385416667</v>
       </c>
       <c r="Q34" s="46" t="inlineStr"/>
@@ -11149,10 +11161,10 @@
           <t>Vacaciones🏖️</t>
         </is>
       </c>
-      <c r="E35" s="47" t="n">
+      <c r="E35" s="52" t="n">
         <v>46049</v>
       </c>
-      <c r="F35" s="47" t="n">
+      <c r="F35" s="52" t="n">
         <v>46049</v>
       </c>
       <c r="G35" s="46" t="inlineStr"/>
@@ -11176,11 +11188,11 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="N35" s="48" t="n">
-        <v>46323.51385416667</v>
+      <c r="N35" s="53" t="n">
+        <v>46324.52037037037</v>
       </c>
       <c r="O35" s="46" t="n"/>
-      <c r="P35" s="48" t="n">
+      <c r="P35" s="53" t="n">
         <v>46323.51385416667</v>
       </c>
       <c r="Q35" s="46" t="inlineStr"/>
@@ -11206,10 +11218,10 @@
           <t>Vacaciones🏖️</t>
         </is>
       </c>
-      <c r="E36" s="47" t="n">
+      <c r="E36" s="52" t="n">
         <v>46097</v>
       </c>
-      <c r="F36" s="47" t="n">
+      <c r="F36" s="52" t="n">
         <v>46097</v>
       </c>
       <c r="G36" s="46" t="inlineStr"/>
@@ -11233,11 +11245,11 @@
           <t>SI</t>
         </is>
       </c>
-      <c r="N36" s="48" t="n">
-        <v>46323.51385416667</v>
+      <c r="N36" s="53" t="n">
+        <v>46324.52037037037</v>
       </c>
       <c r="O36" s="46" t="n"/>
-      <c r="P36" s="48" t="n">
+      <c r="P36" s="53" t="n">
         <v>46323.51385416667</v>
       </c>
       <c r="Q36" s="46" t="inlineStr"/>
@@ -11263,10 +11275,10 @@
           <t>Vacaciones🏖️</t>
         </is>
       </c>
-      <c r="E37" s="47" t="n">
+      <c r="E37" s="52" t="n">
         <v>46080</v>
       </c>
-      <c r="F37" s="47" t="n">
+      <c r="F37" s="52" t="n">
         <v>46080</v>
       </c>
       <c r="G37" s="46" t="inlineStr"/>
@@ -11290,11 +11302,11 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="N37" s="48" t="n">
-        <v>46323.51385416667</v>
+      <c r="N37" s="53" t="n">
+        <v>46324.52037037037</v>
       </c>
       <c r="O37" s="46" t="n"/>
-      <c r="P37" s="48" t="n">
+      <c r="P37" s="53" t="n">
         <v>46323.51385416667</v>
       </c>
       <c r="Q37" s="46" t="inlineStr"/>
@@ -11320,10 +11332,10 @@
           <t>Vacaciones🏖️</t>
         </is>
       </c>
-      <c r="E38" s="47" t="n">
+      <c r="E38" s="52" t="n">
         <v>46065</v>
       </c>
-      <c r="F38" s="47" t="n">
+      <c r="F38" s="52" t="n">
         <v>46065</v>
       </c>
       <c r="G38" s="46" t="inlineStr"/>
@@ -11347,11 +11359,11 @@
           <t>SI</t>
         </is>
       </c>
-      <c r="N38" s="48" t="n">
-        <v>46323.51385416667</v>
+      <c r="N38" s="53" t="n">
+        <v>46324.52037037037</v>
       </c>
       <c r="O38" s="46" t="n"/>
-      <c r="P38" s="48" t="n">
+      <c r="P38" s="53" t="n">
         <v>46323.51385416667</v>
       </c>
       <c r="Q38" s="46" t="inlineStr"/>
@@ -11377,10 +11389,10 @@
           <t>Vacaciones🏖️</t>
         </is>
       </c>
-      <c r="E39" s="47" t="n">
+      <c r="E39" s="52" t="n">
         <v>46085</v>
       </c>
-      <c r="F39" s="47" t="n">
+      <c r="F39" s="52" t="n">
         <v>46087</v>
       </c>
       <c r="G39" s="46" t="inlineStr"/>
@@ -11404,11 +11416,11 @@
           <t>SI</t>
         </is>
       </c>
-      <c r="N39" s="48" t="n">
-        <v>46323.51385416667</v>
+      <c r="N39" s="53" t="n">
+        <v>46324.52037037037</v>
       </c>
       <c r="O39" s="46" t="n"/>
-      <c r="P39" s="48" t="n">
+      <c r="P39" s="53" t="n">
         <v>46323.51385416667</v>
       </c>
       <c r="Q39" s="46" t="inlineStr"/>
@@ -11434,10 +11446,10 @@
           <t>Vacaciones🏖️</t>
         </is>
       </c>
-      <c r="E40" s="47" t="n">
+      <c r="E40" s="52" t="n">
         <v>46072</v>
       </c>
-      <c r="F40" s="47" t="n">
+      <c r="F40" s="52" t="n">
         <v>46072</v>
       </c>
       <c r="G40" s="46" t="inlineStr"/>
@@ -11461,11 +11473,11 @@
           <t>SI</t>
         </is>
       </c>
-      <c r="N40" s="48" t="n">
-        <v>46323.51385416667</v>
+      <c r="N40" s="53" t="n">
+        <v>46324.52037037037</v>
       </c>
       <c r="O40" s="46" t="n"/>
-      <c r="P40" s="48" t="n">
+      <c r="P40" s="53" t="n">
         <v>46323.51385416667</v>
       </c>
       <c r="Q40" s="46" t="inlineStr"/>
@@ -11491,10 +11503,10 @@
           <t>Vacaciones🏖️</t>
         </is>
       </c>
-      <c r="E41" s="47" t="n">
+      <c r="E41" s="52" t="n">
         <v>46111</v>
       </c>
-      <c r="F41" s="47" t="n">
+      <c r="F41" s="52" t="n">
         <v>46113</v>
       </c>
       <c r="G41" s="46" t="inlineStr"/>
@@ -11518,11 +11530,11 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="N41" s="48" t="n">
-        <v>46323.51385416667</v>
+      <c r="N41" s="53" t="n">
+        <v>46324.52037037037</v>
       </c>
       <c r="O41" s="46" t="n"/>
-      <c r="P41" s="48" t="n">
+      <c r="P41" s="53" t="n">
         <v>46323.51385416667</v>
       </c>
       <c r="Q41" s="46" t="inlineStr"/>
@@ -11548,10 +11560,10 @@
           <t>Vacaciones🏖️</t>
         </is>
       </c>
-      <c r="E42" s="47" t="n">
+      <c r="E42" s="52" t="n">
         <v>46108</v>
       </c>
-      <c r="F42" s="47" t="n">
+      <c r="F42" s="52" t="n">
         <v>46108</v>
       </c>
       <c r="G42" s="46" t="inlineStr"/>
@@ -11575,11 +11587,11 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="N42" s="48" t="n">
-        <v>46323.51385416667</v>
+      <c r="N42" s="53" t="n">
+        <v>46324.52037037037</v>
       </c>
       <c r="O42" s="46" t="n"/>
-      <c r="P42" s="48" t="n">
+      <c r="P42" s="53" t="n">
         <v>46323.51385416667</v>
       </c>
       <c r="Q42" s="46" t="inlineStr"/>
@@ -11605,10 +11617,10 @@
           <t>Mudanza, traslado domicilio habitual</t>
         </is>
       </c>
-      <c r="E43" s="47" t="n">
+      <c r="E43" s="52" t="n">
         <v>46104</v>
       </c>
-      <c r="F43" s="47" t="n">
+      <c r="F43" s="52" t="n">
         <v>46104</v>
       </c>
       <c r="G43" s="46" t="inlineStr"/>
@@ -11632,11 +11644,11 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="N43" s="48" t="n">
-        <v>46323.51385416667</v>
+      <c r="N43" s="53" t="n">
+        <v>46324.52037037037</v>
       </c>
       <c r="O43" s="46" t="n"/>
-      <c r="P43" s="48" t="n">
+      <c r="P43" s="53" t="n">
         <v>46323.51385416667</v>
       </c>
       <c r="Q43" s="46" t="inlineStr"/>
@@ -11662,10 +11674,10 @@
           <t>Vacaciones🏖️</t>
         </is>
       </c>
-      <c r="E44" s="47" t="n">
+      <c r="E44" s="52" t="n">
         <v>46105</v>
       </c>
-      <c r="F44" s="47" t="n">
+      <c r="F44" s="52" t="n">
         <v>46111</v>
       </c>
       <c r="G44" s="46" t="inlineStr"/>
@@ -11689,11 +11701,11 @@
           <t>SI</t>
         </is>
       </c>
-      <c r="N44" s="48" t="n">
-        <v>46323.51385416667</v>
+      <c r="N44" s="53" t="n">
+        <v>46324.52037037037</v>
       </c>
       <c r="O44" s="46" t="n"/>
-      <c r="P44" s="48" t="n">
+      <c r="P44" s="53" t="n">
         <v>46323.51385416667</v>
       </c>
       <c r="Q44" s="46" t="inlineStr"/>
@@ -11719,10 +11731,10 @@
           <t>Vacaciones🏖️</t>
         </is>
       </c>
-      <c r="E45" s="47" t="n">
+      <c r="E45" s="52" t="n">
         <v>46217</v>
       </c>
-      <c r="F45" s="47" t="n">
+      <c r="F45" s="52" t="n">
         <v>46234</v>
       </c>
       <c r="G45" s="46" t="inlineStr"/>
@@ -11746,11 +11758,11 @@
           <t>SI</t>
         </is>
       </c>
-      <c r="N45" s="48" t="n">
-        <v>46323.51385416667</v>
+      <c r="N45" s="53" t="n">
+        <v>46324.52037037037</v>
       </c>
       <c r="O45" s="46" t="n"/>
-      <c r="P45" s="48" t="n">
+      <c r="P45" s="53" t="n">
         <v>46323.51385416667</v>
       </c>
       <c r="Q45" s="46" t="inlineStr"/>
@@ -11776,10 +11788,10 @@
           <t>Ausencia</t>
         </is>
       </c>
-      <c r="E46" s="47" t="n">
+      <c r="E46" s="52" t="n">
         <v>46100</v>
       </c>
-      <c r="F46" s="47" t="n">
+      <c r="F46" s="52" t="n">
         <v>46100</v>
       </c>
       <c r="G46" s="46" t="inlineStr"/>
@@ -11803,11 +11815,11 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="N46" s="48" t="n">
-        <v>46323.51385416667</v>
+      <c r="N46" s="53" t="n">
+        <v>46324.52037037037</v>
       </c>
       <c r="O46" s="46" t="n"/>
-      <c r="P46" s="48" t="n">
+      <c r="P46" s="53" t="n">
         <v>46323.51385416667</v>
       </c>
       <c r="Q46" s="46" t="inlineStr"/>
@@ -11833,10 +11845,10 @@
           <t>Ausencia</t>
         </is>
       </c>
-      <c r="E47" s="47" t="n">
+      <c r="E47" s="52" t="n">
         <v>46258</v>
       </c>
-      <c r="F47" s="47" t="n">
+      <c r="F47" s="52" t="n">
         <v>46258</v>
       </c>
       <c r="G47" s="46" t="inlineStr"/>
@@ -11860,11 +11872,11 @@
           <t>SI</t>
         </is>
       </c>
-      <c r="N47" s="48" t="n">
-        <v>46323.51385416667</v>
+      <c r="N47" s="53" t="n">
+        <v>46324.52037037037</v>
       </c>
       <c r="O47" s="46" t="n"/>
-      <c r="P47" s="48" t="n">
+      <c r="P47" s="53" t="n">
         <v>46323.51385416667</v>
       </c>
       <c r="Q47" s="46" t="inlineStr"/>
@@ -11890,10 +11902,10 @@
           <t>Vacaciones🏖️</t>
         </is>
       </c>
-      <c r="E48" s="47" t="n">
+      <c r="E48" s="52" t="n">
         <v>46111</v>
       </c>
-      <c r="F48" s="47" t="n">
+      <c r="F48" s="52" t="n">
         <v>46113</v>
       </c>
       <c r="G48" s="46" t="inlineStr"/>
@@ -11917,11 +11929,11 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="N48" s="48" t="n">
-        <v>46323.51385416667</v>
+      <c r="N48" s="53" t="n">
+        <v>46324.52037037037</v>
       </c>
       <c r="O48" s="46" t="n"/>
-      <c r="P48" s="48" t="n">
+      <c r="P48" s="53" t="n">
         <v>46323.51385416667</v>
       </c>
       <c r="Q48" s="46" t="inlineStr"/>
@@ -11947,10 +11959,10 @@
           <t>Vacaciones🏖️</t>
         </is>
       </c>
-      <c r="E49" s="47" t="n">
+      <c r="E49" s="52" t="n">
         <v>46117</v>
       </c>
-      <c r="F49" s="47" t="n">
+      <c r="F49" s="52" t="n">
         <v>46118</v>
       </c>
       <c r="G49" s="46" t="inlineStr"/>
@@ -11974,11 +11986,11 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="N49" s="48" t="n">
-        <v>46323.51385416667</v>
+      <c r="N49" s="53" t="n">
+        <v>46324.52037037037</v>
       </c>
       <c r="O49" s="46" t="n"/>
-      <c r="P49" s="48" t="n">
+      <c r="P49" s="53" t="n">
         <v>46323.51385416667</v>
       </c>
       <c r="Q49" s="46" t="inlineStr"/>
@@ -12000,10 +12012,10 @@
         </is>
       </c>
       <c r="D50" s="49" t="inlineStr"/>
-      <c r="E50" s="50" t="n">
+      <c r="E50" s="54" t="n">
         <v>46231</v>
       </c>
-      <c r="F50" s="50" t="n">
+      <c r="F50" s="54" t="n">
         <v>46231</v>
       </c>
       <c r="G50" s="49" t="inlineStr"/>
@@ -12027,11 +12039,11 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="N50" s="51" t="n">
-        <v>46323.51385416667</v>
+      <c r="N50" s="55" t="n">
+        <v>46324.52037037037</v>
       </c>
       <c r="O50" s="49" t="n"/>
-      <c r="P50" s="51" t="n">
+      <c r="P50" s="55" t="n">
         <v>46323.51385416667</v>
       </c>
       <c r="Q50" s="49" t="inlineStr">
@@ -12057,10 +12069,10 @@
         </is>
       </c>
       <c r="D51" s="49" t="inlineStr"/>
-      <c r="E51" s="50" t="n">
+      <c r="E51" s="54" t="n">
         <v>46237</v>
       </c>
-      <c r="F51" s="50" t="n">
+      <c r="F51" s="54" t="n">
         <v>46255</v>
       </c>
       <c r="G51" s="49" t="inlineStr"/>
@@ -12084,11 +12096,11 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="N51" s="51" t="n">
-        <v>46323.51385416667</v>
+      <c r="N51" s="55" t="n">
+        <v>46324.52037037037</v>
       </c>
       <c r="O51" s="49" t="n"/>
-      <c r="P51" s="51" t="n">
+      <c r="P51" s="55" t="n">
         <v>46323.51385416667</v>
       </c>
       <c r="Q51" s="49" t="inlineStr">
@@ -12118,10 +12130,10 @@
           <t>Vacaciones🏖️</t>
         </is>
       </c>
-      <c r="E52" s="47" t="n">
+      <c r="E52" s="52" t="n">
         <v>46112</v>
       </c>
-      <c r="F52" s="47" t="n">
+      <c r="F52" s="52" t="n">
         <v>46113</v>
       </c>
       <c r="G52" s="46" t="inlineStr"/>
@@ -12145,11 +12157,11 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="N52" s="48" t="n">
-        <v>46323.51385416667</v>
+      <c r="N52" s="53" t="n">
+        <v>46324.52037037037</v>
       </c>
       <c r="O52" s="46" t="n"/>
-      <c r="P52" s="48" t="n">
+      <c r="P52" s="53" t="n">
         <v>46323.51385416667</v>
       </c>
       <c r="Q52" s="46" t="inlineStr"/>
@@ -12175,10 +12187,10 @@
           <t>Vacaciones🏖️</t>
         </is>
       </c>
-      <c r="E53" s="47" t="n">
+      <c r="E53" s="52" t="n">
         <v>46136</v>
       </c>
-      <c r="F53" s="47" t="n">
+      <c r="F53" s="52" t="n">
         <v>46136</v>
       </c>
       <c r="G53" s="46" t="inlineStr"/>
@@ -12202,11 +12214,11 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="N53" s="48" t="n">
-        <v>46323.51385416667</v>
+      <c r="N53" s="53" t="n">
+        <v>46324.52037037037</v>
       </c>
       <c r="O53" s="46" t="n"/>
-      <c r="P53" s="48" t="n">
+      <c r="P53" s="53" t="n">
         <v>46323.51385416667</v>
       </c>
       <c r="Q53" s="46" t="inlineStr"/>
@@ -12228,10 +12240,10 @@
         </is>
       </c>
       <c r="D54" s="49" t="inlineStr"/>
-      <c r="E54" s="50" t="n">
+      <c r="E54" s="54" t="n">
         <v>46142</v>
       </c>
-      <c r="F54" s="50" t="n">
+      <c r="F54" s="54" t="n">
         <v>46142</v>
       </c>
       <c r="G54" s="49" t="inlineStr"/>
@@ -12255,11 +12267,11 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="N54" s="51" t="n">
-        <v>46323.51385416667</v>
+      <c r="N54" s="55" t="n">
+        <v>46324.52037037037</v>
       </c>
       <c r="O54" s="49" t="n"/>
-      <c r="P54" s="51" t="n">
+      <c r="P54" s="55" t="n">
         <v>46323.51385416667</v>
       </c>
       <c r="Q54" s="49" t="inlineStr">
@@ -12289,10 +12301,10 @@
           <t>Vacaciones🏖️</t>
         </is>
       </c>
-      <c r="E55" s="47" t="n">
+      <c r="E55" s="52" t="n">
         <v>46156</v>
       </c>
-      <c r="F55" s="47" t="n">
+      <c r="F55" s="52" t="n">
         <v>46160</v>
       </c>
       <c r="G55" s="46" t="inlineStr"/>
@@ -12316,11 +12328,11 @@
           <t>SI</t>
         </is>
       </c>
-      <c r="N55" s="48" t="n">
-        <v>46323.51385416667</v>
+      <c r="N55" s="53" t="n">
+        <v>46324.52037037037</v>
       </c>
       <c r="O55" s="46" t="n"/>
-      <c r="P55" s="48" t="n">
+      <c r="P55" s="53" t="n">
         <v>46323.51385416667</v>
       </c>
       <c r="Q55" s="46" t="inlineStr"/>
@@ -12346,10 +12358,10 @@
           <t>Ausencia</t>
         </is>
       </c>
-      <c r="E56" s="47" t="n">
+      <c r="E56" s="52" t="n">
         <v>46192</v>
       </c>
-      <c r="F56" s="47" t="n">
+      <c r="F56" s="52" t="n">
         <v>46192</v>
       </c>
       <c r="G56" s="46" t="inlineStr"/>
@@ -12373,11 +12385,11 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="N56" s="48" t="n">
-        <v>46323.51385416667</v>
+      <c r="N56" s="53" t="n">
+        <v>46324.52037037037</v>
       </c>
       <c r="O56" s="46" t="n"/>
-      <c r="P56" s="48" t="n">
+      <c r="P56" s="53" t="n">
         <v>46323.51385416667</v>
       </c>
       <c r="Q56" s="46" t="inlineStr"/>
@@ -12403,10 +12415,10 @@
           <t>Vacaciones🏖️</t>
         </is>
       </c>
-      <c r="E57" s="47" t="n">
+      <c r="E57" s="52" t="n">
         <v>46191</v>
       </c>
-      <c r="F57" s="47" t="n">
+      <c r="F57" s="52" t="n">
         <v>46191</v>
       </c>
       <c r="G57" s="46" t="inlineStr"/>
@@ -12430,11 +12442,11 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="N57" s="48" t="n">
-        <v>46323.51385416667</v>
+      <c r="N57" s="53" t="n">
+        <v>46324.52037037037</v>
       </c>
       <c r="O57" s="46" t="n"/>
-      <c r="P57" s="48" t="n">
+      <c r="P57" s="53" t="n">
         <v>46323.51385416667</v>
       </c>
       <c r="Q57" s="46" t="inlineStr"/>
@@ -12460,10 +12472,10 @@
           <t>Ausencia</t>
         </is>
       </c>
-      <c r="E58" s="47" t="n">
+      <c r="E58" s="52" t="n">
         <v>46154</v>
       </c>
-      <c r="F58" s="47" t="n">
+      <c r="F58" s="52" t="n">
         <v>46154</v>
       </c>
       <c r="G58" s="46" t="inlineStr"/>
@@ -12487,11 +12499,11 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="N58" s="48" t="n">
-        <v>46323.51385416667</v>
+      <c r="N58" s="53" t="n">
+        <v>46324.52037037037</v>
       </c>
       <c r="O58" s="46" t="n"/>
-      <c r="P58" s="48" t="n">
+      <c r="P58" s="53" t="n">
         <v>46323.51385416667</v>
       </c>
       <c r="Q58" s="46" t="inlineStr"/>
@@ -12517,10 +12529,10 @@
           <t>Ausencia</t>
         </is>
       </c>
-      <c r="E59" s="47" t="n">
+      <c r="E59" s="52" t="n">
         <v>46150</v>
       </c>
-      <c r="F59" s="47" t="n">
+      <c r="F59" s="52" t="n">
         <v>46150</v>
       </c>
       <c r="G59" s="46" t="inlineStr"/>
@@ -12544,11 +12556,11 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="N59" s="48" t="n">
-        <v>46323.51385416667</v>
+      <c r="N59" s="53" t="n">
+        <v>46324.52037037037</v>
       </c>
       <c r="O59" s="46" t="n"/>
-      <c r="P59" s="48" t="n">
+      <c r="P59" s="53" t="n">
         <v>46323.51385416667</v>
       </c>
       <c r="Q59" s="46" t="inlineStr"/>
@@ -12574,10 +12586,10 @@
           <t>Ausencia</t>
         </is>
       </c>
-      <c r="E60" s="47" t="n">
+      <c r="E60" s="52" t="n">
         <v>46149</v>
       </c>
-      <c r="F60" s="47" t="n">
+      <c r="F60" s="52" t="n">
         <v>46149</v>
       </c>
       <c r="G60" s="46" t="inlineStr">
@@ -12609,11 +12621,11 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="N60" s="48" t="n">
-        <v>46323.51385416667</v>
+      <c r="N60" s="53" t="n">
+        <v>46324.52037037037</v>
       </c>
       <c r="O60" s="46" t="n"/>
-      <c r="P60" s="48" t="n">
+      <c r="P60" s="53" t="n">
         <v>46323.51385416667</v>
       </c>
       <c r="Q60" s="46" t="inlineStr"/>
@@ -12639,10 +12651,10 @@
           <t>Ausencia</t>
         </is>
       </c>
-      <c r="E61" s="47" t="n">
+      <c r="E61" s="52" t="n">
         <v>46125</v>
       </c>
-      <c r="F61" s="47" t="n">
+      <c r="F61" s="52" t="n">
         <v>46129</v>
       </c>
       <c r="G61" s="46" t="inlineStr"/>
@@ -12666,11 +12678,11 @@
           <t>SI</t>
         </is>
       </c>
-      <c r="N61" s="48" t="n">
-        <v>46323.51385416667</v>
+      <c r="N61" s="53" t="n">
+        <v>46324.52037037037</v>
       </c>
       <c r="O61" s="46" t="n"/>
-      <c r="P61" s="48" t="n">
+      <c r="P61" s="53" t="n">
         <v>46323.51385416667</v>
       </c>
       <c r="Q61" s="46" t="inlineStr"/>
@@ -12696,10 +12708,10 @@
           <t>Ausencia</t>
         </is>
       </c>
-      <c r="E62" s="50" t="n">
+      <c r="E62" s="54" t="n">
         <v>46223</v>
       </c>
-      <c r="F62" s="50" t="n">
+      <c r="F62" s="54" t="n">
         <v>46237</v>
       </c>
       <c r="G62" s="49" t="inlineStr"/>
@@ -12723,11 +12735,11 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="N62" s="51" t="n">
-        <v>46323.51385416667</v>
+      <c r="N62" s="55" t="n">
+        <v>46324.52037037037</v>
       </c>
       <c r="O62" s="49" t="n"/>
-      <c r="P62" s="51" t="n">
+      <c r="P62" s="55" t="n">
         <v>46323.51385416667</v>
       </c>
       <c r="Q62" s="49" t="inlineStr">
@@ -12757,10 +12769,10 @@
           <t>Vacaciones🏖️</t>
         </is>
       </c>
-      <c r="E63" s="50" t="n">
+      <c r="E63" s="54" t="n">
         <v>46238</v>
       </c>
-      <c r="F63" s="50" t="n">
+      <c r="F63" s="54" t="n">
         <v>46244</v>
       </c>
       <c r="G63" s="49" t="inlineStr"/>
@@ -12784,11 +12796,11 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="N63" s="51" t="n">
-        <v>46323.51385416667</v>
+      <c r="N63" s="55" t="n">
+        <v>46324.52037037037</v>
       </c>
       <c r="O63" s="49" t="n"/>
-      <c r="P63" s="51" t="n">
+      <c r="P63" s="55" t="n">
         <v>46323.51385416667</v>
       </c>
       <c r="Q63" s="49" t="inlineStr">
@@ -12818,10 +12830,10 @@
           <t>Vacaciones🏖️</t>
         </is>
       </c>
-      <c r="E64" s="47" t="n">
+      <c r="E64" s="52" t="n">
         <v>46209</v>
       </c>
-      <c r="F64" s="47" t="n">
+      <c r="F64" s="52" t="n">
         <v>46213</v>
       </c>
       <c r="G64" s="46" t="inlineStr"/>
@@ -12845,11 +12857,11 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="N64" s="48" t="n">
-        <v>46323.51385416667</v>
+      <c r="N64" s="53" t="n">
+        <v>46324.52037037037</v>
       </c>
       <c r="O64" s="46" t="n"/>
-      <c r="P64" s="48" t="n">
+      <c r="P64" s="53" t="n">
         <v>46323.51385416667</v>
       </c>
       <c r="Q64" s="46" t="inlineStr"/>
@@ -12875,10 +12887,10 @@
           <t>Vacaciones🏖️</t>
         </is>
       </c>
-      <c r="E65" s="47" t="n">
+      <c r="E65" s="52" t="n">
         <v>46244</v>
       </c>
-      <c r="F65" s="47" t="n">
+      <c r="F65" s="52" t="n">
         <v>46257</v>
       </c>
       <c r="G65" s="46" t="inlineStr"/>
@@ -12902,11 +12914,11 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="N65" s="48" t="n">
-        <v>46323.51385416667</v>
+      <c r="N65" s="53" t="n">
+        <v>46324.52037037037</v>
       </c>
       <c r="O65" s="46" t="n"/>
-      <c r="P65" s="48" t="n">
+      <c r="P65" s="53" t="n">
         <v>46323.51385416667</v>
       </c>
       <c r="Q65" s="46" t="inlineStr"/>
@@ -12932,10 +12944,10 @@
           <t>Vacaciones🏖️</t>
         </is>
       </c>
-      <c r="E66" s="47" t="n">
+      <c r="E66" s="52" t="n">
         <v>46182</v>
       </c>
-      <c r="F66" s="47" t="n">
+      <c r="F66" s="52" t="n">
         <v>46184</v>
       </c>
       <c r="G66" s="46" t="inlineStr"/>
@@ -12959,11 +12971,11 @@
           <t>SI</t>
         </is>
       </c>
-      <c r="N66" s="48" t="n">
-        <v>46323.51385416667</v>
+      <c r="N66" s="53" t="n">
+        <v>46324.52037037037</v>
       </c>
       <c r="O66" s="46" t="n"/>
-      <c r="P66" s="48" t="n">
+      <c r="P66" s="53" t="n">
         <v>46323.51385416667</v>
       </c>
       <c r="Q66" s="46" t="inlineStr"/>
@@ -12989,10 +13001,10 @@
           <t>Vacaciones🏖️</t>
         </is>
       </c>
-      <c r="E67" s="47" t="n">
+      <c r="E67" s="52" t="n">
         <v>46206</v>
       </c>
-      <c r="F67" s="47" t="n">
+      <c r="F67" s="52" t="n">
         <v>46206</v>
       </c>
       <c r="G67" s="46" t="inlineStr"/>
@@ -13016,11 +13028,11 @@
           <t>SI</t>
         </is>
       </c>
-      <c r="N67" s="48" t="n">
-        <v>46323.51385416667</v>
+      <c r="N67" s="53" t="n">
+        <v>46324.52037037037</v>
       </c>
       <c r="O67" s="46" t="n"/>
-      <c r="P67" s="48" t="n">
+      <c r="P67" s="53" t="n">
         <v>46323.51385416667</v>
       </c>
       <c r="Q67" s="46" t="inlineStr"/>
@@ -13046,10 +13058,10 @@
           <t>Vacaciones🏖️</t>
         </is>
       </c>
-      <c r="E68" s="47" t="n">
+      <c r="E68" s="52" t="n">
         <v>46195</v>
       </c>
-      <c r="F68" s="47" t="n">
+      <c r="F68" s="52" t="n">
         <v>46195</v>
       </c>
       <c r="G68" s="46" t="inlineStr"/>
@@ -13073,11 +13085,11 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="N68" s="48" t="n">
-        <v>46323.51385416667</v>
+      <c r="N68" s="53" t="n">
+        <v>46324.52037037037</v>
       </c>
       <c r="O68" s="46" t="n"/>
-      <c r="P68" s="48" t="n">
+      <c r="P68" s="53" t="n">
         <v>46323.51385416667</v>
       </c>
       <c r="Q68" s="46" t="inlineStr"/>
@@ -13103,10 +13115,10 @@
           <t>Vacaciones🏖️</t>
         </is>
       </c>
-      <c r="E69" s="47" t="n">
+      <c r="E69" s="52" t="n">
         <v>46194</v>
       </c>
-      <c r="F69" s="47" t="n">
+      <c r="F69" s="52" t="n">
         <v>46195</v>
       </c>
       <c r="G69" s="46" t="inlineStr"/>
@@ -13130,11 +13142,11 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="N69" s="48" t="n">
-        <v>46323.51385416667</v>
+      <c r="N69" s="53" t="n">
+        <v>46324.52037037037</v>
       </c>
       <c r="O69" s="46" t="n"/>
-      <c r="P69" s="48" t="n">
+      <c r="P69" s="53" t="n">
         <v>46323.51385416667</v>
       </c>
       <c r="Q69" s="46" t="inlineStr"/>
@@ -13160,10 +13172,10 @@
           <t>Vacaciones🏖️</t>
         </is>
       </c>
-      <c r="E70" s="50" t="n">
+      <c r="E70" s="54" t="n">
         <v>46192</v>
       </c>
-      <c r="F70" s="50" t="n">
+      <c r="F70" s="54" t="n">
         <v>46192</v>
       </c>
       <c r="G70" s="49" t="inlineStr"/>
@@ -13187,11 +13199,11 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="N70" s="51" t="n">
-        <v>46323.51385416667</v>
+      <c r="N70" s="55" t="n">
+        <v>46324.52037037037</v>
       </c>
       <c r="O70" s="49" t="n"/>
-      <c r="P70" s="51" t="n">
+      <c r="P70" s="55" t="n">
         <v>46323.51385416667</v>
       </c>
       <c r="Q70" s="49" t="inlineStr">
@@ -13221,10 +13233,10 @@
           <t>Vacaciones🏖️</t>
         </is>
       </c>
-      <c r="E71" s="47" t="n">
+      <c r="E71" s="52" t="n">
         <v>46199</v>
       </c>
-      <c r="F71" s="47" t="n">
+      <c r="F71" s="52" t="n">
         <v>46199</v>
       </c>
       <c r="G71" s="46" t="inlineStr"/>
@@ -13248,11 +13260,11 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="N71" s="48" t="n">
-        <v>46323.51385416667</v>
+      <c r="N71" s="53" t="n">
+        <v>46324.52037037037</v>
       </c>
       <c r="O71" s="46" t="n"/>
-      <c r="P71" s="48" t="n">
+      <c r="P71" s="53" t="n">
         <v>46323.51385416667</v>
       </c>
       <c r="Q71" s="46" t="inlineStr"/>
@@ -13278,10 +13290,10 @@
           <t>Vacaciones🏖️</t>
         </is>
       </c>
-      <c r="E72" s="47" t="n">
+      <c r="E72" s="52" t="n">
         <v>46216</v>
       </c>
-      <c r="F72" s="47" t="n">
+      <c r="F72" s="52" t="n">
         <v>46233</v>
       </c>
       <c r="G72" s="46" t="inlineStr"/>
@@ -13305,11 +13317,11 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="N72" s="48" t="n">
-        <v>46323.51385416667</v>
+      <c r="N72" s="53" t="n">
+        <v>46324.52037037037</v>
       </c>
       <c r="O72" s="46" t="n"/>
-      <c r="P72" s="48" t="n">
+      <c r="P72" s="53" t="n">
         <v>46323.51385416667</v>
       </c>
       <c r="Q72" s="46" t="inlineStr"/>
@@ -13335,10 +13347,10 @@
           <t>Vacaciones🏖️</t>
         </is>
       </c>
-      <c r="E73" s="47" t="n">
+      <c r="E73" s="52" t="n">
         <v>46234</v>
       </c>
-      <c r="F73" s="47" t="n">
+      <c r="F73" s="52" t="n">
         <v>46234</v>
       </c>
       <c r="G73" s="46" t="inlineStr"/>
@@ -13362,11 +13374,11 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="N73" s="48" t="n">
-        <v>46323.51385416667</v>
+      <c r="N73" s="53" t="n">
+        <v>46324.52037037037</v>
       </c>
       <c r="O73" s="46" t="n"/>
-      <c r="P73" s="48" t="n">
+      <c r="P73" s="53" t="n">
         <v>46323.51385416667</v>
       </c>
       <c r="Q73" s="46" t="inlineStr"/>
@@ -13392,10 +13404,10 @@
           <t>Vacaciones🏖️</t>
         </is>
       </c>
-      <c r="E74" s="47" t="n">
+      <c r="E74" s="52" t="n">
         <v>46237</v>
       </c>
-      <c r="F74" s="47" t="n">
+      <c r="F74" s="52" t="n">
         <v>46241</v>
       </c>
       <c r="G74" s="46" t="inlineStr"/>
@@ -13419,11 +13431,11 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="N74" s="48" t="n">
-        <v>46323.51385416667</v>
+      <c r="N74" s="53" t="n">
+        <v>46324.52037037037</v>
       </c>
       <c r="O74" s="46" t="n"/>
-      <c r="P74" s="48" t="n">
+      <c r="P74" s="53" t="n">
         <v>46323.51385416667</v>
       </c>
       <c r="Q74" s="46" t="inlineStr"/>
@@ -13449,10 +13461,10 @@
           <t>Vacaciones🏖️</t>
         </is>
       </c>
-      <c r="E75" s="47" t="n">
+      <c r="E75" s="52" t="n">
         <v>46246</v>
       </c>
-      <c r="F75" s="47" t="n">
+      <c r="F75" s="52" t="n">
         <v>46248</v>
       </c>
       <c r="G75" s="46" t="inlineStr"/>
@@ -13476,11 +13488,11 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="N75" s="48" t="n">
-        <v>46323.51385416667</v>
+      <c r="N75" s="53" t="n">
+        <v>46324.52037037037</v>
       </c>
       <c r="O75" s="46" t="n"/>
-      <c r="P75" s="48" t="n">
+      <c r="P75" s="53" t="n">
         <v>46323.51385416667</v>
       </c>
       <c r="Q75" s="46" t="inlineStr"/>
@@ -13506,10 +13518,10 @@
           <t>Vacaciones🏖️</t>
         </is>
       </c>
-      <c r="E76" s="47" t="n">
+      <c r="E76" s="52" t="n">
         <v>46255</v>
       </c>
-      <c r="F76" s="47" t="n">
+      <c r="F76" s="52" t="n">
         <v>46272</v>
       </c>
       <c r="G76" s="46" t="inlineStr"/>
@@ -13533,11 +13545,11 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="N76" s="48" t="n">
-        <v>46323.51385416667</v>
+      <c r="N76" s="53" t="n">
+        <v>46324.52037037037</v>
       </c>
       <c r="O76" s="46" t="n"/>
-      <c r="P76" s="48" t="n">
+      <c r="P76" s="53" t="n">
         <v>46323.51385416667</v>
       </c>
       <c r="Q76" s="46" t="inlineStr"/>
@@ -13563,10 +13575,10 @@
           <t>Vacaciones🏖️</t>
         </is>
       </c>
-      <c r="E77" s="47" t="n">
+      <c r="E77" s="52" t="n">
         <v>46238</v>
       </c>
-      <c r="F77" s="47" t="n">
+      <c r="F77" s="52" t="n">
         <v>46251</v>
       </c>
       <c r="G77" s="46" t="inlineStr"/>
@@ -13590,11 +13602,11 @@
           <t>SI</t>
         </is>
       </c>
-      <c r="N77" s="48" t="n">
-        <v>46323.51385416667</v>
+      <c r="N77" s="53" t="n">
+        <v>46324.52037037037</v>
       </c>
       <c r="O77" s="46" t="n"/>
-      <c r="P77" s="48" t="n">
+      <c r="P77" s="53" t="n">
         <v>46323.51385416667</v>
       </c>
       <c r="Q77" s="46" t="inlineStr"/>
@@ -13620,10 +13632,10 @@
           <t>Vacaciones🏖️</t>
         </is>
       </c>
-      <c r="E78" s="47" t="n">
+      <c r="E78" s="52" t="n">
         <v>46244</v>
       </c>
-      <c r="F78" s="47" t="n">
+      <c r="F78" s="52" t="n">
         <v>46255</v>
       </c>
       <c r="G78" s="46" t="inlineStr"/>
@@ -13647,11 +13659,11 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="N78" s="48" t="n">
-        <v>46323.51385416667</v>
+      <c r="N78" s="53" t="n">
+        <v>46324.52037037037</v>
       </c>
       <c r="O78" s="46" t="n"/>
-      <c r="P78" s="48" t="n">
+      <c r="P78" s="53" t="n">
         <v>46323.51385416667</v>
       </c>
       <c r="Q78" s="46" t="inlineStr"/>
@@ -13677,10 +13689,10 @@
           <t>Vacaciones🏖️</t>
         </is>
       </c>
-      <c r="E79" s="47" t="n">
+      <c r="E79" s="52" t="n">
         <v>46269</v>
       </c>
-      <c r="F79" s="47" t="n">
+      <c r="F79" s="52" t="n">
         <v>46276</v>
       </c>
       <c r="G79" s="46" t="inlineStr"/>
@@ -13704,11 +13716,11 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="N79" s="48" t="n">
-        <v>46323.51385416667</v>
+      <c r="N79" s="53" t="n">
+        <v>46324.52037037037</v>
       </c>
       <c r="O79" s="46" t="n"/>
-      <c r="P79" s="48" t="n">
+      <c r="P79" s="53" t="n">
         <v>46323.51385416667</v>
       </c>
       <c r="Q79" s="46" t="inlineStr"/>
@@ -13734,10 +13746,10 @@
           <t>Vacaciones🏖️</t>
         </is>
       </c>
-      <c r="E80" s="47" t="n">
+      <c r="E80" s="52" t="n">
         <v>46238</v>
       </c>
-      <c r="F80" s="47" t="n">
+      <c r="F80" s="52" t="n">
         <v>46240</v>
       </c>
       <c r="G80" s="46" t="inlineStr"/>
@@ -13761,11 +13773,11 @@
           <t>SI</t>
         </is>
       </c>
-      <c r="N80" s="48" t="n">
-        <v>46323.51385416667</v>
+      <c r="N80" s="53" t="n">
+        <v>46324.52037037037</v>
       </c>
       <c r="O80" s="46" t="n"/>
-      <c r="P80" s="48" t="n">
+      <c r="P80" s="53" t="n">
         <v>46323.51385416667</v>
       </c>
       <c r="Q80" s="46" t="inlineStr"/>
@@ -13791,10 +13803,10 @@
           <t>Vacaciones🏖️</t>
         </is>
       </c>
-      <c r="E81" s="47" t="n">
+      <c r="E81" s="52" t="n">
         <v>46251</v>
       </c>
-      <c r="F81" s="47" t="n">
+      <c r="F81" s="52" t="n">
         <v>46260</v>
       </c>
       <c r="G81" s="46" t="inlineStr"/>
@@ -13818,11 +13830,11 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="N81" s="48" t="n">
-        <v>46323.51385416667</v>
+      <c r="N81" s="53" t="n">
+        <v>46324.52037037037</v>
       </c>
       <c r="O81" s="46" t="n"/>
-      <c r="P81" s="48" t="n">
+      <c r="P81" s="53" t="n">
         <v>46323.51385416667</v>
       </c>
       <c r="Q81" s="46" t="inlineStr"/>
@@ -13848,10 +13860,10 @@
           <t>Vacaciones🏖️</t>
         </is>
       </c>
-      <c r="E82" s="47" t="n">
+      <c r="E82" s="52" t="n">
         <v>46240</v>
       </c>
-      <c r="F82" s="47" t="n">
+      <c r="F82" s="52" t="n">
         <v>46240</v>
       </c>
       <c r="G82" s="46" t="inlineStr"/>
@@ -13875,11 +13887,11 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="N82" s="48" t="n">
-        <v>46323.51385416667</v>
+      <c r="N82" s="53" t="n">
+        <v>46324.52037037037</v>
       </c>
       <c r="O82" s="46" t="n"/>
-      <c r="P82" s="48" t="n">
+      <c r="P82" s="53" t="n">
         <v>46323.51385416667</v>
       </c>
       <c r="Q82" s="46" t="inlineStr"/>
@@ -13905,10 +13917,10 @@
           <t>Vacaciones🏖️</t>
         </is>
       </c>
-      <c r="E83" s="47" t="n">
+      <c r="E83" s="52" t="n">
         <v>46241</v>
       </c>
-      <c r="F83" s="47" t="n">
+      <c r="F83" s="52" t="n">
         <v>46241</v>
       </c>
       <c r="G83" s="46" t="inlineStr"/>
@@ -13932,11 +13944,11 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="N83" s="48" t="n">
-        <v>46323.51385416667</v>
+      <c r="N83" s="53" t="n">
+        <v>46324.52037037037</v>
       </c>
       <c r="O83" s="46" t="n"/>
-      <c r="P83" s="48" t="n">
+      <c r="P83" s="53" t="n">
         <v>46323.51385416667</v>
       </c>
       <c r="Q83" s="46" t="inlineStr"/>
@@ -13962,10 +13974,10 @@
           <t>Vacaciones🏖️</t>
         </is>
       </c>
-      <c r="E84" s="47" t="n">
+      <c r="E84" s="52" t="n">
         <v>46251</v>
       </c>
-      <c r="F84" s="47" t="n">
+      <c r="F84" s="52" t="n">
         <v>46255</v>
       </c>
       <c r="G84" s="46" t="inlineStr"/>
@@ -13989,11 +14001,11 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="N84" s="48" t="n">
-        <v>46323.51385416667</v>
+      <c r="N84" s="53" t="n">
+        <v>46324.52037037037</v>
       </c>
       <c r="O84" s="46" t="n"/>
-      <c r="P84" s="48" t="n">
+      <c r="P84" s="53" t="n">
         <v>46323.51385416667</v>
       </c>
       <c r="Q84" s="46" t="inlineStr"/>
@@ -14019,10 +14031,10 @@
           <t>Ausencia</t>
         </is>
       </c>
-      <c r="E85" s="47" t="n">
+      <c r="E85" s="52" t="n">
         <v>46255</v>
       </c>
-      <c r="F85" s="47" t="n">
+      <c r="F85" s="52" t="n">
         <v>46255</v>
       </c>
       <c r="G85" s="46" t="inlineStr"/>
@@ -14046,11 +14058,11 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="N85" s="48" t="n">
-        <v>46323.51385416667</v>
+      <c r="N85" s="53" t="n">
+        <v>46324.52037037037</v>
       </c>
       <c r="O85" s="46" t="n"/>
-      <c r="P85" s="48" t="n">
+      <c r="P85" s="53" t="n">
         <v>46323.51385416667</v>
       </c>
       <c r="Q85" s="46" t="inlineStr"/>
@@ -14076,10 +14088,10 @@
           <t>Mudanza, traslado domicilio habitual</t>
         </is>
       </c>
-      <c r="E86" s="47" t="n">
+      <c r="E86" s="52" t="n">
         <v>46268</v>
       </c>
-      <c r="F86" s="47" t="n">
+      <c r="F86" s="52" t="n">
         <v>46268</v>
       </c>
       <c r="G86" s="46" t="inlineStr"/>
@@ -14103,11 +14115,11 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="N86" s="48" t="n">
-        <v>46323.51385416667</v>
+      <c r="N86" s="53" t="n">
+        <v>46324.52037037037</v>
       </c>
       <c r="O86" s="46" t="n"/>
-      <c r="P86" s="48" t="n">
+      <c r="P86" s="53" t="n">
         <v>46323.51385416667</v>
       </c>
       <c r="Q86" s="46" t="inlineStr"/>
@@ -14133,10 +14145,10 @@
           <t>Vacaciones🏖️</t>
         </is>
       </c>
-      <c r="E87" s="47" t="n">
+      <c r="E87" s="52" t="n">
         <v>46244</v>
       </c>
-      <c r="F87" s="47" t="n">
+      <c r="F87" s="52" t="n">
         <v>46248</v>
       </c>
       <c r="G87" s="46" t="inlineStr"/>
@@ -14160,11 +14172,11 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="N87" s="48" t="n">
-        <v>46323.51385416667</v>
+      <c r="N87" s="53" t="n">
+        <v>46324.52037037037</v>
       </c>
       <c r="O87" s="46" t="n"/>
-      <c r="P87" s="48" t="n">
+      <c r="P87" s="53" t="n">
         <v>46323.51385416667</v>
       </c>
       <c r="Q87" s="46" t="inlineStr"/>
@@ -14190,10 +14202,10 @@
           <t>Vacaciones🏖️</t>
         </is>
       </c>
-      <c r="E88" s="47" t="n">
+      <c r="E88" s="52" t="n">
         <v>46251</v>
       </c>
-      <c r="F88" s="47" t="n">
+      <c r="F88" s="52" t="n">
         <v>46255</v>
       </c>
       <c r="G88" s="46" t="inlineStr"/>
@@ -14217,11 +14229,11 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="N88" s="48" t="n">
-        <v>46323.51385416667</v>
+      <c r="N88" s="53" t="n">
+        <v>46324.52037037037</v>
       </c>
       <c r="O88" s="46" t="n"/>
-      <c r="P88" s="48" t="n">
+      <c r="P88" s="53" t="n">
         <v>46323.51385416667</v>
       </c>
       <c r="Q88" s="46" t="inlineStr"/>
@@ -14247,10 +14259,10 @@
           <t>Ausencia</t>
         </is>
       </c>
-      <c r="E89" s="47" t="n">
+      <c r="E89" s="52" t="n">
         <v>46275</v>
       </c>
-      <c r="F89" s="47" t="n">
+      <c r="F89" s="52" t="n">
         <v>46275</v>
       </c>
       <c r="G89" s="46" t="inlineStr">
@@ -14282,11 +14294,11 @@
           <t>SI</t>
         </is>
       </c>
-      <c r="N89" s="48" t="n">
-        <v>46323.51385416667</v>
+      <c r="N89" s="53" t="n">
+        <v>46324.52037037037</v>
       </c>
       <c r="O89" s="46" t="n"/>
-      <c r="P89" s="48" t="n">
+      <c r="P89" s="53" t="n">
         <v>46323.51385416667</v>
       </c>
       <c r="Q89" s="46" t="inlineStr"/>
@@ -14312,10 +14324,10 @@
           <t>Ausencia</t>
         </is>
       </c>
-      <c r="E90" s="47" t="n">
+      <c r="E90" s="52" t="n">
         <v>46261</v>
       </c>
-      <c r="F90" s="47" t="n">
+      <c r="F90" s="52" t="n">
         <v>46261</v>
       </c>
       <c r="G90" s="46" t="inlineStr"/>
@@ -14339,11 +14351,11 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="N90" s="48" t="n">
-        <v>46323.51385416667</v>
+      <c r="N90" s="53" t="n">
+        <v>46324.52037037037</v>
       </c>
       <c r="O90" s="46" t="n"/>
-      <c r="P90" s="48" t="n">
+      <c r="P90" s="53" t="n">
         <v>46323.51385416667</v>
       </c>
       <c r="Q90" s="46" t="inlineStr"/>
@@ -14369,10 +14381,10 @@
           <t>Vacaciones🏖️</t>
         </is>
       </c>
-      <c r="E91" s="47" t="n">
+      <c r="E91" s="52" t="n">
         <v>46262</v>
       </c>
-      <c r="F91" s="47" t="n">
+      <c r="F91" s="52" t="n">
         <v>46262</v>
       </c>
       <c r="G91" s="46" t="inlineStr"/>
@@ -14396,11 +14408,11 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="N91" s="48" t="n">
-        <v>46323.51385416667</v>
+      <c r="N91" s="53" t="n">
+        <v>46324.52037037037</v>
       </c>
       <c r="O91" s="46" t="n"/>
-      <c r="P91" s="48" t="n">
+      <c r="P91" s="53" t="n">
         <v>46323.51385416667</v>
       </c>
       <c r="Q91" s="46" t="inlineStr"/>
@@ -14426,10 +14438,10 @@
           <t>Vacaciones🏖️</t>
         </is>
       </c>
-      <c r="E92" s="47" t="n">
+      <c r="E92" s="52" t="n">
         <v>46272</v>
       </c>
-      <c r="F92" s="47" t="n">
+      <c r="F92" s="52" t="n">
         <v>46276</v>
       </c>
       <c r="G92" s="46" t="inlineStr"/>
@@ -14453,11 +14465,11 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="N92" s="48" t="n">
-        <v>46323.51385416667</v>
+      <c r="N92" s="53" t="n">
+        <v>46324.52037037037</v>
       </c>
       <c r="O92" s="46" t="n"/>
-      <c r="P92" s="48" t="n">
+      <c r="P92" s="53" t="n">
         <v>46323.51385416667</v>
       </c>
       <c r="Q92" s="46" t="inlineStr"/>
@@ -14483,10 +14495,10 @@
           <t>Vacaciones🏖️</t>
         </is>
       </c>
-      <c r="E93" s="47" t="n">
+      <c r="E93" s="52" t="n">
         <v>46296</v>
       </c>
-      <c r="F93" s="47" t="n">
+      <c r="F93" s="52" t="n">
         <v>46300</v>
       </c>
       <c r="G93" s="46" t="inlineStr"/>
@@ -14510,11 +14522,11 @@
           <t>SI</t>
         </is>
       </c>
-      <c r="N93" s="48" t="n">
-        <v>46323.51385416667</v>
+      <c r="N93" s="53" t="n">
+        <v>46324.52037037037</v>
       </c>
       <c r="O93" s="46" t="n"/>
-      <c r="P93" s="48" t="n">
+      <c r="P93" s="53" t="n">
         <v>46323.51385416667</v>
       </c>
       <c r="Q93" s="46" t="inlineStr"/>
@@ -14540,10 +14552,10 @@
           <t>Vacaciones🏖️</t>
         </is>
       </c>
-      <c r="E94" s="50" t="n">
+      <c r="E94" s="54" t="n">
         <v>46276</v>
       </c>
-      <c r="F94" s="50" t="n">
+      <c r="F94" s="54" t="n">
         <v>46276</v>
       </c>
       <c r="G94" s="49" t="inlineStr"/>
@@ -14567,11 +14579,11 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="N94" s="51" t="n">
-        <v>46323.51385416667</v>
+      <c r="N94" s="55" t="n">
+        <v>46324.52037037037</v>
       </c>
       <c r="O94" s="49" t="n"/>
-      <c r="P94" s="51" t="n">
+      <c r="P94" s="55" t="n">
         <v>46323.51385416667</v>
       </c>
       <c r="Q94" s="49" t="inlineStr">
@@ -14601,10 +14613,10 @@
           <t>Ausencia</t>
         </is>
       </c>
-      <c r="E95" s="47" t="n">
+      <c r="E95" s="52" t="n">
         <v>46290</v>
       </c>
-      <c r="F95" s="47" t="n">
+      <c r="F95" s="52" t="n">
         <v>46290</v>
       </c>
       <c r="G95" s="46" t="inlineStr"/>
@@ -14628,11 +14640,11 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="N95" s="48" t="n">
-        <v>46323.51385416667</v>
+      <c r="N95" s="53" t="n">
+        <v>46324.52037037037</v>
       </c>
       <c r="O95" s="46" t="n"/>
-      <c r="P95" s="48" t="n">
+      <c r="P95" s="53" t="n">
         <v>46323.51385416667</v>
       </c>
       <c r="Q95" s="46" t="inlineStr"/>
@@ -14658,10 +14670,10 @@
           <t>Vacaciones🏖️</t>
         </is>
       </c>
-      <c r="E96" s="47" t="n">
+      <c r="E96" s="52" t="n">
         <v>46310</v>
       </c>
-      <c r="F96" s="47" t="n">
+      <c r="F96" s="52" t="n">
         <v>46316</v>
       </c>
       <c r="G96" s="46" t="inlineStr"/>
@@ -14689,11 +14701,11 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="N96" s="48" t="n">
-        <v>46323.51385416667</v>
+      <c r="N96" s="53" t="n">
+        <v>46324.52037037037</v>
       </c>
       <c r="O96" s="46" t="n"/>
-      <c r="P96" s="48" t="n">
+      <c r="P96" s="53" t="n">
         <v>46323.51385416667</v>
       </c>
       <c r="Q96" s="46" t="inlineStr"/>
@@ -14719,10 +14731,10 @@
           <t>Mudanza, traslado domicilio habitual</t>
         </is>
       </c>
-      <c r="E97" s="47" t="n">
+      <c r="E97" s="52" t="n">
         <v>46300</v>
       </c>
-      <c r="F97" s="47" t="n">
+      <c r="F97" s="52" t="n">
         <v>46300</v>
       </c>
       <c r="G97" s="46" t="inlineStr"/>
@@ -14746,11 +14758,11 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="N97" s="48" t="n">
-        <v>46323.51385416667</v>
+      <c r="N97" s="53" t="n">
+        <v>46324.52037037037</v>
       </c>
       <c r="O97" s="46" t="n"/>
-      <c r="P97" s="48" t="n">
+      <c r="P97" s="53" t="n">
         <v>46323.51385416667</v>
       </c>
       <c r="Q97" s="46" t="inlineStr"/>
@@ -14776,10 +14788,10 @@
           <t>Ausencia</t>
         </is>
       </c>
-      <c r="E98" s="47" t="n">
+      <c r="E98" s="52" t="n">
         <v>46336</v>
       </c>
-      <c r="F98" s="47" t="n">
+      <c r="F98" s="52" t="n">
         <v>46336</v>
       </c>
       <c r="G98" s="46" t="inlineStr">
@@ -14815,11 +14827,11 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="N98" s="48" t="n">
-        <v>46323.51385416667</v>
+      <c r="N98" s="53" t="n">
+        <v>46324.52037037037</v>
       </c>
       <c r="O98" s="46" t="n"/>
-      <c r="P98" s="48" t="n">
+      <c r="P98" s="53" t="n">
         <v>46323.51385416667</v>
       </c>
       <c r="Q98" s="46" t="inlineStr"/>
@@ -14845,10 +14857,10 @@
           <t>Vacaciones🏖️</t>
         </is>
       </c>
-      <c r="E99" s="47" t="n">
+      <c r="E99" s="52" t="n">
         <v>46304</v>
       </c>
-      <c r="F99" s="47" t="n">
+      <c r="F99" s="52" t="n">
         <v>46304</v>
       </c>
       <c r="G99" s="46" t="inlineStr"/>
@@ -14872,11 +14884,11 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="N99" s="48" t="n">
-        <v>46323.51385416667</v>
+      <c r="N99" s="53" t="n">
+        <v>46324.52037037037</v>
       </c>
       <c r="O99" s="46" t="n"/>
-      <c r="P99" s="48" t="n">
+      <c r="P99" s="53" t="n">
         <v>46323.51385416667</v>
       </c>
       <c r="Q99" s="46" t="inlineStr"/>
@@ -14902,10 +14914,10 @@
           <t>Vacaciones🏖️</t>
         </is>
       </c>
-      <c r="E100" s="47" t="n">
+      <c r="E100" s="52" t="n">
         <v>46308</v>
       </c>
-      <c r="F100" s="47" t="n">
+      <c r="F100" s="52" t="n">
         <v>46308</v>
       </c>
       <c r="G100" s="46" t="inlineStr"/>
@@ -14933,11 +14945,11 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="N100" s="48" t="n">
-        <v>46323.51385416667</v>
+      <c r="N100" s="53" t="n">
+        <v>46324.52037037037</v>
       </c>
       <c r="O100" s="46" t="n"/>
-      <c r="P100" s="48" t="n">
+      <c r="P100" s="53" t="n">
         <v>46323.51385416667</v>
       </c>
       <c r="Q100" s="46" t="inlineStr"/>
@@ -14963,10 +14975,10 @@
           <t>Vacaciones🏖️</t>
         </is>
       </c>
-      <c r="E101" s="47" t="n">
+      <c r="E101" s="52" t="n">
         <v>46301</v>
       </c>
-      <c r="F101" s="47" t="n">
+      <c r="F101" s="52" t="n">
         <v>46301</v>
       </c>
       <c r="G101" s="46" t="inlineStr"/>
@@ -14990,11 +15002,11 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="N101" s="48" t="n">
-        <v>46323.51385416667</v>
+      <c r="N101" s="53" t="n">
+        <v>46324.52037037037</v>
       </c>
       <c r="O101" s="46" t="n"/>
-      <c r="P101" s="48" t="n">
+      <c r="P101" s="53" t="n">
         <v>46323.51385416667</v>
       </c>
       <c r="Q101" s="46" t="inlineStr"/>
@@ -15016,10 +15028,10 @@
         </is>
       </c>
       <c r="D102" s="49" t="inlineStr"/>
-      <c r="E102" s="50" t="n">
+      <c r="E102" s="54" t="n">
         <v>46297</v>
       </c>
-      <c r="F102" s="50" t="n">
+      <c r="F102" s="54" t="n">
         <v>46297</v>
       </c>
       <c r="G102" s="49" t="inlineStr"/>
@@ -15043,11 +15055,11 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="N102" s="51" t="n">
-        <v>46323.51385416667</v>
+      <c r="N102" s="55" t="n">
+        <v>46324.52037037037</v>
       </c>
       <c r="O102" s="49" t="n"/>
-      <c r="P102" s="51" t="n">
+      <c r="P102" s="55" t="n">
         <v>46323.51385416667</v>
       </c>
       <c r="Q102" s="49" t="inlineStr">
@@ -15077,10 +15089,10 @@
           <t>Vacaciones🏖️</t>
         </is>
       </c>
-      <c r="E103" s="47" t="n">
+      <c r="E103" s="52" t="n">
         <v>46300</v>
       </c>
-      <c r="F103" s="47" t="n">
+      <c r="F103" s="52" t="n">
         <v>46300</v>
       </c>
       <c r="G103" s="46" t="inlineStr"/>
@@ -15104,11 +15116,11 @@
           <t>SI</t>
         </is>
       </c>
-      <c r="N103" s="48" t="n">
-        <v>46323.51385416667</v>
+      <c r="N103" s="53" t="n">
+        <v>46324.52037037037</v>
       </c>
       <c r="O103" s="46" t="n"/>
-      <c r="P103" s="48" t="n">
+      <c r="P103" s="53" t="n">
         <v>46323.51385416667</v>
       </c>
       <c r="Q103" s="46" t="inlineStr"/>
@@ -15134,10 +15146,10 @@
           <t>Vacaciones🏖️</t>
         </is>
       </c>
-      <c r="E104" s="47" t="n">
+      <c r="E104" s="52" t="n">
         <v>46377</v>
       </c>
-      <c r="F104" s="47" t="n">
+      <c r="F104" s="52" t="n">
         <v>46379</v>
       </c>
       <c r="G104" s="46" t="inlineStr"/>
@@ -15165,11 +15177,11 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="N104" s="48" t="n">
-        <v>46323.51385416667</v>
+      <c r="N104" s="53" t="n">
+        <v>46324.52037037037</v>
       </c>
       <c r="O104" s="46" t="n"/>
-      <c r="P104" s="48" t="n">
+      <c r="P104" s="53" t="n">
         <v>46323.51385416667</v>
       </c>
       <c r="Q104" s="46" t="inlineStr"/>
@@ -15195,10 +15207,10 @@
           <t>Ausencia</t>
         </is>
       </c>
-      <c r="E105" s="47" t="n">
+      <c r="E105" s="52" t="n">
         <v>46302</v>
       </c>
-      <c r="F105" s="47" t="n">
+      <c r="F105" s="52" t="n">
         <v>46302</v>
       </c>
       <c r="G105" s="46" t="inlineStr"/>
@@ -15222,11 +15234,11 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="N105" s="48" t="n">
-        <v>46323.51385416667</v>
+      <c r="N105" s="53" t="n">
+        <v>46324.52037037037</v>
       </c>
       <c r="O105" s="46" t="n"/>
-      <c r="P105" s="48" t="n">
+      <c r="P105" s="53" t="n">
         <v>46323.51385416667</v>
       </c>
       <c r="Q105" s="46" t="inlineStr"/>
@@ -15252,10 +15264,10 @@
           <t>Vacaciones🏖️</t>
         </is>
       </c>
-      <c r="E106" s="47" t="n">
+      <c r="E106" s="52" t="n">
         <v>46308</v>
       </c>
-      <c r="F106" s="47" t="n">
+      <c r="F106" s="52" t="n">
         <v>46308</v>
       </c>
       <c r="G106" s="46" t="inlineStr"/>
@@ -15283,11 +15295,11 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="N106" s="48" t="n">
-        <v>46323.51385416667</v>
+      <c r="N106" s="53" t="n">
+        <v>46324.52037037037</v>
       </c>
       <c r="O106" s="46" t="n"/>
-      <c r="P106" s="48" t="n">
+      <c r="P106" s="53" t="n">
         <v>46323.51385416667</v>
       </c>
       <c r="Q106" s="46" t="inlineStr"/>
@@ -15313,10 +15325,10 @@
           <t>Ausencia</t>
         </is>
       </c>
-      <c r="E107" s="47" t="n">
+      <c r="E107" s="52" t="n">
         <v>46304</v>
       </c>
-      <c r="F107" s="47" t="n">
+      <c r="F107" s="52" t="n">
         <v>46304</v>
       </c>
       <c r="G107" s="46" t="inlineStr"/>
@@ -15340,11 +15352,11 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="N107" s="48" t="n">
-        <v>46323.51385416667</v>
+      <c r="N107" s="53" t="n">
+        <v>46324.52037037037</v>
       </c>
       <c r="O107" s="46" t="n"/>
-      <c r="P107" s="48" t="n">
+      <c r="P107" s="53" t="n">
         <v>46323.51385416667</v>
       </c>
       <c r="Q107" s="46" t="inlineStr"/>
@@ -15370,10 +15382,10 @@
           <t>Vacaciones🏖️</t>
         </is>
       </c>
-      <c r="E108" s="47" t="n">
+      <c r="E108" s="52" t="n">
         <v>46317</v>
       </c>
-      <c r="F108" s="47" t="n">
+      <c r="F108" s="52" t="n">
         <v>46317</v>
       </c>
       <c r="G108" s="46" t="inlineStr"/>
@@ -15401,11 +15413,11 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="N108" s="48" t="n">
-        <v>46323.51385416667</v>
+      <c r="N108" s="53" t="n">
+        <v>46324.52037037037</v>
       </c>
       <c r="O108" s="46" t="n"/>
-      <c r="P108" s="48" t="n">
+      <c r="P108" s="53" t="n">
         <v>46323.51385416667</v>
       </c>
       <c r="Q108" s="46" t="inlineStr"/>
@@ -15431,10 +15443,10 @@
           <t>Ausencia</t>
         </is>
       </c>
-      <c r="E109" s="47" t="n">
+      <c r="E109" s="52" t="n">
         <v>46345</v>
       </c>
-      <c r="F109" s="47" t="n">
+      <c r="F109" s="52" t="n">
         <v>46345</v>
       </c>
       <c r="G109" s="46" t="inlineStr">
@@ -15470,11 +15482,11 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="N109" s="48" t="n">
-        <v>46323.51385416667</v>
+      <c r="N109" s="53" t="n">
+        <v>46324.52037037037</v>
       </c>
       <c r="O109" s="46" t="n"/>
-      <c r="P109" s="48" t="n">
+      <c r="P109" s="53" t="n">
         <v>46323.51385416667</v>
       </c>
       <c r="Q109" s="46" t="inlineStr"/>
@@ -15500,10 +15512,10 @@
           <t>Vacaciones🏖️</t>
         </is>
       </c>
-      <c r="E110" s="47" t="n">
+      <c r="E110" s="52" t="n">
         <v>46365</v>
       </c>
-      <c r="F110" s="47" t="n">
+      <c r="F110" s="52" t="n">
         <v>46367</v>
       </c>
       <c r="G110" s="46" t="inlineStr"/>
@@ -15531,11 +15543,11 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="N110" s="48" t="n">
-        <v>46323.51385416667</v>
+      <c r="N110" s="53" t="n">
+        <v>46324.52037037037</v>
       </c>
       <c r="O110" s="46" t="n"/>
-      <c r="P110" s="48" t="n">
+      <c r="P110" s="53" t="n">
         <v>46323.51385416667</v>
       </c>
       <c r="Q110" s="46" t="inlineStr"/>
@@ -15561,10 +15573,10 @@
           <t>Vacaciones🏖️</t>
         </is>
       </c>
-      <c r="E111" s="47" t="n">
+      <c r="E111" s="52" t="n">
         <v>46379</v>
       </c>
-      <c r="F111" s="47" t="n">
+      <c r="F111" s="52" t="n">
         <v>46394</v>
       </c>
       <c r="G111" s="46" t="inlineStr"/>
@@ -15592,11 +15604,11 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="N111" s="48" t="n">
-        <v>46323.51385416667</v>
+      <c r="N111" s="53" t="n">
+        <v>46324.52037037037</v>
       </c>
       <c r="O111" s="46" t="n"/>
-      <c r="P111" s="48" t="n">
+      <c r="P111" s="53" t="n">
         <v>46323.51385416667</v>
       </c>
       <c r="Q111" s="46" t="inlineStr"/>
@@ -15622,10 +15634,10 @@
           <t>Vacaciones🏖️</t>
         </is>
       </c>
-      <c r="E112" s="47" t="n">
+      <c r="E112" s="52" t="n">
         <v>46318</v>
       </c>
-      <c r="F112" s="47" t="n">
+      <c r="F112" s="52" t="n">
         <v>46319</v>
       </c>
       <c r="G112" s="46" t="inlineStr"/>
@@ -15653,11 +15665,11 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="N112" s="48" t="n">
-        <v>46323.51385416667</v>
+      <c r="N112" s="53" t="n">
+        <v>46324.52037037037</v>
       </c>
       <c r="O112" s="46" t="n"/>
-      <c r="P112" s="48" t="n">
+      <c r="P112" s="53" t="n">
         <v>46323.51385416667</v>
       </c>
       <c r="Q112" s="46" t="inlineStr"/>
@@ -15683,10 +15695,10 @@
           <t>Vacaciones🏖️</t>
         </is>
       </c>
-      <c r="E113" s="47" t="n">
+      <c r="E113" s="52" t="n">
         <v>46353</v>
       </c>
-      <c r="F113" s="47" t="n">
+      <c r="F113" s="52" t="n">
         <v>46353</v>
       </c>
       <c r="G113" s="46" t="inlineStr"/>
@@ -15714,11 +15726,11 @@
           <t>SI</t>
         </is>
       </c>
-      <c r="N113" s="48" t="n">
-        <v>46323.51385416667</v>
+      <c r="N113" s="53" t="n">
+        <v>46324.52037037037</v>
       </c>
       <c r="O113" s="46" t="n"/>
-      <c r="P113" s="48" t="n">
+      <c r="P113" s="53" t="n">
         <v>46323.51385416667</v>
       </c>
       <c r="Q113" s="46" t="inlineStr"/>
@@ -15744,10 +15756,10 @@
           <t>Vacaciones🏖️</t>
         </is>
       </c>
-      <c r="E114" s="47" t="n">
+      <c r="E114" s="52" t="n">
         <v>46324</v>
       </c>
-      <c r="F114" s="47" t="n">
+      <c r="F114" s="52" t="n">
         <v>46324</v>
       </c>
       <c r="G114" s="46" t="inlineStr"/>
@@ -15775,14 +15787,75 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="N114" s="48" t="n">
+      <c r="N114" s="53" t="n">
+        <v>46324.52037037037</v>
+      </c>
+      <c r="O114" s="46" t="n"/>
+      <c r="P114" s="53" t="n">
         <v>46323.51385416667</v>
       </c>
-      <c r="O114" s="46" t="n"/>
-      <c r="P114" s="48" t="n">
-        <v>46323.51385416667</v>
-      </c>
       <c r="Q114" s="46" t="inlineStr"/>
+    </row>
+    <row r="115">
+      <c r="A115" s="46" t="inlineStr">
+        <is>
+          <t>23652108</t>
+        </is>
+      </c>
+      <c r="B115" s="46" t="inlineStr">
+        <is>
+          <t>Sofía</t>
+        </is>
+      </c>
+      <c r="C115" s="46" t="inlineStr">
+        <is>
+          <t>SOFIA MEDIALDEA CONTRERAS</t>
+        </is>
+      </c>
+      <c r="D115" s="46" t="inlineStr">
+        <is>
+          <t>Vacaciones🏖️</t>
+        </is>
+      </c>
+      <c r="E115" s="52" t="n">
+        <v>46339</v>
+      </c>
+      <c r="F115" s="52" t="n">
+        <v>46350</v>
+      </c>
+      <c r="G115" s="46" t="inlineStr"/>
+      <c r="H115" s="46" t="inlineStr"/>
+      <c r="I115" s="46" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="J115" s="46" t="inlineStr">
+        <is>
+          <t>9 NOV, 16 NOV, 23 NOV</t>
+        </is>
+      </c>
+      <c r="K115" s="46" t="n">
+        <v>3</v>
+      </c>
+      <c r="L115" s="46" t="inlineStr">
+        <is>
+          <t>CONFIRMADA</t>
+        </is>
+      </c>
+      <c r="M115" s="46" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="N115" s="53" t="n">
+        <v>46324.52037037037</v>
+      </c>
+      <c r="O115" s="46" t="n"/>
+      <c r="P115" s="53" t="n">
+        <v>46324.52037037037</v>
+      </c>
+      <c r="Q115" s="46" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
sync: ausencias Bizneo 2026-10-30 12:20 UTC
</commit_message>
<xml_diff>
--- a/PM_ESTUDIO_MASTER_COMPLETO.xlsx
+++ b/PM_ESTUDIO_MASTER_COMPLETO.xlsx
@@ -24,11 +24,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="4">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="DD/MM/YYYY"/>
     <numFmt numFmtId="165" formatCode="DD/MM/YYYY HH:MM"/>
-    <numFmt numFmtId="166" formatCode="yyyy-mm-dd"/>
-    <numFmt numFmtId="167" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
   <fonts count="19">
     <font>
@@ -9308,7 +9306,7 @@
         </is>
       </c>
       <c r="N2" s="53" t="n">
-        <v>46324.52037037037</v>
+        <v>46325.51431712963</v>
       </c>
       <c r="O2" s="46" t="n"/>
       <c r="P2" s="53" t="n">
@@ -9365,7 +9363,7 @@
         </is>
       </c>
       <c r="N3" s="53" t="n">
-        <v>46324.52037037037</v>
+        <v>46325.51431712963</v>
       </c>
       <c r="O3" s="46" t="n"/>
       <c r="P3" s="53" t="n">
@@ -9422,7 +9420,7 @@
         </is>
       </c>
       <c r="N4" s="53" t="n">
-        <v>46324.52037037037</v>
+        <v>46325.51431712963</v>
       </c>
       <c r="O4" s="46" t="n"/>
       <c r="P4" s="53" t="n">
@@ -9479,7 +9477,7 @@
         </is>
       </c>
       <c r="N5" s="53" t="n">
-        <v>46324.52037037037</v>
+        <v>46325.51431712963</v>
       </c>
       <c r="O5" s="46" t="n"/>
       <c r="P5" s="53" t="n">
@@ -9536,7 +9534,7 @@
         </is>
       </c>
       <c r="N6" s="53" t="n">
-        <v>46324.52037037037</v>
+        <v>46325.51431712963</v>
       </c>
       <c r="O6" s="46" t="n"/>
       <c r="P6" s="53" t="n">
@@ -9593,7 +9591,7 @@
         </is>
       </c>
       <c r="N7" s="53" t="n">
-        <v>46324.52037037037</v>
+        <v>46325.51431712963</v>
       </c>
       <c r="O7" s="46" t="n"/>
       <c r="P7" s="53" t="n">
@@ -9650,7 +9648,7 @@
         </is>
       </c>
       <c r="N8" s="53" t="n">
-        <v>46324.52037037037</v>
+        <v>46325.51431712963</v>
       </c>
       <c r="O8" s="46" t="n"/>
       <c r="P8" s="53" t="n">
@@ -9707,7 +9705,7 @@
         </is>
       </c>
       <c r="N9" s="53" t="n">
-        <v>46324.52037037037</v>
+        <v>46325.51431712963</v>
       </c>
       <c r="O9" s="46" t="n"/>
       <c r="P9" s="53" t="n">
@@ -9764,7 +9762,7 @@
         </is>
       </c>
       <c r="N10" s="53" t="n">
-        <v>46324.52037037037</v>
+        <v>46325.51431712963</v>
       </c>
       <c r="O10" s="46" t="n"/>
       <c r="P10" s="53" t="n">
@@ -9821,7 +9819,7 @@
         </is>
       </c>
       <c r="N11" s="53" t="n">
-        <v>46324.52037037037</v>
+        <v>46325.51431712963</v>
       </c>
       <c r="O11" s="46" t="n"/>
       <c r="P11" s="53" t="n">
@@ -9878,7 +9876,7 @@
         </is>
       </c>
       <c r="N12" s="53" t="n">
-        <v>46324.52037037037</v>
+        <v>46325.51431712963</v>
       </c>
       <c r="O12" s="46" t="n"/>
       <c r="P12" s="53" t="n">
@@ -9935,7 +9933,7 @@
         </is>
       </c>
       <c r="N13" s="53" t="n">
-        <v>46324.52037037037</v>
+        <v>46325.51431712963</v>
       </c>
       <c r="O13" s="46" t="n"/>
       <c r="P13" s="53" t="n">
@@ -9988,7 +9986,7 @@
         </is>
       </c>
       <c r="N14" s="55" t="n">
-        <v>46324.52037037037</v>
+        <v>46325.51431712963</v>
       </c>
       <c r="O14" s="49" t="n"/>
       <c r="P14" s="55" t="n">
@@ -10049,7 +10047,7 @@
         </is>
       </c>
       <c r="N15" s="53" t="n">
-        <v>46324.52037037037</v>
+        <v>46325.51431712963</v>
       </c>
       <c r="O15" s="46" t="n"/>
       <c r="P15" s="53" t="n">
@@ -10106,7 +10104,7 @@
         </is>
       </c>
       <c r="N16" s="53" t="n">
-        <v>46324.52037037037</v>
+        <v>46325.51431712963</v>
       </c>
       <c r="O16" s="46" t="n"/>
       <c r="P16" s="53" t="n">
@@ -10163,7 +10161,7 @@
         </is>
       </c>
       <c r="N17" s="53" t="n">
-        <v>46324.52037037037</v>
+        <v>46325.51431712963</v>
       </c>
       <c r="O17" s="46" t="n"/>
       <c r="P17" s="53" t="n">
@@ -10220,7 +10218,7 @@
         </is>
       </c>
       <c r="N18" s="53" t="n">
-        <v>46324.52037037037</v>
+        <v>46325.51431712963</v>
       </c>
       <c r="O18" s="46" t="n"/>
       <c r="P18" s="53" t="n">
@@ -10277,7 +10275,7 @@
         </is>
       </c>
       <c r="N19" s="53" t="n">
-        <v>46324.52037037037</v>
+        <v>46325.51431712963</v>
       </c>
       <c r="O19" s="46" t="n"/>
       <c r="P19" s="53" t="n">
@@ -10334,7 +10332,7 @@
         </is>
       </c>
       <c r="N20" s="53" t="n">
-        <v>46324.52037037037</v>
+        <v>46325.51431712963</v>
       </c>
       <c r="O20" s="46" t="n"/>
       <c r="P20" s="53" t="n">
@@ -10391,7 +10389,7 @@
         </is>
       </c>
       <c r="N21" s="53" t="n">
-        <v>46324.52037037037</v>
+        <v>46325.51431712963</v>
       </c>
       <c r="O21" s="46" t="n"/>
       <c r="P21" s="53" t="n">
@@ -10448,7 +10446,7 @@
         </is>
       </c>
       <c r="N22" s="53" t="n">
-        <v>46324.52037037037</v>
+        <v>46325.51431712963</v>
       </c>
       <c r="O22" s="46" t="n"/>
       <c r="P22" s="53" t="n">
@@ -10505,7 +10503,7 @@
         </is>
       </c>
       <c r="N23" s="53" t="n">
-        <v>46324.52037037037</v>
+        <v>46325.51431712963</v>
       </c>
       <c r="O23" s="46" t="n"/>
       <c r="P23" s="53" t="n">
@@ -10562,7 +10560,7 @@
         </is>
       </c>
       <c r="N24" s="53" t="n">
-        <v>46324.52037037037</v>
+        <v>46325.51431712963</v>
       </c>
       <c r="O24" s="46" t="n"/>
       <c r="P24" s="53" t="n">
@@ -10619,7 +10617,7 @@
         </is>
       </c>
       <c r="N25" s="53" t="n">
-        <v>46324.52037037037</v>
+        <v>46325.51431712963</v>
       </c>
       <c r="O25" s="46" t="n"/>
       <c r="P25" s="53" t="n">
@@ -10676,7 +10674,7 @@
         </is>
       </c>
       <c r="N26" s="53" t="n">
-        <v>46324.52037037037</v>
+        <v>46325.51431712963</v>
       </c>
       <c r="O26" s="46" t="n"/>
       <c r="P26" s="53" t="n">
@@ -10733,7 +10731,7 @@
         </is>
       </c>
       <c r="N27" s="53" t="n">
-        <v>46324.52037037037</v>
+        <v>46325.51431712963</v>
       </c>
       <c r="O27" s="46" t="n"/>
       <c r="P27" s="53" t="n">
@@ -10790,7 +10788,7 @@
         </is>
       </c>
       <c r="N28" s="53" t="n">
-        <v>46324.52037037037</v>
+        <v>46325.51431712963</v>
       </c>
       <c r="O28" s="46" t="n"/>
       <c r="P28" s="53" t="n">
@@ -10847,7 +10845,7 @@
         </is>
       </c>
       <c r="N29" s="53" t="n">
-        <v>46324.52037037037</v>
+        <v>46325.51431712963</v>
       </c>
       <c r="O29" s="46" t="n"/>
       <c r="P29" s="53" t="n">
@@ -10904,7 +10902,7 @@
         </is>
       </c>
       <c r="N30" s="53" t="n">
-        <v>46324.52037037037</v>
+        <v>46325.51431712963</v>
       </c>
       <c r="O30" s="46" t="n"/>
       <c r="P30" s="53" t="n">
@@ -10961,7 +10959,7 @@
         </is>
       </c>
       <c r="N31" s="53" t="n">
-        <v>46324.52037037037</v>
+        <v>46325.51431712963</v>
       </c>
       <c r="O31" s="46" t="n"/>
       <c r="P31" s="53" t="n">
@@ -11018,7 +11016,7 @@
         </is>
       </c>
       <c r="N32" s="53" t="n">
-        <v>46324.52037037037</v>
+        <v>46325.51431712963</v>
       </c>
       <c r="O32" s="46" t="n"/>
       <c r="P32" s="53" t="n">
@@ -11075,7 +11073,7 @@
         </is>
       </c>
       <c r="N33" s="53" t="n">
-        <v>46324.52037037037</v>
+        <v>46325.51431712963</v>
       </c>
       <c r="O33" s="46" t="n"/>
       <c r="P33" s="53" t="n">
@@ -11132,7 +11130,7 @@
         </is>
       </c>
       <c r="N34" s="53" t="n">
-        <v>46324.52037037037</v>
+        <v>46325.51431712963</v>
       </c>
       <c r="O34" s="46" t="n"/>
       <c r="P34" s="53" t="n">
@@ -11189,7 +11187,7 @@
         </is>
       </c>
       <c r="N35" s="53" t="n">
-        <v>46324.52037037037</v>
+        <v>46325.51431712963</v>
       </c>
       <c r="O35" s="46" t="n"/>
       <c r="P35" s="53" t="n">
@@ -11246,7 +11244,7 @@
         </is>
       </c>
       <c r="N36" s="53" t="n">
-        <v>46324.52037037037</v>
+        <v>46325.51431712963</v>
       </c>
       <c r="O36" s="46" t="n"/>
       <c r="P36" s="53" t="n">
@@ -11303,7 +11301,7 @@
         </is>
       </c>
       <c r="N37" s="53" t="n">
-        <v>46324.52037037037</v>
+        <v>46325.51431712963</v>
       </c>
       <c r="O37" s="46" t="n"/>
       <c r="P37" s="53" t="n">
@@ -11360,7 +11358,7 @@
         </is>
       </c>
       <c r="N38" s="53" t="n">
-        <v>46324.52037037037</v>
+        <v>46325.51431712963</v>
       </c>
       <c r="O38" s="46" t="n"/>
       <c r="P38" s="53" t="n">
@@ -11417,7 +11415,7 @@
         </is>
       </c>
       <c r="N39" s="53" t="n">
-        <v>46324.52037037037</v>
+        <v>46325.51431712963</v>
       </c>
       <c r="O39" s="46" t="n"/>
       <c r="P39" s="53" t="n">
@@ -11474,7 +11472,7 @@
         </is>
       </c>
       <c r="N40" s="53" t="n">
-        <v>46324.52037037037</v>
+        <v>46325.51431712963</v>
       </c>
       <c r="O40" s="46" t="n"/>
       <c r="P40" s="53" t="n">
@@ -11531,7 +11529,7 @@
         </is>
       </c>
       <c r="N41" s="53" t="n">
-        <v>46324.52037037037</v>
+        <v>46325.51431712963</v>
       </c>
       <c r="O41" s="46" t="n"/>
       <c r="P41" s="53" t="n">
@@ -11588,7 +11586,7 @@
         </is>
       </c>
       <c r="N42" s="53" t="n">
-        <v>46324.52037037037</v>
+        <v>46325.51431712963</v>
       </c>
       <c r="O42" s="46" t="n"/>
       <c r="P42" s="53" t="n">
@@ -11645,7 +11643,7 @@
         </is>
       </c>
       <c r="N43" s="53" t="n">
-        <v>46324.52037037037</v>
+        <v>46325.51431712963</v>
       </c>
       <c r="O43" s="46" t="n"/>
       <c r="P43" s="53" t="n">
@@ -11702,7 +11700,7 @@
         </is>
       </c>
       <c r="N44" s="53" t="n">
-        <v>46324.52037037037</v>
+        <v>46325.51431712963</v>
       </c>
       <c r="O44" s="46" t="n"/>
       <c r="P44" s="53" t="n">
@@ -11759,7 +11757,7 @@
         </is>
       </c>
       <c r="N45" s="53" t="n">
-        <v>46324.52037037037</v>
+        <v>46325.51431712963</v>
       </c>
       <c r="O45" s="46" t="n"/>
       <c r="P45" s="53" t="n">
@@ -11816,7 +11814,7 @@
         </is>
       </c>
       <c r="N46" s="53" t="n">
-        <v>46324.52037037037</v>
+        <v>46325.51431712963</v>
       </c>
       <c r="O46" s="46" t="n"/>
       <c r="P46" s="53" t="n">
@@ -11873,7 +11871,7 @@
         </is>
       </c>
       <c r="N47" s="53" t="n">
-        <v>46324.52037037037</v>
+        <v>46325.51431712963</v>
       </c>
       <c r="O47" s="46" t="n"/>
       <c r="P47" s="53" t="n">
@@ -11930,7 +11928,7 @@
         </is>
       </c>
       <c r="N48" s="53" t="n">
-        <v>46324.52037037037</v>
+        <v>46325.51431712963</v>
       </c>
       <c r="O48" s="46" t="n"/>
       <c r="P48" s="53" t="n">
@@ -11987,7 +11985,7 @@
         </is>
       </c>
       <c r="N49" s="53" t="n">
-        <v>46324.52037037037</v>
+        <v>46325.51431712963</v>
       </c>
       <c r="O49" s="46" t="n"/>
       <c r="P49" s="53" t="n">
@@ -12040,7 +12038,7 @@
         </is>
       </c>
       <c r="N50" s="55" t="n">
-        <v>46324.52037037037</v>
+        <v>46325.51431712963</v>
       </c>
       <c r="O50" s="49" t="n"/>
       <c r="P50" s="55" t="n">
@@ -12097,7 +12095,7 @@
         </is>
       </c>
       <c r="N51" s="55" t="n">
-        <v>46324.52037037037</v>
+        <v>46325.51431712963</v>
       </c>
       <c r="O51" s="49" t="n"/>
       <c r="P51" s="55" t="n">
@@ -12158,7 +12156,7 @@
         </is>
       </c>
       <c r="N52" s="53" t="n">
-        <v>46324.52037037037</v>
+        <v>46325.51431712963</v>
       </c>
       <c r="O52" s="46" t="n"/>
       <c r="P52" s="53" t="n">
@@ -12215,7 +12213,7 @@
         </is>
       </c>
       <c r="N53" s="53" t="n">
-        <v>46324.52037037037</v>
+        <v>46325.51431712963</v>
       </c>
       <c r="O53" s="46" t="n"/>
       <c r="P53" s="53" t="n">
@@ -12268,7 +12266,7 @@
         </is>
       </c>
       <c r="N54" s="55" t="n">
-        <v>46324.52037037037</v>
+        <v>46325.51431712963</v>
       </c>
       <c r="O54" s="49" t="n"/>
       <c r="P54" s="55" t="n">
@@ -12329,7 +12327,7 @@
         </is>
       </c>
       <c r="N55" s="53" t="n">
-        <v>46324.52037037037</v>
+        <v>46325.51431712963</v>
       </c>
       <c r="O55" s="46" t="n"/>
       <c r="P55" s="53" t="n">
@@ -12386,7 +12384,7 @@
         </is>
       </c>
       <c r="N56" s="53" t="n">
-        <v>46324.52037037037</v>
+        <v>46325.51431712963</v>
       </c>
       <c r="O56" s="46" t="n"/>
       <c r="P56" s="53" t="n">
@@ -12443,7 +12441,7 @@
         </is>
       </c>
       <c r="N57" s="53" t="n">
-        <v>46324.52037037037</v>
+        <v>46325.51431712963</v>
       </c>
       <c r="O57" s="46" t="n"/>
       <c r="P57" s="53" t="n">
@@ -12500,7 +12498,7 @@
         </is>
       </c>
       <c r="N58" s="53" t="n">
-        <v>46324.52037037037</v>
+        <v>46325.51431712963</v>
       </c>
       <c r="O58" s="46" t="n"/>
       <c r="P58" s="53" t="n">
@@ -12557,7 +12555,7 @@
         </is>
       </c>
       <c r="N59" s="53" t="n">
-        <v>46324.52037037037</v>
+        <v>46325.51431712963</v>
       </c>
       <c r="O59" s="46" t="n"/>
       <c r="P59" s="53" t="n">
@@ -12622,7 +12620,7 @@
         </is>
       </c>
       <c r="N60" s="53" t="n">
-        <v>46324.52037037037</v>
+        <v>46325.51431712963</v>
       </c>
       <c r="O60" s="46" t="n"/>
       <c r="P60" s="53" t="n">
@@ -12679,7 +12677,7 @@
         </is>
       </c>
       <c r="N61" s="53" t="n">
-        <v>46324.52037037037</v>
+        <v>46325.51431712963</v>
       </c>
       <c r="O61" s="46" t="n"/>
       <c r="P61" s="53" t="n">
@@ -12736,7 +12734,7 @@
         </is>
       </c>
       <c r="N62" s="55" t="n">
-        <v>46324.52037037037</v>
+        <v>46325.51431712963</v>
       </c>
       <c r="O62" s="49" t="n"/>
       <c r="P62" s="55" t="n">
@@ -12797,7 +12795,7 @@
         </is>
       </c>
       <c r="N63" s="55" t="n">
-        <v>46324.52037037037</v>
+        <v>46325.51431712963</v>
       </c>
       <c r="O63" s="49" t="n"/>
       <c r="P63" s="55" t="n">
@@ -12858,7 +12856,7 @@
         </is>
       </c>
       <c r="N64" s="53" t="n">
-        <v>46324.52037037037</v>
+        <v>46325.51431712963</v>
       </c>
       <c r="O64" s="46" t="n"/>
       <c r="P64" s="53" t="n">
@@ -12915,7 +12913,7 @@
         </is>
       </c>
       <c r="N65" s="53" t="n">
-        <v>46324.52037037037</v>
+        <v>46325.51431712963</v>
       </c>
       <c r="O65" s="46" t="n"/>
       <c r="P65" s="53" t="n">
@@ -12972,7 +12970,7 @@
         </is>
       </c>
       <c r="N66" s="53" t="n">
-        <v>46324.52037037037</v>
+        <v>46325.51431712963</v>
       </c>
       <c r="O66" s="46" t="n"/>
       <c r="P66" s="53" t="n">
@@ -13029,7 +13027,7 @@
         </is>
       </c>
       <c r="N67" s="53" t="n">
-        <v>46324.52037037037</v>
+        <v>46325.51431712963</v>
       </c>
       <c r="O67" s="46" t="n"/>
       <c r="P67" s="53" t="n">
@@ -13086,7 +13084,7 @@
         </is>
       </c>
       <c r="N68" s="53" t="n">
-        <v>46324.52037037037</v>
+        <v>46325.51431712963</v>
       </c>
       <c r="O68" s="46" t="n"/>
       <c r="P68" s="53" t="n">
@@ -13143,7 +13141,7 @@
         </is>
       </c>
       <c r="N69" s="53" t="n">
-        <v>46324.52037037037</v>
+        <v>46325.51431712963</v>
       </c>
       <c r="O69" s="46" t="n"/>
       <c r="P69" s="53" t="n">
@@ -13200,7 +13198,7 @@
         </is>
       </c>
       <c r="N70" s="55" t="n">
-        <v>46324.52037037037</v>
+        <v>46325.51431712963</v>
       </c>
       <c r="O70" s="49" t="n"/>
       <c r="P70" s="55" t="n">
@@ -13261,7 +13259,7 @@
         </is>
       </c>
       <c r="N71" s="53" t="n">
-        <v>46324.52037037037</v>
+        <v>46325.51431712963</v>
       </c>
       <c r="O71" s="46" t="n"/>
       <c r="P71" s="53" t="n">
@@ -13318,7 +13316,7 @@
         </is>
       </c>
       <c r="N72" s="53" t="n">
-        <v>46324.52037037037</v>
+        <v>46325.51431712963</v>
       </c>
       <c r="O72" s="46" t="n"/>
       <c r="P72" s="53" t="n">
@@ -13375,7 +13373,7 @@
         </is>
       </c>
       <c r="N73" s="53" t="n">
-        <v>46324.52037037037</v>
+        <v>46325.51431712963</v>
       </c>
       <c r="O73" s="46" t="n"/>
       <c r="P73" s="53" t="n">
@@ -13432,7 +13430,7 @@
         </is>
       </c>
       <c r="N74" s="53" t="n">
-        <v>46324.52037037037</v>
+        <v>46325.51431712963</v>
       </c>
       <c r="O74" s="46" t="n"/>
       <c r="P74" s="53" t="n">
@@ -13489,7 +13487,7 @@
         </is>
       </c>
       <c r="N75" s="53" t="n">
-        <v>46324.52037037037</v>
+        <v>46325.51431712963</v>
       </c>
       <c r="O75" s="46" t="n"/>
       <c r="P75" s="53" t="n">
@@ -13546,7 +13544,7 @@
         </is>
       </c>
       <c r="N76" s="53" t="n">
-        <v>46324.52037037037</v>
+        <v>46325.51431712963</v>
       </c>
       <c r="O76" s="46" t="n"/>
       <c r="P76" s="53" t="n">
@@ -13603,7 +13601,7 @@
         </is>
       </c>
       <c r="N77" s="53" t="n">
-        <v>46324.52037037037</v>
+        <v>46325.51431712963</v>
       </c>
       <c r="O77" s="46" t="n"/>
       <c r="P77" s="53" t="n">
@@ -13660,7 +13658,7 @@
         </is>
       </c>
       <c r="N78" s="53" t="n">
-        <v>46324.52037037037</v>
+        <v>46325.51431712963</v>
       </c>
       <c r="O78" s="46" t="n"/>
       <c r="P78" s="53" t="n">
@@ -13717,7 +13715,7 @@
         </is>
       </c>
       <c r="N79" s="53" t="n">
-        <v>46324.52037037037</v>
+        <v>46325.51431712963</v>
       </c>
       <c r="O79" s="46" t="n"/>
       <c r="P79" s="53" t="n">
@@ -13774,7 +13772,7 @@
         </is>
       </c>
       <c r="N80" s="53" t="n">
-        <v>46324.52037037037</v>
+        <v>46325.51431712963</v>
       </c>
       <c r="O80" s="46" t="n"/>
       <c r="P80" s="53" t="n">
@@ -13831,7 +13829,7 @@
         </is>
       </c>
       <c r="N81" s="53" t="n">
-        <v>46324.52037037037</v>
+        <v>46325.51431712963</v>
       </c>
       <c r="O81" s="46" t="n"/>
       <c r="P81" s="53" t="n">
@@ -13888,7 +13886,7 @@
         </is>
       </c>
       <c r="N82" s="53" t="n">
-        <v>46324.52037037037</v>
+        <v>46325.51431712963</v>
       </c>
       <c r="O82" s="46" t="n"/>
       <c r="P82" s="53" t="n">
@@ -13945,7 +13943,7 @@
         </is>
       </c>
       <c r="N83" s="53" t="n">
-        <v>46324.52037037037</v>
+        <v>46325.51431712963</v>
       </c>
       <c r="O83" s="46" t="n"/>
       <c r="P83" s="53" t="n">
@@ -14002,7 +14000,7 @@
         </is>
       </c>
       <c r="N84" s="53" t="n">
-        <v>46324.52037037037</v>
+        <v>46325.51431712963</v>
       </c>
       <c r="O84" s="46" t="n"/>
       <c r="P84" s="53" t="n">
@@ -14059,7 +14057,7 @@
         </is>
       </c>
       <c r="N85" s="53" t="n">
-        <v>46324.52037037037</v>
+        <v>46325.51431712963</v>
       </c>
       <c r="O85" s="46" t="n"/>
       <c r="P85" s="53" t="n">
@@ -14116,7 +14114,7 @@
         </is>
       </c>
       <c r="N86" s="53" t="n">
-        <v>46324.52037037037</v>
+        <v>46325.51431712963</v>
       </c>
       <c r="O86" s="46" t="n"/>
       <c r="P86" s="53" t="n">
@@ -14173,7 +14171,7 @@
         </is>
       </c>
       <c r="N87" s="53" t="n">
-        <v>46324.52037037037</v>
+        <v>46325.51431712963</v>
       </c>
       <c r="O87" s="46" t="n"/>
       <c r="P87" s="53" t="n">
@@ -14230,7 +14228,7 @@
         </is>
       </c>
       <c r="N88" s="53" t="n">
-        <v>46324.52037037037</v>
+        <v>46325.51431712963</v>
       </c>
       <c r="O88" s="46" t="n"/>
       <c r="P88" s="53" t="n">
@@ -14295,7 +14293,7 @@
         </is>
       </c>
       <c r="N89" s="53" t="n">
-        <v>46324.52037037037</v>
+        <v>46325.51431712963</v>
       </c>
       <c r="O89" s="46" t="n"/>
       <c r="P89" s="53" t="n">
@@ -14352,7 +14350,7 @@
         </is>
       </c>
       <c r="N90" s="53" t="n">
-        <v>46324.52037037037</v>
+        <v>46325.51431712963</v>
       </c>
       <c r="O90" s="46" t="n"/>
       <c r="P90" s="53" t="n">
@@ -14409,7 +14407,7 @@
         </is>
       </c>
       <c r="N91" s="53" t="n">
-        <v>46324.52037037037</v>
+        <v>46325.51431712963</v>
       </c>
       <c r="O91" s="46" t="n"/>
       <c r="P91" s="53" t="n">
@@ -14466,7 +14464,7 @@
         </is>
       </c>
       <c r="N92" s="53" t="n">
-        <v>46324.52037037037</v>
+        <v>46325.51431712963</v>
       </c>
       <c r="O92" s="46" t="n"/>
       <c r="P92" s="53" t="n">
@@ -14523,7 +14521,7 @@
         </is>
       </c>
       <c r="N93" s="53" t="n">
-        <v>46324.52037037037</v>
+        <v>46325.51431712963</v>
       </c>
       <c r="O93" s="46" t="n"/>
       <c r="P93" s="53" t="n">
@@ -14580,7 +14578,7 @@
         </is>
       </c>
       <c r="N94" s="55" t="n">
-        <v>46324.52037037037</v>
+        <v>46325.51431712963</v>
       </c>
       <c r="O94" s="49" t="n"/>
       <c r="P94" s="55" t="n">
@@ -14641,7 +14639,7 @@
         </is>
       </c>
       <c r="N95" s="53" t="n">
-        <v>46324.52037037037</v>
+        <v>46325.51431712963</v>
       </c>
       <c r="O95" s="46" t="n"/>
       <c r="P95" s="53" t="n">
@@ -14702,7 +14700,7 @@
         </is>
       </c>
       <c r="N96" s="53" t="n">
-        <v>46324.52037037037</v>
+        <v>46325.51431712963</v>
       </c>
       <c r="O96" s="46" t="n"/>
       <c r="P96" s="53" t="n">
@@ -14759,7 +14757,7 @@
         </is>
       </c>
       <c r="N97" s="53" t="n">
-        <v>46324.52037037037</v>
+        <v>46325.51431712963</v>
       </c>
       <c r="O97" s="46" t="n"/>
       <c r="P97" s="53" t="n">
@@ -14828,7 +14826,7 @@
         </is>
       </c>
       <c r="N98" s="53" t="n">
-        <v>46324.52037037037</v>
+        <v>46325.51431712963</v>
       </c>
       <c r="O98" s="46" t="n"/>
       <c r="P98" s="53" t="n">
@@ -14885,7 +14883,7 @@
         </is>
       </c>
       <c r="N99" s="53" t="n">
-        <v>46324.52037037037</v>
+        <v>46325.51431712963</v>
       </c>
       <c r="O99" s="46" t="n"/>
       <c r="P99" s="53" t="n">
@@ -14946,7 +14944,7 @@
         </is>
       </c>
       <c r="N100" s="53" t="n">
-        <v>46324.52037037037</v>
+        <v>46325.51431712963</v>
       </c>
       <c r="O100" s="46" t="n"/>
       <c r="P100" s="53" t="n">
@@ -15003,7 +15001,7 @@
         </is>
       </c>
       <c r="N101" s="53" t="n">
-        <v>46324.52037037037</v>
+        <v>46325.51431712963</v>
       </c>
       <c r="O101" s="46" t="n"/>
       <c r="P101" s="53" t="n">
@@ -15056,7 +15054,7 @@
         </is>
       </c>
       <c r="N102" s="55" t="n">
-        <v>46324.52037037037</v>
+        <v>46325.51431712963</v>
       </c>
       <c r="O102" s="49" t="n"/>
       <c r="P102" s="55" t="n">
@@ -15117,7 +15115,7 @@
         </is>
       </c>
       <c r="N103" s="53" t="n">
-        <v>46324.52037037037</v>
+        <v>46325.51431712963</v>
       </c>
       <c r="O103" s="46" t="n"/>
       <c r="P103" s="53" t="n">
@@ -15178,7 +15176,7 @@
         </is>
       </c>
       <c r="N104" s="53" t="n">
-        <v>46324.52037037037</v>
+        <v>46325.51431712963</v>
       </c>
       <c r="O104" s="46" t="n"/>
       <c r="P104" s="53" t="n">
@@ -15235,7 +15233,7 @@
         </is>
       </c>
       <c r="N105" s="53" t="n">
-        <v>46324.52037037037</v>
+        <v>46325.51431712963</v>
       </c>
       <c r="O105" s="46" t="n"/>
       <c r="P105" s="53" t="n">
@@ -15296,7 +15294,7 @@
         </is>
       </c>
       <c r="N106" s="53" t="n">
-        <v>46324.52037037037</v>
+        <v>46325.51431712963</v>
       </c>
       <c r="O106" s="46" t="n"/>
       <c r="P106" s="53" t="n">
@@ -15353,7 +15351,7 @@
         </is>
       </c>
       <c r="N107" s="53" t="n">
-        <v>46324.52037037037</v>
+        <v>46325.51431712963</v>
       </c>
       <c r="O107" s="46" t="n"/>
       <c r="P107" s="53" t="n">
@@ -15414,7 +15412,7 @@
         </is>
       </c>
       <c r="N108" s="53" t="n">
-        <v>46324.52037037037</v>
+        <v>46325.51431712963</v>
       </c>
       <c r="O108" s="46" t="n"/>
       <c r="P108" s="53" t="n">
@@ -15483,7 +15481,7 @@
         </is>
       </c>
       <c r="N109" s="53" t="n">
-        <v>46324.52037037037</v>
+        <v>46325.51431712963</v>
       </c>
       <c r="O109" s="46" t="n"/>
       <c r="P109" s="53" t="n">
@@ -15544,7 +15542,7 @@
         </is>
       </c>
       <c r="N110" s="53" t="n">
-        <v>46324.52037037037</v>
+        <v>46325.51431712963</v>
       </c>
       <c r="O110" s="46" t="n"/>
       <c r="P110" s="53" t="n">
@@ -15605,7 +15603,7 @@
         </is>
       </c>
       <c r="N111" s="53" t="n">
-        <v>46324.52037037037</v>
+        <v>46325.51431712963</v>
       </c>
       <c r="O111" s="46" t="n"/>
       <c r="P111" s="53" t="n">
@@ -15666,7 +15664,7 @@
         </is>
       </c>
       <c r="N112" s="53" t="n">
-        <v>46324.52037037037</v>
+        <v>46325.51431712963</v>
       </c>
       <c r="O112" s="46" t="n"/>
       <c r="P112" s="53" t="n">
@@ -15727,7 +15725,7 @@
         </is>
       </c>
       <c r="N113" s="53" t="n">
-        <v>46324.52037037037</v>
+        <v>46325.51431712963</v>
       </c>
       <c r="O113" s="46" t="n"/>
       <c r="P113" s="53" t="n">
@@ -15788,7 +15786,7 @@
         </is>
       </c>
       <c r="N114" s="53" t="n">
-        <v>46324.52037037037</v>
+        <v>46325.51431712963</v>
       </c>
       <c r="O114" s="46" t="n"/>
       <c r="P114" s="53" t="n">
@@ -15849,7 +15847,7 @@
         </is>
       </c>
       <c r="N115" s="53" t="n">
-        <v>46324.52037037037</v>
+        <v>46325.51431712963</v>
       </c>
       <c r="O115" s="46" t="n"/>
       <c r="P115" s="53" t="n">

</xml_diff>

<commit_message>
sync: ausencias Bizneo 2026-10-31 11:51 UTC
</commit_message>
<xml_diff>
--- a/PM_ESTUDIO_MASTER_COMPLETO.xlsx
+++ b/PM_ESTUDIO_MASTER_COMPLETO.xlsx
@@ -9306,7 +9306,7 @@
         </is>
       </c>
       <c r="N2" s="53" t="n">
-        <v>46325.51431712963</v>
+        <v>46326.49396990741</v>
       </c>
       <c r="O2" s="46" t="n"/>
       <c r="P2" s="53" t="n">
@@ -9363,7 +9363,7 @@
         </is>
       </c>
       <c r="N3" s="53" t="n">
-        <v>46325.51431712963</v>
+        <v>46326.49396990741</v>
       </c>
       <c r="O3" s="46" t="n"/>
       <c r="P3" s="53" t="n">
@@ -9420,7 +9420,7 @@
         </is>
       </c>
       <c r="N4" s="53" t="n">
-        <v>46325.51431712963</v>
+        <v>46326.49396990741</v>
       </c>
       <c r="O4" s="46" t="n"/>
       <c r="P4" s="53" t="n">
@@ -9477,7 +9477,7 @@
         </is>
       </c>
       <c r="N5" s="53" t="n">
-        <v>46325.51431712963</v>
+        <v>46326.49396990741</v>
       </c>
       <c r="O5" s="46" t="n"/>
       <c r="P5" s="53" t="n">
@@ -9534,7 +9534,7 @@
         </is>
       </c>
       <c r="N6" s="53" t="n">
-        <v>46325.51431712963</v>
+        <v>46326.49396990741</v>
       </c>
       <c r="O6" s="46" t="n"/>
       <c r="P6" s="53" t="n">
@@ -9591,7 +9591,7 @@
         </is>
       </c>
       <c r="N7" s="53" t="n">
-        <v>46325.51431712963</v>
+        <v>46326.49396990741</v>
       </c>
       <c r="O7" s="46" t="n"/>
       <c r="P7" s="53" t="n">
@@ -9648,7 +9648,7 @@
         </is>
       </c>
       <c r="N8" s="53" t="n">
-        <v>46325.51431712963</v>
+        <v>46326.49396990741</v>
       </c>
       <c r="O8" s="46" t="n"/>
       <c r="P8" s="53" t="n">
@@ -9705,7 +9705,7 @@
         </is>
       </c>
       <c r="N9" s="53" t="n">
-        <v>46325.51431712963</v>
+        <v>46326.49396990741</v>
       </c>
       <c r="O9" s="46" t="n"/>
       <c r="P9" s="53" t="n">
@@ -9762,7 +9762,7 @@
         </is>
       </c>
       <c r="N10" s="53" t="n">
-        <v>46325.51431712963</v>
+        <v>46326.49396990741</v>
       </c>
       <c r="O10" s="46" t="n"/>
       <c r="P10" s="53" t="n">
@@ -9819,7 +9819,7 @@
         </is>
       </c>
       <c r="N11" s="53" t="n">
-        <v>46325.51431712963</v>
+        <v>46326.49396990741</v>
       </c>
       <c r="O11" s="46" t="n"/>
       <c r="P11" s="53" t="n">
@@ -9876,7 +9876,7 @@
         </is>
       </c>
       <c r="N12" s="53" t="n">
-        <v>46325.51431712963</v>
+        <v>46326.49396990741</v>
       </c>
       <c r="O12" s="46" t="n"/>
       <c r="P12" s="53" t="n">
@@ -9933,7 +9933,7 @@
         </is>
       </c>
       <c r="N13" s="53" t="n">
-        <v>46325.51431712963</v>
+        <v>46326.49396990741</v>
       </c>
       <c r="O13" s="46" t="n"/>
       <c r="P13" s="53" t="n">
@@ -9986,7 +9986,7 @@
         </is>
       </c>
       <c r="N14" s="55" t="n">
-        <v>46325.51431712963</v>
+        <v>46326.49396990741</v>
       </c>
       <c r="O14" s="49" t="n"/>
       <c r="P14" s="55" t="n">
@@ -10047,7 +10047,7 @@
         </is>
       </c>
       <c r="N15" s="53" t="n">
-        <v>46325.51431712963</v>
+        <v>46326.49396990741</v>
       </c>
       <c r="O15" s="46" t="n"/>
       <c r="P15" s="53" t="n">
@@ -10104,7 +10104,7 @@
         </is>
       </c>
       <c r="N16" s="53" t="n">
-        <v>46325.51431712963</v>
+        <v>46326.49396990741</v>
       </c>
       <c r="O16" s="46" t="n"/>
       <c r="P16" s="53" t="n">
@@ -10161,7 +10161,7 @@
         </is>
       </c>
       <c r="N17" s="53" t="n">
-        <v>46325.51431712963</v>
+        <v>46326.49396990741</v>
       </c>
       <c r="O17" s="46" t="n"/>
       <c r="P17" s="53" t="n">
@@ -10218,7 +10218,7 @@
         </is>
       </c>
       <c r="N18" s="53" t="n">
-        <v>46325.51431712963</v>
+        <v>46326.49396990741</v>
       </c>
       <c r="O18" s="46" t="n"/>
       <c r="P18" s="53" t="n">
@@ -10275,7 +10275,7 @@
         </is>
       </c>
       <c r="N19" s="53" t="n">
-        <v>46325.51431712963</v>
+        <v>46326.49396990741</v>
       </c>
       <c r="O19" s="46" t="n"/>
       <c r="P19" s="53" t="n">
@@ -10332,7 +10332,7 @@
         </is>
       </c>
       <c r="N20" s="53" t="n">
-        <v>46325.51431712963</v>
+        <v>46326.49396990741</v>
       </c>
       <c r="O20" s="46" t="n"/>
       <c r="P20" s="53" t="n">
@@ -10389,7 +10389,7 @@
         </is>
       </c>
       <c r="N21" s="53" t="n">
-        <v>46325.51431712963</v>
+        <v>46326.49396990741</v>
       </c>
       <c r="O21" s="46" t="n"/>
       <c r="P21" s="53" t="n">
@@ -10446,7 +10446,7 @@
         </is>
       </c>
       <c r="N22" s="53" t="n">
-        <v>46325.51431712963</v>
+        <v>46326.49396990741</v>
       </c>
       <c r="O22" s="46" t="n"/>
       <c r="P22" s="53" t="n">
@@ -10503,7 +10503,7 @@
         </is>
       </c>
       <c r="N23" s="53" t="n">
-        <v>46325.51431712963</v>
+        <v>46326.49396990741</v>
       </c>
       <c r="O23" s="46" t="n"/>
       <c r="P23" s="53" t="n">
@@ -10560,7 +10560,7 @@
         </is>
       </c>
       <c r="N24" s="53" t="n">
-        <v>46325.51431712963</v>
+        <v>46326.49396990741</v>
       </c>
       <c r="O24" s="46" t="n"/>
       <c r="P24" s="53" t="n">
@@ -10617,7 +10617,7 @@
         </is>
       </c>
       <c r="N25" s="53" t="n">
-        <v>46325.51431712963</v>
+        <v>46326.49396990741</v>
       </c>
       <c r="O25" s="46" t="n"/>
       <c r="P25" s="53" t="n">
@@ -10674,7 +10674,7 @@
         </is>
       </c>
       <c r="N26" s="53" t="n">
-        <v>46325.51431712963</v>
+        <v>46326.49396990741</v>
       </c>
       <c r="O26" s="46" t="n"/>
       <c r="P26" s="53" t="n">
@@ -10731,7 +10731,7 @@
         </is>
       </c>
       <c r="N27" s="53" t="n">
-        <v>46325.51431712963</v>
+        <v>46326.49396990741</v>
       </c>
       <c r="O27" s="46" t="n"/>
       <c r="P27" s="53" t="n">
@@ -10788,7 +10788,7 @@
         </is>
       </c>
       <c r="N28" s="53" t="n">
-        <v>46325.51431712963</v>
+        <v>46326.49396990741</v>
       </c>
       <c r="O28" s="46" t="n"/>
       <c r="P28" s="53" t="n">
@@ -10845,7 +10845,7 @@
         </is>
       </c>
       <c r="N29" s="53" t="n">
-        <v>46325.51431712963</v>
+        <v>46326.49396990741</v>
       </c>
       <c r="O29" s="46" t="n"/>
       <c r="P29" s="53" t="n">
@@ -10902,7 +10902,7 @@
         </is>
       </c>
       <c r="N30" s="53" t="n">
-        <v>46325.51431712963</v>
+        <v>46326.49396990741</v>
       </c>
       <c r="O30" s="46" t="n"/>
       <c r="P30" s="53" t="n">
@@ -10959,7 +10959,7 @@
         </is>
       </c>
       <c r="N31" s="53" t="n">
-        <v>46325.51431712963</v>
+        <v>46326.49396990741</v>
       </c>
       <c r="O31" s="46" t="n"/>
       <c r="P31" s="53" t="n">
@@ -11016,7 +11016,7 @@
         </is>
       </c>
       <c r="N32" s="53" t="n">
-        <v>46325.51431712963</v>
+        <v>46326.49396990741</v>
       </c>
       <c r="O32" s="46" t="n"/>
       <c r="P32" s="53" t="n">
@@ -11073,7 +11073,7 @@
         </is>
       </c>
       <c r="N33" s="53" t="n">
-        <v>46325.51431712963</v>
+        <v>46326.49396990741</v>
       </c>
       <c r="O33" s="46" t="n"/>
       <c r="P33" s="53" t="n">
@@ -11130,7 +11130,7 @@
         </is>
       </c>
       <c r="N34" s="53" t="n">
-        <v>46325.51431712963</v>
+        <v>46326.49396990741</v>
       </c>
       <c r="O34" s="46" t="n"/>
       <c r="P34" s="53" t="n">
@@ -11187,7 +11187,7 @@
         </is>
       </c>
       <c r="N35" s="53" t="n">
-        <v>46325.51431712963</v>
+        <v>46326.49396990741</v>
       </c>
       <c r="O35" s="46" t="n"/>
       <c r="P35" s="53" t="n">
@@ -11244,7 +11244,7 @@
         </is>
       </c>
       <c r="N36" s="53" t="n">
-        <v>46325.51431712963</v>
+        <v>46326.49396990741</v>
       </c>
       <c r="O36" s="46" t="n"/>
       <c r="P36" s="53" t="n">
@@ -11301,7 +11301,7 @@
         </is>
       </c>
       <c r="N37" s="53" t="n">
-        <v>46325.51431712963</v>
+        <v>46326.49396990741</v>
       </c>
       <c r="O37" s="46" t="n"/>
       <c r="P37" s="53" t="n">
@@ -11358,7 +11358,7 @@
         </is>
       </c>
       <c r="N38" s="53" t="n">
-        <v>46325.51431712963</v>
+        <v>46326.49396990741</v>
       </c>
       <c r="O38" s="46" t="n"/>
       <c r="P38" s="53" t="n">
@@ -11415,7 +11415,7 @@
         </is>
       </c>
       <c r="N39" s="53" t="n">
-        <v>46325.51431712963</v>
+        <v>46326.49396990741</v>
       </c>
       <c r="O39" s="46" t="n"/>
       <c r="P39" s="53" t="n">
@@ -11472,7 +11472,7 @@
         </is>
       </c>
       <c r="N40" s="53" t="n">
-        <v>46325.51431712963</v>
+        <v>46326.49396990741</v>
       </c>
       <c r="O40" s="46" t="n"/>
       <c r="P40" s="53" t="n">
@@ -11529,7 +11529,7 @@
         </is>
       </c>
       <c r="N41" s="53" t="n">
-        <v>46325.51431712963</v>
+        <v>46326.49396990741</v>
       </c>
       <c r="O41" s="46" t="n"/>
       <c r="P41" s="53" t="n">
@@ -11586,7 +11586,7 @@
         </is>
       </c>
       <c r="N42" s="53" t="n">
-        <v>46325.51431712963</v>
+        <v>46326.49396990741</v>
       </c>
       <c r="O42" s="46" t="n"/>
       <c r="P42" s="53" t="n">
@@ -11643,7 +11643,7 @@
         </is>
       </c>
       <c r="N43" s="53" t="n">
-        <v>46325.51431712963</v>
+        <v>46326.49396990741</v>
       </c>
       <c r="O43" s="46" t="n"/>
       <c r="P43" s="53" t="n">
@@ -11700,7 +11700,7 @@
         </is>
       </c>
       <c r="N44" s="53" t="n">
-        <v>46325.51431712963</v>
+        <v>46326.49396990741</v>
       </c>
       <c r="O44" s="46" t="n"/>
       <c r="P44" s="53" t="n">
@@ -11757,7 +11757,7 @@
         </is>
       </c>
       <c r="N45" s="53" t="n">
-        <v>46325.51431712963</v>
+        <v>46326.49396990741</v>
       </c>
       <c r="O45" s="46" t="n"/>
       <c r="P45" s="53" t="n">
@@ -11814,7 +11814,7 @@
         </is>
       </c>
       <c r="N46" s="53" t="n">
-        <v>46325.51431712963</v>
+        <v>46326.49396990741</v>
       </c>
       <c r="O46" s="46" t="n"/>
       <c r="P46" s="53" t="n">
@@ -11871,7 +11871,7 @@
         </is>
       </c>
       <c r="N47" s="53" t="n">
-        <v>46325.51431712963</v>
+        <v>46326.49396990741</v>
       </c>
       <c r="O47" s="46" t="n"/>
       <c r="P47" s="53" t="n">
@@ -11928,7 +11928,7 @@
         </is>
       </c>
       <c r="N48" s="53" t="n">
-        <v>46325.51431712963</v>
+        <v>46326.49396990741</v>
       </c>
       <c r="O48" s="46" t="n"/>
       <c r="P48" s="53" t="n">
@@ -11985,7 +11985,7 @@
         </is>
       </c>
       <c r="N49" s="53" t="n">
-        <v>46325.51431712963</v>
+        <v>46326.49396990741</v>
       </c>
       <c r="O49" s="46" t="n"/>
       <c r="P49" s="53" t="n">
@@ -12038,7 +12038,7 @@
         </is>
       </c>
       <c r="N50" s="55" t="n">
-        <v>46325.51431712963</v>
+        <v>46326.49396990741</v>
       </c>
       <c r="O50" s="49" t="n"/>
       <c r="P50" s="55" t="n">
@@ -12095,7 +12095,7 @@
         </is>
       </c>
       <c r="N51" s="55" t="n">
-        <v>46325.51431712963</v>
+        <v>46326.49396990741</v>
       </c>
       <c r="O51" s="49" t="n"/>
       <c r="P51" s="55" t="n">
@@ -12156,7 +12156,7 @@
         </is>
       </c>
       <c r="N52" s="53" t="n">
-        <v>46325.51431712963</v>
+        <v>46326.49396990741</v>
       </c>
       <c r="O52" s="46" t="n"/>
       <c r="P52" s="53" t="n">
@@ -12213,7 +12213,7 @@
         </is>
       </c>
       <c r="N53" s="53" t="n">
-        <v>46325.51431712963</v>
+        <v>46326.49396990741</v>
       </c>
       <c r="O53" s="46" t="n"/>
       <c r="P53" s="53" t="n">
@@ -12266,7 +12266,7 @@
         </is>
       </c>
       <c r="N54" s="55" t="n">
-        <v>46325.51431712963</v>
+        <v>46326.49396990741</v>
       </c>
       <c r="O54" s="49" t="n"/>
       <c r="P54" s="55" t="n">
@@ -12327,7 +12327,7 @@
         </is>
       </c>
       <c r="N55" s="53" t="n">
-        <v>46325.51431712963</v>
+        <v>46326.49396990741</v>
       </c>
       <c r="O55" s="46" t="n"/>
       <c r="P55" s="53" t="n">
@@ -12384,7 +12384,7 @@
         </is>
       </c>
       <c r="N56" s="53" t="n">
-        <v>46325.51431712963</v>
+        <v>46326.49396990741</v>
       </c>
       <c r="O56" s="46" t="n"/>
       <c r="P56" s="53" t="n">
@@ -12441,7 +12441,7 @@
         </is>
       </c>
       <c r="N57" s="53" t="n">
-        <v>46325.51431712963</v>
+        <v>46326.49396990741</v>
       </c>
       <c r="O57" s="46" t="n"/>
       <c r="P57" s="53" t="n">
@@ -12498,7 +12498,7 @@
         </is>
       </c>
       <c r="N58" s="53" t="n">
-        <v>46325.51431712963</v>
+        <v>46326.49396990741</v>
       </c>
       <c r="O58" s="46" t="n"/>
       <c r="P58" s="53" t="n">
@@ -12555,7 +12555,7 @@
         </is>
       </c>
       <c r="N59" s="53" t="n">
-        <v>46325.51431712963</v>
+        <v>46326.49396990741</v>
       </c>
       <c r="O59" s="46" t="n"/>
       <c r="P59" s="53" t="n">
@@ -12620,7 +12620,7 @@
         </is>
       </c>
       <c r="N60" s="53" t="n">
-        <v>46325.51431712963</v>
+        <v>46326.49396990741</v>
       </c>
       <c r="O60" s="46" t="n"/>
       <c r="P60" s="53" t="n">
@@ -12677,7 +12677,7 @@
         </is>
       </c>
       <c r="N61" s="53" t="n">
-        <v>46325.51431712963</v>
+        <v>46326.49396990741</v>
       </c>
       <c r="O61" s="46" t="n"/>
       <c r="P61" s="53" t="n">
@@ -12734,7 +12734,7 @@
         </is>
       </c>
       <c r="N62" s="55" t="n">
-        <v>46325.51431712963</v>
+        <v>46326.49396990741</v>
       </c>
       <c r="O62" s="49" t="n"/>
       <c r="P62" s="55" t="n">
@@ -12795,7 +12795,7 @@
         </is>
       </c>
       <c r="N63" s="55" t="n">
-        <v>46325.51431712963</v>
+        <v>46326.49396990741</v>
       </c>
       <c r="O63" s="49" t="n"/>
       <c r="P63" s="55" t="n">
@@ -12856,7 +12856,7 @@
         </is>
       </c>
       <c r="N64" s="53" t="n">
-        <v>46325.51431712963</v>
+        <v>46326.49396990741</v>
       </c>
       <c r="O64" s="46" t="n"/>
       <c r="P64" s="53" t="n">
@@ -12913,7 +12913,7 @@
         </is>
       </c>
       <c r="N65" s="53" t="n">
-        <v>46325.51431712963</v>
+        <v>46326.49396990741</v>
       </c>
       <c r="O65" s="46" t="n"/>
       <c r="P65" s="53" t="n">
@@ -12970,7 +12970,7 @@
         </is>
       </c>
       <c r="N66" s="53" t="n">
-        <v>46325.51431712963</v>
+        <v>46326.49396990741</v>
       </c>
       <c r="O66" s="46" t="n"/>
       <c r="P66" s="53" t="n">
@@ -13027,7 +13027,7 @@
         </is>
       </c>
       <c r="N67" s="53" t="n">
-        <v>46325.51431712963</v>
+        <v>46326.49396990741</v>
       </c>
       <c r="O67" s="46" t="n"/>
       <c r="P67" s="53" t="n">
@@ -13084,7 +13084,7 @@
         </is>
       </c>
       <c r="N68" s="53" t="n">
-        <v>46325.51431712963</v>
+        <v>46326.49396990741</v>
       </c>
       <c r="O68" s="46" t="n"/>
       <c r="P68" s="53" t="n">
@@ -13141,7 +13141,7 @@
         </is>
       </c>
       <c r="N69" s="53" t="n">
-        <v>46325.51431712963</v>
+        <v>46326.49396990741</v>
       </c>
       <c r="O69" s="46" t="n"/>
       <c r="P69" s="53" t="n">
@@ -13198,7 +13198,7 @@
         </is>
       </c>
       <c r="N70" s="55" t="n">
-        <v>46325.51431712963</v>
+        <v>46326.49396990741</v>
       </c>
       <c r="O70" s="49" t="n"/>
       <c r="P70" s="55" t="n">
@@ -13259,7 +13259,7 @@
         </is>
       </c>
       <c r="N71" s="53" t="n">
-        <v>46325.51431712963</v>
+        <v>46326.49396990741</v>
       </c>
       <c r="O71" s="46" t="n"/>
       <c r="P71" s="53" t="n">
@@ -13316,7 +13316,7 @@
         </is>
       </c>
       <c r="N72" s="53" t="n">
-        <v>46325.51431712963</v>
+        <v>46326.49396990741</v>
       </c>
       <c r="O72" s="46" t="n"/>
       <c r="P72" s="53" t="n">
@@ -13373,7 +13373,7 @@
         </is>
       </c>
       <c r="N73" s="53" t="n">
-        <v>46325.51431712963</v>
+        <v>46326.49396990741</v>
       </c>
       <c r="O73" s="46" t="n"/>
       <c r="P73" s="53" t="n">
@@ -13430,7 +13430,7 @@
         </is>
       </c>
       <c r="N74" s="53" t="n">
-        <v>46325.51431712963</v>
+        <v>46326.49396990741</v>
       </c>
       <c r="O74" s="46" t="n"/>
       <c r="P74" s="53" t="n">
@@ -13487,7 +13487,7 @@
         </is>
       </c>
       <c r="N75" s="53" t="n">
-        <v>46325.51431712963</v>
+        <v>46326.49396990741</v>
       </c>
       <c r="O75" s="46" t="n"/>
       <c r="P75" s="53" t="n">
@@ -13544,7 +13544,7 @@
         </is>
       </c>
       <c r="N76" s="53" t="n">
-        <v>46325.51431712963</v>
+        <v>46326.49396990741</v>
       </c>
       <c r="O76" s="46" t="n"/>
       <c r="P76" s="53" t="n">
@@ -13601,7 +13601,7 @@
         </is>
       </c>
       <c r="N77" s="53" t="n">
-        <v>46325.51431712963</v>
+        <v>46326.49396990741</v>
       </c>
       <c r="O77" s="46" t="n"/>
       <c r="P77" s="53" t="n">
@@ -13658,7 +13658,7 @@
         </is>
       </c>
       <c r="N78" s="53" t="n">
-        <v>46325.51431712963</v>
+        <v>46326.49396990741</v>
       </c>
       <c r="O78" s="46" t="n"/>
       <c r="P78" s="53" t="n">
@@ -13715,7 +13715,7 @@
         </is>
       </c>
       <c r="N79" s="53" t="n">
-        <v>46325.51431712963</v>
+        <v>46326.49396990741</v>
       </c>
       <c r="O79" s="46" t="n"/>
       <c r="P79" s="53" t="n">
@@ -13772,7 +13772,7 @@
         </is>
       </c>
       <c r="N80" s="53" t="n">
-        <v>46325.51431712963</v>
+        <v>46326.49396990741</v>
       </c>
       <c r="O80" s="46" t="n"/>
       <c r="P80" s="53" t="n">
@@ -13829,7 +13829,7 @@
         </is>
       </c>
       <c r="N81" s="53" t="n">
-        <v>46325.51431712963</v>
+        <v>46326.49396990741</v>
       </c>
       <c r="O81" s="46" t="n"/>
       <c r="P81" s="53" t="n">
@@ -13886,7 +13886,7 @@
         </is>
       </c>
       <c r="N82" s="53" t="n">
-        <v>46325.51431712963</v>
+        <v>46326.49396990741</v>
       </c>
       <c r="O82" s="46" t="n"/>
       <c r="P82" s="53" t="n">
@@ -13943,7 +13943,7 @@
         </is>
       </c>
       <c r="N83" s="53" t="n">
-        <v>46325.51431712963</v>
+        <v>46326.49396990741</v>
       </c>
       <c r="O83" s="46" t="n"/>
       <c r="P83" s="53" t="n">
@@ -14000,7 +14000,7 @@
         </is>
       </c>
       <c r="N84" s="53" t="n">
-        <v>46325.51431712963</v>
+        <v>46326.49396990741</v>
       </c>
       <c r="O84" s="46" t="n"/>
       <c r="P84" s="53" t="n">
@@ -14057,7 +14057,7 @@
         </is>
       </c>
       <c r="N85" s="53" t="n">
-        <v>46325.51431712963</v>
+        <v>46326.49396990741</v>
       </c>
       <c r="O85" s="46" t="n"/>
       <c r="P85" s="53" t="n">
@@ -14114,7 +14114,7 @@
         </is>
       </c>
       <c r="N86" s="53" t="n">
-        <v>46325.51431712963</v>
+        <v>46326.49396990741</v>
       </c>
       <c r="O86" s="46" t="n"/>
       <c r="P86" s="53" t="n">
@@ -14171,7 +14171,7 @@
         </is>
       </c>
       <c r="N87" s="53" t="n">
-        <v>46325.51431712963</v>
+        <v>46326.49396990741</v>
       </c>
       <c r="O87" s="46" t="n"/>
       <c r="P87" s="53" t="n">
@@ -14228,7 +14228,7 @@
         </is>
       </c>
       <c r="N88" s="53" t="n">
-        <v>46325.51431712963</v>
+        <v>46326.49396990741</v>
       </c>
       <c r="O88" s="46" t="n"/>
       <c r="P88" s="53" t="n">
@@ -14293,7 +14293,7 @@
         </is>
       </c>
       <c r="N89" s="53" t="n">
-        <v>46325.51431712963</v>
+        <v>46326.49396990741</v>
       </c>
       <c r="O89" s="46" t="n"/>
       <c r="P89" s="53" t="n">
@@ -14350,7 +14350,7 @@
         </is>
       </c>
       <c r="N90" s="53" t="n">
-        <v>46325.51431712963</v>
+        <v>46326.49396990741</v>
       </c>
       <c r="O90" s="46" t="n"/>
       <c r="P90" s="53" t="n">
@@ -14407,7 +14407,7 @@
         </is>
       </c>
       <c r="N91" s="53" t="n">
-        <v>46325.51431712963</v>
+        <v>46326.49396990741</v>
       </c>
       <c r="O91" s="46" t="n"/>
       <c r="P91" s="53" t="n">
@@ -14464,7 +14464,7 @@
         </is>
       </c>
       <c r="N92" s="53" t="n">
-        <v>46325.51431712963</v>
+        <v>46326.49396990741</v>
       </c>
       <c r="O92" s="46" t="n"/>
       <c r="P92" s="53" t="n">
@@ -14521,7 +14521,7 @@
         </is>
       </c>
       <c r="N93" s="53" t="n">
-        <v>46325.51431712963</v>
+        <v>46326.49396990741</v>
       </c>
       <c r="O93" s="46" t="n"/>
       <c r="P93" s="53" t="n">
@@ -14578,7 +14578,7 @@
         </is>
       </c>
       <c r="N94" s="55" t="n">
-        <v>46325.51431712963</v>
+        <v>46326.49396990741</v>
       </c>
       <c r="O94" s="49" t="n"/>
       <c r="P94" s="55" t="n">
@@ -14639,7 +14639,7 @@
         </is>
       </c>
       <c r="N95" s="53" t="n">
-        <v>46325.51431712963</v>
+        <v>46326.49396990741</v>
       </c>
       <c r="O95" s="46" t="n"/>
       <c r="P95" s="53" t="n">
@@ -14700,7 +14700,7 @@
         </is>
       </c>
       <c r="N96" s="53" t="n">
-        <v>46325.51431712963</v>
+        <v>46326.49396990741</v>
       </c>
       <c r="O96" s="46" t="n"/>
       <c r="P96" s="53" t="n">
@@ -14757,7 +14757,7 @@
         </is>
       </c>
       <c r="N97" s="53" t="n">
-        <v>46325.51431712963</v>
+        <v>46326.49396990741</v>
       </c>
       <c r="O97" s="46" t="n"/>
       <c r="P97" s="53" t="n">
@@ -14826,7 +14826,7 @@
         </is>
       </c>
       <c r="N98" s="53" t="n">
-        <v>46325.51431712963</v>
+        <v>46326.49396990741</v>
       </c>
       <c r="O98" s="46" t="n"/>
       <c r="P98" s="53" t="n">
@@ -14883,7 +14883,7 @@
         </is>
       </c>
       <c r="N99" s="53" t="n">
-        <v>46325.51431712963</v>
+        <v>46326.49396990741</v>
       </c>
       <c r="O99" s="46" t="n"/>
       <c r="P99" s="53" t="n">
@@ -14944,7 +14944,7 @@
         </is>
       </c>
       <c r="N100" s="53" t="n">
-        <v>46325.51431712963</v>
+        <v>46326.49396990741</v>
       </c>
       <c r="O100" s="46" t="n"/>
       <c r="P100" s="53" t="n">
@@ -15001,7 +15001,7 @@
         </is>
       </c>
       <c r="N101" s="53" t="n">
-        <v>46325.51431712963</v>
+        <v>46326.49396990741</v>
       </c>
       <c r="O101" s="46" t="n"/>
       <c r="P101" s="53" t="n">
@@ -15054,7 +15054,7 @@
         </is>
       </c>
       <c r="N102" s="55" t="n">
-        <v>46325.51431712963</v>
+        <v>46326.49396990741</v>
       </c>
       <c r="O102" s="49" t="n"/>
       <c r="P102" s="55" t="n">
@@ -15115,7 +15115,7 @@
         </is>
       </c>
       <c r="N103" s="53" t="n">
-        <v>46325.51431712963</v>
+        <v>46326.49396990741</v>
       </c>
       <c r="O103" s="46" t="n"/>
       <c r="P103" s="53" t="n">
@@ -15176,7 +15176,7 @@
         </is>
       </c>
       <c r="N104" s="53" t="n">
-        <v>46325.51431712963</v>
+        <v>46326.49396990741</v>
       </c>
       <c r="O104" s="46" t="n"/>
       <c r="P104" s="53" t="n">
@@ -15233,7 +15233,7 @@
         </is>
       </c>
       <c r="N105" s="53" t="n">
-        <v>46325.51431712963</v>
+        <v>46326.49396990741</v>
       </c>
       <c r="O105" s="46" t="n"/>
       <c r="P105" s="53" t="n">
@@ -15294,7 +15294,7 @@
         </is>
       </c>
       <c r="N106" s="53" t="n">
-        <v>46325.51431712963</v>
+        <v>46326.49396990741</v>
       </c>
       <c r="O106" s="46" t="n"/>
       <c r="P106" s="53" t="n">
@@ -15351,7 +15351,7 @@
         </is>
       </c>
       <c r="N107" s="53" t="n">
-        <v>46325.51431712963</v>
+        <v>46326.49396990741</v>
       </c>
       <c r="O107" s="46" t="n"/>
       <c r="P107" s="53" t="n">
@@ -15412,7 +15412,7 @@
         </is>
       </c>
       <c r="N108" s="53" t="n">
-        <v>46325.51431712963</v>
+        <v>46326.49396990741</v>
       </c>
       <c r="O108" s="46" t="n"/>
       <c r="P108" s="53" t="n">
@@ -15481,7 +15481,7 @@
         </is>
       </c>
       <c r="N109" s="53" t="n">
-        <v>46325.51431712963</v>
+        <v>46326.49396990741</v>
       </c>
       <c r="O109" s="46" t="n"/>
       <c r="P109" s="53" t="n">
@@ -15542,7 +15542,7 @@
         </is>
       </c>
       <c r="N110" s="53" t="n">
-        <v>46325.51431712963</v>
+        <v>46326.49396990741</v>
       </c>
       <c r="O110" s="46" t="n"/>
       <c r="P110" s="53" t="n">
@@ -15603,7 +15603,7 @@
         </is>
       </c>
       <c r="N111" s="53" t="n">
-        <v>46325.51431712963</v>
+        <v>46326.49396990741</v>
       </c>
       <c r="O111" s="46" t="n"/>
       <c r="P111" s="53" t="n">
@@ -15664,7 +15664,7 @@
         </is>
       </c>
       <c r="N112" s="53" t="n">
-        <v>46325.51431712963</v>
+        <v>46326.49396990741</v>
       </c>
       <c r="O112" s="46" t="n"/>
       <c r="P112" s="53" t="n">
@@ -15725,7 +15725,7 @@
         </is>
       </c>
       <c r="N113" s="53" t="n">
-        <v>46325.51431712963</v>
+        <v>46326.49396990741</v>
       </c>
       <c r="O113" s="46" t="n"/>
       <c r="P113" s="53" t="n">
@@ -15786,7 +15786,7 @@
         </is>
       </c>
       <c r="N114" s="53" t="n">
-        <v>46325.51431712963</v>
+        <v>46326.49396990741</v>
       </c>
       <c r="O114" s="46" t="n"/>
       <c r="P114" s="53" t="n">
@@ -15847,7 +15847,7 @@
         </is>
       </c>
       <c r="N115" s="53" t="n">
-        <v>46325.51431712963</v>
+        <v>46326.49396990741</v>
       </c>
       <c r="O115" s="46" t="n"/>
       <c r="P115" s="53" t="n">

</xml_diff>